<commit_message>
--CONFECCION EN CURSO DEL FORMULARIO DE CARGA MANUAL
--CREACION DE FUNCION PARA BUSQUEDA DE EMPRESAS COMPLETA DENTRO DEL SERVICIO DE BUSCADOR POR CUIT, DATO QUE FUNCIONA COMO CLAVE UNICA
</commit_message>
<xml_diff>
--- a/Control de Facturas/Assets/Plantillas/BENEFICIARIOS AGUA, GAS Y LUZ.xlsx
+++ b/Control de Facturas/Assets/Plantillas/BENEFICIARIOS AGUA, GAS Y LUZ.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Programa Servicios Basicos\Control de Facturas\Assets\Plantillas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93066361-B353-4A51-A998-F2CE0DC5B42B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA448181-691C-40FB-A646-EBEFC189D38F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-20610" yWindow="-60" windowWidth="20730" windowHeight="11040" xr2:uid="{82731452-31CB-4A50-BC16-E3FD7323D481}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{82731452-31CB-4A50-BC16-E3FD7323D481}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11893" uniqueCount="5947">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11893" uniqueCount="5948">
   <si>
     <t>Número</t>
   </si>
@@ -17870,6 +17870,9 @@
   </si>
   <si>
     <t>AGUAS DE FORMOSA</t>
+  </si>
+  <si>
+    <t>false</t>
   </si>
 </sst>
 </file>
@@ -18309,7 +18312,7 @@
         <v>113</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>4</v>
+        <v>5947</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
--IMPLEMENTACIONES: *MODELO DE DATOSFACTURA -> modelado de datos parciales que componen el modelo de factura, el cual esta destinado a ser el objeto resultante de una carga manual.
*PROCESADOR DE CARGAMANUAL  -> destinado a procesar los modelos de datosfactura, con la finalidad de crear los objetos factura

**FORM DE CARGAMANUAL  --> formulario de carga manual de facturas.

Se implemento la totalidad de la logica para el acoplamiento de estas nuevas funcionalidades con el resto del programa, permitiendo asi generar facturas de forma manual
</commit_message>
<xml_diff>
--- a/Control de Facturas/Assets/Plantillas/BENEFICIARIOS AGUA, GAS Y LUZ.xlsx
+++ b/Control de Facturas/Assets/Plantillas/BENEFICIARIOS AGUA, GAS Y LUZ.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Programa Servicios Basicos\Control de Facturas\Assets\Plantillas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CA9D6C1-4CFC-41AC-9BAF-267FDB27AF48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4C043DF-90CE-4F56-B1D7-21352E5AE5FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{82731452-31CB-4A50-BC16-E3FD7323D481}"/>
   </bookViews>
@@ -16381,9 +16381,6 @@
     <t>AMICONEDEKALInoFFGABRIELA</t>
   </si>
   <si>
-    <t>AGUAS DEL noRTE</t>
-  </si>
-  <si>
     <t>COOPERATIVAELECTRICADEAMEGHInoLTDA</t>
   </si>
   <si>
@@ -17870,6 +17867,9 @@
   </si>
   <si>
     <t>TATIANAsiLVANAALEGRE</t>
+  </si>
+  <si>
+    <t>AGUAS DEL NORTE</t>
   </si>
 </sst>
 </file>
@@ -18343,7 +18343,7 @@
         <v>74</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>5667</v>
+        <v>5666</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -18360,7 +18360,7 @@
         <v>75</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>5667</v>
+        <v>5666</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -18402,7 +18402,7 @@
         <v>1202</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>5668</v>
+        <v>5667</v>
       </c>
       <c r="C8" s="3" t="s">
         <v>4</v>
@@ -18428,7 +18428,7 @@
         <v>76</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>5667</v>
+        <v>5666</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -18453,7 +18453,7 @@
         <v>1325</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>5669</v>
+        <v>5668</v>
       </c>
       <c r="C11" s="3" t="s">
         <v>4</v>
@@ -18496,7 +18496,7 @@
         <v>2971</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>5667</v>
+        <v>5666</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -18606,7 +18606,7 @@
         <v>2603</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>5670</v>
+        <v>5669</v>
       </c>
       <c r="C20" s="3" t="s">
         <v>4</v>
@@ -18657,7 +18657,7 @@
         <v>3814</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>5671</v>
+        <v>5670</v>
       </c>
       <c r="C23" s="3" t="s">
         <v>4</v>
@@ -18683,7 +18683,7 @@
         <v>137</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>5667</v>
+        <v>5666</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -18708,7 +18708,7 @@
         <v>3937</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>5672</v>
+        <v>5671</v>
       </c>
       <c r="C26" s="3" t="s">
         <v>4</v>
@@ -18717,7 +18717,7 @@
         <v>198</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>5667</v>
+        <v>5666</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -18734,7 +18734,7 @@
         <v>2952</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>5667</v>
+        <v>5666</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -18751,7 +18751,7 @@
         <v>138</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>5667</v>
+        <v>5666</v>
       </c>
     </row>
     <row r="29" spans="1:5" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -18819,7 +18819,7 @@
         <v>119</v>
       </c>
       <c r="E32" s="3" t="s">
-        <v>5667</v>
+        <v>5666</v>
       </c>
     </row>
     <row r="33" spans="1:5" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -18878,7 +18878,7 @@
         <v>4876</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>5673</v>
+        <v>5672</v>
       </c>
       <c r="C36" s="3" t="s">
         <v>4</v>
@@ -18904,7 +18904,7 @@
         <v>159</v>
       </c>
       <c r="E37" s="3" t="s">
-        <v>5667</v>
+        <v>5666</v>
       </c>
     </row>
     <row r="38" spans="1:5" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -18989,7 +18989,7 @@
         <v>217</v>
       </c>
       <c r="E42" s="3" t="s">
-        <v>5667</v>
+        <v>5666</v>
       </c>
     </row>
     <row r="43" spans="1:5" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -19006,7 +19006,7 @@
         <v>2966</v>
       </c>
       <c r="E43" s="3" t="s">
-        <v>5667</v>
+        <v>5666</v>
       </c>
     </row>
     <row r="44" spans="1:5" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -19040,7 +19040,7 @@
         <v>176</v>
       </c>
       <c r="E45" s="3" t="s">
-        <v>5667</v>
+        <v>5666</v>
       </c>
     </row>
     <row r="46" spans="1:5" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -19082,7 +19082,7 @@
         <v>5331</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>5674</v>
+        <v>5673</v>
       </c>
       <c r="C48" s="3" t="s">
         <v>4</v>
@@ -19159,7 +19159,7 @@
         <v>177</v>
       </c>
       <c r="E52" s="3" t="s">
-        <v>5667</v>
+        <v>5666</v>
       </c>
     </row>
     <row r="53" spans="1:5" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -19210,7 +19210,7 @@
         <v>202</v>
       </c>
       <c r="E55" s="3" t="s">
-        <v>5667</v>
+        <v>5666</v>
       </c>
     </row>
     <row r="56" spans="1:5" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -19252,7 +19252,7 @@
         <v>6255</v>
       </c>
       <c r="B58" s="3" t="s">
-        <v>5675</v>
+        <v>5674</v>
       </c>
       <c r="C58" s="3" t="s">
         <v>4</v>
@@ -19269,7 +19269,7 @@
         <v>6298</v>
       </c>
       <c r="B59" s="3" t="s">
-        <v>5676</v>
+        <v>5675</v>
       </c>
       <c r="C59" s="3" t="s">
         <v>4</v>
@@ -19286,7 +19286,7 @@
         <v>7007</v>
       </c>
       <c r="B60" s="3" t="s">
-        <v>5677</v>
+        <v>5676</v>
       </c>
       <c r="C60" s="3" t="s">
         <v>4</v>
@@ -19516,7 +19516,7 @@
         <v>11</v>
       </c>
       <c r="E73" s="3" t="s">
-        <v>5667</v>
+        <v>5666</v>
       </c>
     </row>
     <row r="74" spans="1:5" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -19558,7 +19558,7 @@
         <v>7561</v>
       </c>
       <c r="B76" s="3" t="s">
-        <v>5678</v>
+        <v>5677</v>
       </c>
       <c r="C76" s="3" t="s">
         <v>4</v>
@@ -19592,7 +19592,7 @@
         <v>7571</v>
       </c>
       <c r="B78" s="3" t="s">
-        <v>5679</v>
+        <v>5678</v>
       </c>
       <c r="C78" s="3" t="s">
         <v>4</v>
@@ -19609,7 +19609,7 @@
         <v>7572</v>
       </c>
       <c r="B79" s="3" t="s">
-        <v>5680</v>
+        <v>5679</v>
       </c>
       <c r="C79" s="3" t="s">
         <v>4</v>
@@ -19643,7 +19643,7 @@
         <v>7578</v>
       </c>
       <c r="B81" s="3" t="s">
-        <v>5681</v>
+        <v>5680</v>
       </c>
       <c r="C81" s="3" t="s">
         <v>4</v>
@@ -19660,7 +19660,7 @@
         <v>7605</v>
       </c>
       <c r="B82" s="3" t="s">
-        <v>5682</v>
+        <v>5681</v>
       </c>
       <c r="C82" s="3" t="s">
         <v>4</v>
@@ -19881,7 +19881,7 @@
         <v>8469</v>
       </c>
       <c r="B95" s="3" t="s">
-        <v>5683</v>
+        <v>5682</v>
       </c>
       <c r="C95" s="3" t="s">
         <v>4</v>
@@ -19898,7 +19898,7 @@
         <v>8567</v>
       </c>
       <c r="B96" s="3" t="s">
-        <v>5684</v>
+        <v>5683</v>
       </c>
       <c r="C96" s="3" t="s">
         <v>4</v>
@@ -20102,7 +20102,7 @@
         <v>9028</v>
       </c>
       <c r="B108" s="3" t="s">
-        <v>5685</v>
+        <v>5684</v>
       </c>
       <c r="C108" s="3" t="s">
         <v>4</v>
@@ -20153,7 +20153,7 @@
         <v>9733</v>
       </c>
       <c r="B111" s="3" t="s">
-        <v>5686</v>
+        <v>5685</v>
       </c>
       <c r="C111" s="3" t="s">
         <v>4</v>
@@ -20196,7 +20196,7 @@
         <v>151</v>
       </c>
       <c r="E113" s="3" t="s">
-        <v>5667</v>
+        <v>5666</v>
       </c>
     </row>
     <row r="114" spans="1:5" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -20221,7 +20221,7 @@
         <v>9969</v>
       </c>
       <c r="B115" s="3" t="s">
-        <v>5687</v>
+        <v>5686</v>
       </c>
       <c r="C115" s="3" t="s">
         <v>4</v>
@@ -20323,7 +20323,7 @@
         <v>10627</v>
       </c>
       <c r="B121" s="3" t="s">
-        <v>5688</v>
+        <v>5687</v>
       </c>
       <c r="C121" s="3" t="s">
         <v>4</v>
@@ -20340,7 +20340,7 @@
         <v>10646</v>
       </c>
       <c r="B122" s="3" t="s">
-        <v>5689</v>
+        <v>5688</v>
       </c>
       <c r="C122" s="3" t="s">
         <v>4</v>
@@ -20510,7 +20510,7 @@
         <v>10888</v>
       </c>
       <c r="B132" s="3" t="s">
-        <v>5690</v>
+        <v>5689</v>
       </c>
       <c r="C132" s="3" t="s">
         <v>4</v>
@@ -20519,7 +20519,7 @@
         <v>1177</v>
       </c>
       <c r="E132" s="3" t="s">
-        <v>5667</v>
+        <v>5666</v>
       </c>
     </row>
     <row r="133" spans="1:5" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -20578,7 +20578,7 @@
         <v>10943</v>
       </c>
       <c r="B136" s="3" t="s">
-        <v>5691</v>
+        <v>5690</v>
       </c>
       <c r="C136" s="3" t="s">
         <v>4</v>
@@ -20663,7 +20663,7 @@
         <v>11003</v>
       </c>
       <c r="B141" s="3" t="s">
-        <v>5692</v>
+        <v>5691</v>
       </c>
       <c r="C141" s="3" t="s">
         <v>4</v>
@@ -20791,7 +20791,7 @@
         <v>62</v>
       </c>
       <c r="E148" s="3" t="s">
-        <v>5667</v>
+        <v>5666</v>
       </c>
     </row>
     <row r="149" spans="1:5" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -20918,7 +20918,7 @@
         <v>12357</v>
       </c>
       <c r="B156" s="3" t="s">
-        <v>5693</v>
+        <v>5692</v>
       </c>
       <c r="C156" s="3" t="s">
         <v>4</v>
@@ -21003,7 +21003,7 @@
         <v>12580</v>
       </c>
       <c r="B161" s="3" t="s">
-        <v>5694</v>
+        <v>5693</v>
       </c>
       <c r="C161" s="3" t="s">
         <v>4</v>
@@ -21080,7 +21080,7 @@
         <v>2938</v>
       </c>
       <c r="E165" s="3" t="s">
-        <v>5667</v>
+        <v>5666</v>
       </c>
     </row>
     <row r="166" spans="1:5" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -21114,7 +21114,7 @@
         <v>247</v>
       </c>
       <c r="E167" s="3" t="s">
-        <v>5667</v>
+        <v>5666</v>
       </c>
     </row>
     <row r="168" spans="1:5" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -21173,7 +21173,7 @@
         <v>12863</v>
       </c>
       <c r="B171" s="3" t="s">
-        <v>5695</v>
+        <v>5694</v>
       </c>
       <c r="C171" s="3" t="s">
         <v>4</v>
@@ -21190,7 +21190,7 @@
         <v>12864</v>
       </c>
       <c r="B172" s="3" t="s">
-        <v>5696</v>
+        <v>5695</v>
       </c>
       <c r="C172" s="3" t="s">
         <v>4</v>
@@ -21250,7 +21250,7 @@
         <v>2947</v>
       </c>
       <c r="E175" s="3" t="s">
-        <v>5667</v>
+        <v>5666</v>
       </c>
     </row>
     <row r="176" spans="1:5" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -21343,7 +21343,7 @@
         <v>14181</v>
       </c>
       <c r="B181" s="3" t="s">
-        <v>5697</v>
+        <v>5696</v>
       </c>
       <c r="C181" s="3" t="s">
         <v>4</v>
@@ -21386,7 +21386,7 @@
         <v>235</v>
       </c>
       <c r="E183" s="3" t="s">
-        <v>5667</v>
+        <v>5666</v>
       </c>
     </row>
     <row r="184" spans="1:5" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -21420,7 +21420,7 @@
         <v>67</v>
       </c>
       <c r="E185" s="3" t="s">
-        <v>5667</v>
+        <v>5666</v>
       </c>
     </row>
     <row r="186" spans="1:5" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -21547,7 +21547,7 @@
         <v>17805</v>
       </c>
       <c r="B193" s="3" t="s">
-        <v>5698</v>
+        <v>5697</v>
       </c>
       <c r="C193" s="3" t="s">
         <v>4</v>
@@ -21649,7 +21649,7 @@
         <v>20477</v>
       </c>
       <c r="B199" s="3" t="s">
-        <v>5699</v>
+        <v>5698</v>
       </c>
       <c r="C199" s="3" t="s">
         <v>4</v>
@@ -21692,7 +21692,7 @@
         <v>241</v>
       </c>
       <c r="E201" s="3" t="s">
-        <v>5667</v>
+        <v>5666</v>
       </c>
     </row>
     <row r="202" spans="1:5" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -21726,7 +21726,7 @@
         <v>35</v>
       </c>
       <c r="E203" s="3" t="s">
-        <v>5667</v>
+        <v>5666</v>
       </c>
     </row>
     <row r="204" spans="1:5" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -21887,7 +21887,7 @@
         <v>26156</v>
       </c>
       <c r="B213" s="3" t="s">
-        <v>5700</v>
+        <v>5699</v>
       </c>
       <c r="C213" s="3" t="s">
         <v>4</v>
@@ -22049,7 +22049,7 @@
         <v>2922</v>
       </c>
       <c r="E222" s="3" t="s">
-        <v>5667</v>
+        <v>5666</v>
       </c>
     </row>
     <row r="223" spans="1:5" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -22117,7 +22117,7 @@
         <v>272</v>
       </c>
       <c r="E226" s="3" t="s">
-        <v>5667</v>
+        <v>5666</v>
       </c>
     </row>
     <row r="227" spans="1:5" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -22142,7 +22142,7 @@
         <v>33533</v>
       </c>
       <c r="B228" s="3" t="s">
-        <v>5701</v>
+        <v>5700</v>
       </c>
       <c r="C228" s="3" t="s">
         <v>4</v>
@@ -22295,7 +22295,7 @@
         <v>35750</v>
       </c>
       <c r="B237" s="3" t="s">
-        <v>5702</v>
+        <v>5701</v>
       </c>
       <c r="C237" s="3" t="s">
         <v>4</v>
@@ -22423,7 +22423,7 @@
         <v>265</v>
       </c>
       <c r="E244" s="3" t="s">
-        <v>5667</v>
+        <v>5666</v>
       </c>
     </row>
     <row r="245" spans="1:5" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -22839,7 +22839,7 @@
         <v>46145</v>
       </c>
       <c r="B269" s="3" t="s">
-        <v>5703</v>
+        <v>5702</v>
       </c>
       <c r="C269" s="3" t="s">
         <v>4</v>
@@ -22890,7 +22890,7 @@
         <v>48338</v>
       </c>
       <c r="B272" s="3" t="s">
-        <v>5704</v>
+        <v>5703</v>
       </c>
       <c r="C272" s="3" t="s">
         <v>4</v>
@@ -22916,7 +22916,7 @@
         <v>2219</v>
       </c>
       <c r="E273" s="3" t="s">
-        <v>5667</v>
+        <v>5666</v>
       </c>
     </row>
     <row r="274" spans="1:5" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -22941,7 +22941,7 @@
         <v>48805</v>
       </c>
       <c r="B275" s="3" t="s">
-        <v>5705</v>
+        <v>5704</v>
       </c>
       <c r="C275" s="3" t="s">
         <v>4</v>
@@ -23060,7 +23060,7 @@
         <v>49829</v>
       </c>
       <c r="B282" s="3" t="s">
-        <v>5706</v>
+        <v>5705</v>
       </c>
       <c r="C282" s="3" t="s">
         <v>4</v>
@@ -23213,7 +23213,7 @@
         <v>57520</v>
       </c>
       <c r="B291" s="3" t="s">
-        <v>5707</v>
+        <v>5706</v>
       </c>
       <c r="C291" s="3" t="s">
         <v>4</v>
@@ -23332,7 +23332,7 @@
         <v>58737</v>
       </c>
       <c r="B298" s="3" t="s">
-        <v>5708</v>
+        <v>5707</v>
       </c>
       <c r="C298" s="3" t="s">
         <v>4</v>
@@ -23528,7 +23528,7 @@
         <v>125</v>
       </c>
       <c r="E309" s="3" t="s">
-        <v>5667</v>
+        <v>5666</v>
       </c>
     </row>
     <row r="310" spans="1:5" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -23553,7 +23553,7 @@
         <v>68602</v>
       </c>
       <c r="B311" s="3" t="s">
-        <v>5709</v>
+        <v>5708</v>
       </c>
       <c r="C311" s="3" t="s">
         <v>4</v>
@@ -23596,7 +23596,7 @@
         <v>2889</v>
       </c>
       <c r="E313" s="3" t="s">
-        <v>5667</v>
+        <v>5666</v>
       </c>
     </row>
     <row r="314" spans="1:5" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -24012,7 +24012,7 @@
         <v>82472</v>
       </c>
       <c r="B338" s="3" t="s">
-        <v>5710</v>
+        <v>5709</v>
       </c>
       <c r="C338" s="3" t="s">
         <v>4</v>
@@ -24046,7 +24046,7 @@
         <v>82772</v>
       </c>
       <c r="B340" s="3" t="s">
-        <v>5711</v>
+        <v>5710</v>
       </c>
       <c r="C340" s="3" t="s">
         <v>4</v>
@@ -24055,7 +24055,7 @@
         <v>2886</v>
       </c>
       <c r="E340" s="3" t="s">
-        <v>5667</v>
+        <v>5666</v>
       </c>
     </row>
     <row r="341" spans="1:5" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -24208,7 +24208,7 @@
         <v>2888</v>
       </c>
       <c r="E349" s="3" t="s">
-        <v>5667</v>
+        <v>5666</v>
       </c>
     </row>
     <row r="350" spans="1:5" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -24403,7 +24403,7 @@
         <v>92681</v>
       </c>
       <c r="B361" s="3" t="s">
-        <v>5712</v>
+        <v>5711</v>
       </c>
       <c r="C361" s="3" t="s">
         <v>4</v>
@@ -24590,7 +24590,7 @@
         <v>99451</v>
       </c>
       <c r="B372" s="3" t="s">
-        <v>5713</v>
+        <v>5712</v>
       </c>
       <c r="C372" s="3" t="s">
         <v>4</v>
@@ -24607,7 +24607,7 @@
         <v>99598</v>
       </c>
       <c r="B373" s="3" t="s">
-        <v>5714</v>
+        <v>5713</v>
       </c>
       <c r="C373" s="3" t="s">
         <v>4</v>
@@ -24616,7 +24616,7 @@
         <v>2863</v>
       </c>
       <c r="E373" s="3" t="s">
-        <v>5667</v>
+        <v>5666</v>
       </c>
     </row>
     <row r="374" spans="1:5" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -25015,7 +25015,7 @@
         <v>110674</v>
       </c>
       <c r="B397" s="3" t="s">
-        <v>5715</v>
+        <v>5714</v>
       </c>
       <c r="C397" s="3" t="s">
         <v>4</v>
@@ -25032,7 +25032,7 @@
         <v>111078</v>
       </c>
       <c r="B398" s="3" t="s">
-        <v>5716</v>
+        <v>5715</v>
       </c>
       <c r="C398" s="3" t="s">
         <v>4</v>
@@ -25083,7 +25083,7 @@
         <v>111715</v>
       </c>
       <c r="B401" s="3" t="s">
-        <v>5717</v>
+        <v>5716</v>
       </c>
       <c r="C401" s="3" t="s">
         <v>4</v>
@@ -25440,7 +25440,7 @@
         <v>122357</v>
       </c>
       <c r="B422" s="3" t="s">
-        <v>5718</v>
+        <v>5717</v>
       </c>
       <c r="C422" s="3" t="s">
         <v>4</v>
@@ -25644,7 +25644,7 @@
         <v>124361</v>
       </c>
       <c r="B434" s="3" t="s">
-        <v>5719</v>
+        <v>5718</v>
       </c>
       <c r="C434" s="3" t="s">
         <v>4</v>
@@ -25763,7 +25763,7 @@
         <v>125649</v>
       </c>
       <c r="B441" s="3" t="s">
-        <v>5720</v>
+        <v>5719</v>
       </c>
       <c r="C441" s="3" t="s">
         <v>4</v>
@@ -25780,7 +25780,7 @@
         <v>125851</v>
       </c>
       <c r="B442" s="3" t="s">
-        <v>5721</v>
+        <v>5720</v>
       </c>
       <c r="C442" s="3" t="s">
         <v>4</v>
@@ -26018,7 +26018,7 @@
         <v>132364</v>
       </c>
       <c r="B456" s="3" t="s">
-        <v>5722</v>
+        <v>5721</v>
       </c>
       <c r="C456" s="3" t="s">
         <v>4</v>
@@ -26418,7 +26418,7 @@
         <v>2823</v>
       </c>
       <c r="E479" s="3" t="s">
-        <v>5667</v>
+        <v>5666</v>
       </c>
     </row>
     <row r="480" spans="1:5" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -26511,7 +26511,7 @@
         <v>158689</v>
       </c>
       <c r="B485" s="3" t="s">
-        <v>5723</v>
+        <v>5722</v>
       </c>
       <c r="C485" s="3" t="s">
         <v>4</v>
@@ -26732,7 +26732,7 @@
         <v>171813</v>
       </c>
       <c r="B498" s="3" t="s">
-        <v>5724</v>
+        <v>5723</v>
       </c>
       <c r="C498" s="3" t="s">
         <v>4</v>
@@ -26792,7 +26792,7 @@
         <v>2800</v>
       </c>
       <c r="E501" s="3" t="s">
-        <v>5667</v>
+        <v>5666</v>
       </c>
     </row>
     <row r="502" spans="1:5" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -26936,7 +26936,7 @@
         <v>178027</v>
       </c>
       <c r="B510" s="3" t="s">
-        <v>5725</v>
+        <v>5724</v>
       </c>
       <c r="C510" s="3" t="s">
         <v>4</v>
@@ -27106,7 +27106,7 @@
         <v>189468</v>
       </c>
       <c r="B520" s="3" t="s">
-        <v>5726</v>
+        <v>5725</v>
       </c>
       <c r="C520" s="3" t="s">
         <v>4</v>
@@ -27684,7 +27684,7 @@
         <v>190558</v>
       </c>
       <c r="B554" s="3" t="s">
-        <v>5727</v>
+        <v>5726</v>
       </c>
       <c r="C554" s="3" t="s">
         <v>4</v>
@@ -27752,7 +27752,7 @@
         <v>191311</v>
       </c>
       <c r="B558" s="3" t="s">
-        <v>5728</v>
+        <v>5727</v>
       </c>
       <c r="C558" s="3" t="s">
         <v>4</v>
@@ -27803,7 +27803,7 @@
         <v>191951</v>
       </c>
       <c r="B561" s="3" t="s">
-        <v>5729</v>
+        <v>5728</v>
       </c>
       <c r="C561" s="3" t="s">
         <v>4</v>
@@ -27820,7 +27820,7 @@
         <v>192881</v>
       </c>
       <c r="B562" s="3" t="s">
-        <v>5730</v>
+        <v>5729</v>
       </c>
       <c r="C562" s="3" t="s">
         <v>4</v>
@@ -27837,7 +27837,7 @@
         <v>193054</v>
       </c>
       <c r="B563" s="3" t="s">
-        <v>5731</v>
+        <v>5730</v>
       </c>
       <c r="C563" s="3" t="s">
         <v>4</v>
@@ -27990,7 +27990,7 @@
         <v>197127</v>
       </c>
       <c r="B572" s="3" t="s">
-        <v>5732</v>
+        <v>5731</v>
       </c>
       <c r="C572" s="3" t="s">
         <v>4</v>
@@ -28143,7 +28143,7 @@
         <v>202738</v>
       </c>
       <c r="B581" s="3" t="s">
-        <v>5733</v>
+        <v>5732</v>
       </c>
       <c r="C581" s="3" t="s">
         <v>4</v>
@@ -28228,7 +28228,7 @@
         <v>204941</v>
       </c>
       <c r="B586" s="3" t="s">
-        <v>5734</v>
+        <v>5733</v>
       </c>
       <c r="C586" s="3" t="s">
         <v>4</v>
@@ -28381,7 +28381,7 @@
         <v>219118</v>
       </c>
       <c r="B595" s="3" t="s">
-        <v>5735</v>
+        <v>5734</v>
       </c>
       <c r="C595" s="3" t="s">
         <v>4</v>
@@ -28602,7 +28602,7 @@
         <v>226297</v>
       </c>
       <c r="B608" s="3" t="s">
-        <v>5736</v>
+        <v>5735</v>
       </c>
       <c r="C608" s="3" t="s">
         <v>4</v>
@@ -28619,7 +28619,7 @@
         <v>226401</v>
       </c>
       <c r="B609" s="3" t="s">
-        <v>5737</v>
+        <v>5736</v>
       </c>
       <c r="C609" s="3" t="s">
         <v>4</v>
@@ -28721,7 +28721,7 @@
         <v>230376</v>
       </c>
       <c r="B615" s="3" t="s">
-        <v>5738</v>
+        <v>5737</v>
       </c>
       <c r="C615" s="3" t="s">
         <v>4</v>
@@ -28755,7 +28755,7 @@
         <v>232246</v>
       </c>
       <c r="B617" s="3" t="s">
-        <v>5739</v>
+        <v>5738</v>
       </c>
       <c r="C617" s="3" t="s">
         <v>4</v>
@@ -28874,7 +28874,7 @@
         <v>235510</v>
       </c>
       <c r="B624" s="3" t="s">
-        <v>5740</v>
+        <v>5739</v>
       </c>
       <c r="C624" s="3" t="s">
         <v>4</v>
@@ -28891,7 +28891,7 @@
         <v>235512</v>
       </c>
       <c r="B625" s="3" t="s">
-        <v>5741</v>
+        <v>5740</v>
       </c>
       <c r="C625" s="3" t="s">
         <v>4</v>
@@ -28908,7 +28908,7 @@
         <v>235513</v>
       </c>
       <c r="B626" s="3" t="s">
-        <v>5742</v>
+        <v>5741</v>
       </c>
       <c r="C626" s="3" t="s">
         <v>4</v>
@@ -28959,7 +28959,7 @@
         <v>235622</v>
       </c>
       <c r="B629" s="3" t="s">
-        <v>5743</v>
+        <v>5742</v>
       </c>
       <c r="C629" s="3" t="s">
         <v>4</v>
@@ -28993,7 +28993,7 @@
         <v>236048</v>
       </c>
       <c r="B631" s="3" t="s">
-        <v>5744</v>
+        <v>5743</v>
       </c>
       <c r="C631" s="3" t="s">
         <v>4</v>
@@ -29010,7 +29010,7 @@
         <v>236636</v>
       </c>
       <c r="B632" s="3" t="s">
-        <v>5745</v>
+        <v>5744</v>
       </c>
       <c r="C632" s="3" t="s">
         <v>4</v>
@@ -29231,7 +29231,7 @@
         <v>240657</v>
       </c>
       <c r="B645" s="3" t="s">
-        <v>5746</v>
+        <v>5745</v>
       </c>
       <c r="C645" s="3" t="s">
         <v>4</v>
@@ -29299,7 +29299,7 @@
         <v>241576</v>
       </c>
       <c r="B649" s="3" t="s">
-        <v>5747</v>
+        <v>5746</v>
       </c>
       <c r="C649" s="3" t="s">
         <v>4</v>
@@ -29316,7 +29316,7 @@
         <v>241577</v>
       </c>
       <c r="B650" s="3" t="s">
-        <v>5748</v>
+        <v>5747</v>
       </c>
       <c r="C650" s="3" t="s">
         <v>4</v>
@@ -29435,7 +29435,7 @@
         <v>243126</v>
       </c>
       <c r="B657" s="3" t="s">
-        <v>5749</v>
+        <v>5748</v>
       </c>
       <c r="C657" s="3" t="s">
         <v>4</v>
@@ -29571,7 +29571,7 @@
         <v>245792</v>
       </c>
       <c r="B665" s="3" t="s">
-        <v>5750</v>
+        <v>5749</v>
       </c>
       <c r="C665" s="3" t="s">
         <v>4</v>
@@ -29605,7 +29605,7 @@
         <v>246010</v>
       </c>
       <c r="B667" s="3" t="s">
-        <v>5751</v>
+        <v>5750</v>
       </c>
       <c r="C667" s="3" t="s">
         <v>4</v>
@@ -29682,7 +29682,7 @@
         <v>2979</v>
       </c>
       <c r="E671" s="3" t="s">
-        <v>5667</v>
+        <v>5666</v>
       </c>
     </row>
     <row r="672" spans="1:5" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -29724,7 +29724,7 @@
         <v>250552</v>
       </c>
       <c r="B674" s="3" t="s">
-        <v>5752</v>
+        <v>5751</v>
       </c>
       <c r="C674" s="3" t="s">
         <v>4</v>
@@ -29733,7 +29733,7 @@
         <v>2754</v>
       </c>
       <c r="E674" s="3" t="s">
-        <v>5667</v>
+        <v>5666</v>
       </c>
     </row>
     <row r="675" spans="1:5" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -29860,7 +29860,7 @@
         <v>255046</v>
       </c>
       <c r="B682" s="3" t="s">
-        <v>5753</v>
+        <v>5752</v>
       </c>
       <c r="C682" s="3" t="s">
         <v>4</v>
@@ -29928,7 +29928,7 @@
         <v>256609</v>
       </c>
       <c r="B686" s="3" t="s">
-        <v>5754</v>
+        <v>5753</v>
       </c>
       <c r="C686" s="3" t="s">
         <v>4</v>
@@ -30030,7 +30030,7 @@
         <v>260696</v>
       </c>
       <c r="B692" s="3" t="s">
-        <v>5755</v>
+        <v>5754</v>
       </c>
       <c r="C692" s="3" t="s">
         <v>4</v>
@@ -30115,7 +30115,7 @@
         <v>262595</v>
       </c>
       <c r="B697" s="3" t="s">
-        <v>5756</v>
+        <v>5755</v>
       </c>
       <c r="C697" s="3" t="s">
         <v>4</v>
@@ -30124,7 +30124,7 @@
         <v>2391</v>
       </c>
       <c r="E697" s="3" t="s">
-        <v>5667</v>
+        <v>5666</v>
       </c>
     </row>
     <row r="698" spans="1:5" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -30166,7 +30166,7 @@
         <v>262648</v>
       </c>
       <c r="B700" s="3" t="s">
-        <v>5757</v>
+        <v>5756</v>
       </c>
       <c r="C700" s="3" t="s">
         <v>4</v>
@@ -30285,7 +30285,7 @@
         <v>269554</v>
       </c>
       <c r="B707" s="3" t="s">
-        <v>5758</v>
+        <v>5757</v>
       </c>
       <c r="C707" s="3" t="s">
         <v>4</v>
@@ -30472,7 +30472,7 @@
         <v>276933</v>
       </c>
       <c r="B718" s="3" t="s">
-        <v>5759</v>
+        <v>5758</v>
       </c>
       <c r="C718" s="3" t="s">
         <v>4</v>
@@ -30540,7 +30540,7 @@
         <v>278058</v>
       </c>
       <c r="B722" s="3" t="s">
-        <v>5760</v>
+        <v>5759</v>
       </c>
       <c r="C722" s="3" t="s">
         <v>4</v>
@@ -30608,7 +30608,7 @@
         <v>281556</v>
       </c>
       <c r="B726" s="3" t="s">
-        <v>5761</v>
+        <v>5760</v>
       </c>
       <c r="C726" s="3" t="s">
         <v>4</v>
@@ -30693,7 +30693,7 @@
         <v>285507</v>
       </c>
       <c r="B731" s="3" t="s">
-        <v>5762</v>
+        <v>5761</v>
       </c>
       <c r="C731" s="3" t="s">
         <v>4</v>
@@ -30778,7 +30778,7 @@
         <v>287851</v>
       </c>
       <c r="B736" s="3" t="s">
-        <v>5763</v>
+        <v>5762</v>
       </c>
       <c r="C736" s="3" t="s">
         <v>4</v>
@@ -30914,7 +30914,7 @@
         <v>291978</v>
       </c>
       <c r="B744" s="3" t="s">
-        <v>5764</v>
+        <v>5763</v>
       </c>
       <c r="C744" s="3" t="s">
         <v>4</v>
@@ -30948,7 +30948,7 @@
         <v>295086</v>
       </c>
       <c r="B746" s="3" t="s">
-        <v>5765</v>
+        <v>5764</v>
       </c>
       <c r="C746" s="3" t="s">
         <v>4</v>
@@ -30965,7 +30965,7 @@
         <v>297792</v>
       </c>
       <c r="B747" s="3" t="s">
-        <v>5766</v>
+        <v>5765</v>
       </c>
       <c r="C747" s="3" t="s">
         <v>4</v>
@@ -30982,7 +30982,7 @@
         <v>298556</v>
       </c>
       <c r="B748" s="3" t="s">
-        <v>5767</v>
+        <v>5766</v>
       </c>
       <c r="C748" s="3" t="s">
         <v>4</v>
@@ -31050,7 +31050,7 @@
         <v>300800</v>
       </c>
       <c r="B752" s="3" t="s">
-        <v>5768</v>
+        <v>5767</v>
       </c>
       <c r="C752" s="3" t="s">
         <v>4</v>
@@ -31067,7 +31067,7 @@
         <v>301705</v>
       </c>
       <c r="B753" s="3" t="s">
-        <v>5769</v>
+        <v>5768</v>
       </c>
       <c r="C753" s="3" t="s">
         <v>4</v>
@@ -31101,7 +31101,7 @@
         <v>307867</v>
       </c>
       <c r="B755" s="3" t="s">
-        <v>5770</v>
+        <v>5769</v>
       </c>
       <c r="C755" s="3" t="s">
         <v>4</v>
@@ -31263,7 +31263,7 @@
         <v>454</v>
       </c>
       <c r="E764" s="3" t="s">
-        <v>5667</v>
+        <v>5666</v>
       </c>
     </row>
     <row r="765" spans="1:5" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -31356,7 +31356,7 @@
         <v>324503</v>
       </c>
       <c r="B770" s="3" t="s">
-        <v>5771</v>
+        <v>5770</v>
       </c>
       <c r="C770" s="3" t="s">
         <v>4</v>
@@ -31373,7 +31373,7 @@
         <v>324977</v>
       </c>
       <c r="B771" s="3" t="s">
-        <v>5772</v>
+        <v>5771</v>
       </c>
       <c r="C771" s="3" t="s">
         <v>4</v>
@@ -31458,7 +31458,7 @@
         <v>327658</v>
       </c>
       <c r="B776" s="3" t="s">
-        <v>5773</v>
+        <v>5772</v>
       </c>
       <c r="C776" s="3" t="s">
         <v>4</v>
@@ -31467,7 +31467,7 @@
         <v>451</v>
       </c>
       <c r="E776" s="3" t="s">
-        <v>5667</v>
+        <v>5666</v>
       </c>
     </row>
     <row r="777" spans="1:5" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -31475,7 +31475,7 @@
         <v>328124</v>
       </c>
       <c r="B777" s="3" t="s">
-        <v>5774</v>
+        <v>5773</v>
       </c>
       <c r="C777" s="3" t="s">
         <v>4</v>
@@ -31815,7 +31815,7 @@
         <v>343290</v>
       </c>
       <c r="B797" s="3" t="s">
-        <v>5775</v>
+        <v>5774</v>
       </c>
       <c r="C797" s="3" t="s">
         <v>4</v>
@@ -31866,7 +31866,7 @@
         <v>344829</v>
       </c>
       <c r="B800" s="5" t="s">
-        <v>5450</v>
+        <v>5946</v>
       </c>
       <c r="C800" s="3" t="s">
         <v>4</v>
@@ -31900,7 +31900,7 @@
         <v>345453</v>
       </c>
       <c r="B802" s="3" t="s">
-        <v>5776</v>
+        <v>5775</v>
       </c>
       <c r="C802" s="3" t="s">
         <v>4</v>
@@ -31917,7 +31917,7 @@
         <v>346087</v>
       </c>
       <c r="B803" s="3" t="s">
-        <v>5451</v>
+        <v>5450</v>
       </c>
       <c r="C803" s="3" t="s">
         <v>4</v>
@@ -31934,7 +31934,7 @@
         <v>346199</v>
       </c>
       <c r="B804" s="3" t="s">
-        <v>5452</v>
+        <v>5451</v>
       </c>
       <c r="C804" s="3" t="s">
         <v>4</v>
@@ -31985,7 +31985,7 @@
         <v>347739</v>
       </c>
       <c r="B807" s="3" t="s">
-        <v>5777</v>
+        <v>5776</v>
       </c>
       <c r="C807" s="3" t="s">
         <v>4</v>
@@ -32019,7 +32019,7 @@
         <v>349673</v>
       </c>
       <c r="B809" s="3" t="s">
-        <v>5453</v>
+        <v>5452</v>
       </c>
       <c r="C809" s="3" t="s">
         <v>4</v>
@@ -32053,7 +32053,7 @@
         <v>350234</v>
       </c>
       <c r="B811" s="3" t="s">
-        <v>5778</v>
+        <v>5777</v>
       </c>
       <c r="C811" s="3" t="s">
         <v>4</v>
@@ -32121,7 +32121,7 @@
         <v>352365</v>
       </c>
       <c r="B815" s="3" t="s">
-        <v>5454</v>
+        <v>5453</v>
       </c>
       <c r="C815" s="3" t="s">
         <v>4</v>
@@ -32155,7 +32155,7 @@
         <v>354314</v>
       </c>
       <c r="B817" s="3" t="s">
-        <v>5455</v>
+        <v>5454</v>
       </c>
       <c r="C817" s="3" t="s">
         <v>4</v>
@@ -32223,7 +32223,7 @@
         <v>355329</v>
       </c>
       <c r="B821" s="3" t="s">
-        <v>5456</v>
+        <v>5455</v>
       </c>
       <c r="C821" s="3" t="s">
         <v>4</v>
@@ -32240,7 +32240,7 @@
         <v>357514</v>
       </c>
       <c r="B822" s="3" t="s">
-        <v>5457</v>
+        <v>5456</v>
       </c>
       <c r="C822" s="3" t="s">
         <v>4</v>
@@ -32325,7 +32325,7 @@
         <v>360931</v>
       </c>
       <c r="B827" s="3" t="s">
-        <v>5458</v>
+        <v>5457</v>
       </c>
       <c r="C827" s="3" t="s">
         <v>4</v>
@@ -32410,7 +32410,7 @@
         <v>365326</v>
       </c>
       <c r="B832" s="3" t="s">
-        <v>5459</v>
+        <v>5458</v>
       </c>
       <c r="C832" s="3" t="s">
         <v>4</v>
@@ -32427,7 +32427,7 @@
         <v>365501</v>
       </c>
       <c r="B833" s="3" t="s">
-        <v>5779</v>
+        <v>5778</v>
       </c>
       <c r="C833" s="3" t="s">
         <v>4</v>
@@ -32453,7 +32453,7 @@
         <v>473</v>
       </c>
       <c r="E834" s="3" t="s">
-        <v>5667</v>
+        <v>5666</v>
       </c>
     </row>
     <row r="835" spans="1:5" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -32512,7 +32512,7 @@
         <v>368363</v>
       </c>
       <c r="B838" s="3" t="s">
-        <v>5460</v>
+        <v>5459</v>
       </c>
       <c r="C838" s="3" t="s">
         <v>4</v>
@@ -32546,7 +32546,7 @@
         <v>368986</v>
       </c>
       <c r="B840" s="3" t="s">
-        <v>5461</v>
+        <v>5460</v>
       </c>
       <c r="C840" s="3" t="s">
         <v>4</v>
@@ -32597,7 +32597,7 @@
         <v>370379</v>
       </c>
       <c r="B843" s="3" t="s">
-        <v>5462</v>
+        <v>5461</v>
       </c>
       <c r="C843" s="3" t="s">
         <v>4</v>
@@ -32614,7 +32614,7 @@
         <v>370761</v>
       </c>
       <c r="B844" s="3" t="s">
-        <v>5463</v>
+        <v>5462</v>
       </c>
       <c r="C844" s="3" t="s">
         <v>4</v>
@@ -32699,7 +32699,7 @@
         <v>372272</v>
       </c>
       <c r="B849" s="3" t="s">
-        <v>5780</v>
+        <v>5779</v>
       </c>
       <c r="C849" s="3" t="s">
         <v>4</v>
@@ -32716,7 +32716,7 @@
         <v>372443</v>
       </c>
       <c r="B850" s="3" t="s">
-        <v>5781</v>
+        <v>5780</v>
       </c>
       <c r="C850" s="3" t="s">
         <v>4</v>
@@ -32733,7 +32733,7 @@
         <v>372530</v>
       </c>
       <c r="B851" s="3" t="s">
-        <v>5464</v>
+        <v>5463</v>
       </c>
       <c r="C851" s="3" t="s">
         <v>4</v>
@@ -32818,7 +32818,7 @@
         <v>373863</v>
       </c>
       <c r="B856" s="3" t="s">
-        <v>5782</v>
+        <v>5781</v>
       </c>
       <c r="C856" s="3" t="s">
         <v>4</v>
@@ -32937,7 +32937,7 @@
         <v>376974</v>
       </c>
       <c r="B863" s="3" t="s">
-        <v>5465</v>
+        <v>5464</v>
       </c>
       <c r="C863" s="3" t="s">
         <v>4</v>
@@ -33056,7 +33056,7 @@
         <v>383882</v>
       </c>
       <c r="B870" s="3" t="s">
-        <v>5466</v>
+        <v>5465</v>
       </c>
       <c r="C870" s="3" t="s">
         <v>4</v>
@@ -33073,7 +33073,7 @@
         <v>384192</v>
       </c>
       <c r="B871" s="3" t="s">
-        <v>5783</v>
+        <v>5782</v>
       </c>
       <c r="C871" s="3" t="s">
         <v>4</v>
@@ -33099,7 +33099,7 @@
         <v>2652</v>
       </c>
       <c r="E872" s="3" t="s">
-        <v>5667</v>
+        <v>5666</v>
       </c>
     </row>
     <row r="873" spans="1:5" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -33277,7 +33277,7 @@
         <v>388346</v>
       </c>
       <c r="B883" s="3" t="s">
-        <v>5467</v>
+        <v>5466</v>
       </c>
       <c r="C883" s="3" t="s">
         <v>4</v>
@@ -33311,7 +33311,7 @@
         <v>389701</v>
       </c>
       <c r="B885" s="3" t="s">
-        <v>5784</v>
+        <v>5783</v>
       </c>
       <c r="C885" s="3" t="s">
         <v>4</v>
@@ -33345,7 +33345,7 @@
         <v>392098</v>
       </c>
       <c r="B887" s="3" t="s">
-        <v>5785</v>
+        <v>5784</v>
       </c>
       <c r="C887" s="3" t="s">
         <v>4</v>
@@ -33430,7 +33430,7 @@
         <v>394655</v>
       </c>
       <c r="B892" s="3" t="s">
-        <v>5786</v>
+        <v>5785</v>
       </c>
       <c r="C892" s="3" t="s">
         <v>4</v>
@@ -33447,7 +33447,7 @@
         <v>394709</v>
       </c>
       <c r="B893" s="3" t="s">
-        <v>5787</v>
+        <v>5786</v>
       </c>
       <c r="C893" s="3" t="s">
         <v>4</v>
@@ -33464,7 +33464,7 @@
         <v>394861</v>
       </c>
       <c r="B894" s="3" t="s">
-        <v>5788</v>
+        <v>5787</v>
       </c>
       <c r="C894" s="3" t="s">
         <v>4</v>
@@ -33498,7 +33498,7 @@
         <v>395525</v>
       </c>
       <c r="B896" s="3" t="s">
-        <v>5789</v>
+        <v>5788</v>
       </c>
       <c r="C896" s="3" t="s">
         <v>4</v>
@@ -33515,7 +33515,7 @@
         <v>395560</v>
       </c>
       <c r="B897" s="3" t="s">
-        <v>5468</v>
+        <v>5467</v>
       </c>
       <c r="C897" s="3" t="s">
         <v>4</v>
@@ -33566,7 +33566,7 @@
         <v>397509</v>
       </c>
       <c r="B900" s="3" t="s">
-        <v>5790</v>
+        <v>5789</v>
       </c>
       <c r="C900" s="3" t="s">
         <v>4</v>
@@ -33685,7 +33685,7 @@
         <v>401447</v>
       </c>
       <c r="B907" s="3" t="s">
-        <v>5469</v>
+        <v>5468</v>
       </c>
       <c r="C907" s="3" t="s">
         <v>4</v>
@@ -33804,7 +33804,7 @@
         <v>406298</v>
       </c>
       <c r="B914" s="3" t="s">
-        <v>5470</v>
+        <v>5469</v>
       </c>
       <c r="C914" s="3" t="s">
         <v>4</v>
@@ -33872,7 +33872,7 @@
         <v>409909</v>
       </c>
       <c r="B918" s="3" t="s">
-        <v>5791</v>
+        <v>5790</v>
       </c>
       <c r="C918" s="3" t="s">
         <v>4</v>
@@ -33974,7 +33974,7 @@
         <v>412340</v>
       </c>
       <c r="B924" s="3" t="s">
-        <v>5471</v>
+        <v>5470</v>
       </c>
       <c r="C924" s="3" t="s">
         <v>4</v>
@@ -34110,7 +34110,7 @@
         <v>413789</v>
       </c>
       <c r="B932" s="3" t="s">
-        <v>5792</v>
+        <v>5791</v>
       </c>
       <c r="C932" s="3" t="s">
         <v>4</v>
@@ -34127,7 +34127,7 @@
         <v>414649</v>
       </c>
       <c r="B933" s="3" t="s">
-        <v>5472</v>
+        <v>5471</v>
       </c>
       <c r="C933" s="3" t="s">
         <v>4</v>
@@ -34144,7 +34144,7 @@
         <v>415197</v>
       </c>
       <c r="B934" s="3" t="s">
-        <v>5793</v>
+        <v>5792</v>
       </c>
       <c r="C934" s="3" t="s">
         <v>4</v>
@@ -34433,7 +34433,7 @@
         <v>423286</v>
       </c>
       <c r="B951" s="3" t="s">
-        <v>5473</v>
+        <v>5472</v>
       </c>
       <c r="C951" s="3" t="s">
         <v>4</v>
@@ -34586,7 +34586,7 @@
         <v>429725</v>
       </c>
       <c r="B960" s="3" t="s">
-        <v>5794</v>
+        <v>5793</v>
       </c>
       <c r="C960" s="3" t="s">
         <v>4</v>
@@ -34671,7 +34671,7 @@
         <v>431885</v>
       </c>
       <c r="B965" s="3" t="s">
-        <v>5795</v>
+        <v>5794</v>
       </c>
       <c r="C965" s="3" t="s">
         <v>4</v>
@@ -34705,7 +34705,7 @@
         <v>432712</v>
       </c>
       <c r="B967" s="3" t="s">
-        <v>5796</v>
+        <v>5795</v>
       </c>
       <c r="C967" s="3" t="s">
         <v>4</v>
@@ -34824,7 +34824,7 @@
         <v>436912</v>
       </c>
       <c r="B974" s="3" t="s">
-        <v>5797</v>
+        <v>5796</v>
       </c>
       <c r="C974" s="3" t="s">
         <v>4</v>
@@ -34977,7 +34977,7 @@
         <v>441476</v>
       </c>
       <c r="B983" s="3" t="s">
-        <v>5474</v>
+        <v>5473</v>
       </c>
       <c r="C983" s="3" t="s">
         <v>4</v>
@@ -34994,7 +34994,7 @@
         <v>441593</v>
       </c>
       <c r="B984" s="3" t="s">
-        <v>5798</v>
+        <v>5797</v>
       </c>
       <c r="C984" s="3" t="s">
         <v>4</v>
@@ -35011,7 +35011,7 @@
         <v>441873</v>
       </c>
       <c r="B985" s="3" t="s">
-        <v>5799</v>
+        <v>5798</v>
       </c>
       <c r="C985" s="3" t="s">
         <v>4</v>
@@ -35062,7 +35062,7 @@
         <v>443033</v>
       </c>
       <c r="B988" s="3" t="s">
-        <v>5475</v>
+        <v>5474</v>
       </c>
       <c r="C988" s="3" t="s">
         <v>4</v>
@@ -35079,7 +35079,7 @@
         <v>443358</v>
       </c>
       <c r="B989" s="3" t="s">
-        <v>5476</v>
+        <v>5475</v>
       </c>
       <c r="C989" s="3" t="s">
         <v>4</v>
@@ -35164,7 +35164,7 @@
         <v>445141</v>
       </c>
       <c r="B994" s="3" t="s">
-        <v>5800</v>
+        <v>5799</v>
       </c>
       <c r="C994" s="3" t="s">
         <v>4</v>
@@ -35181,7 +35181,7 @@
         <v>448194</v>
       </c>
       <c r="B995" s="3" t="s">
-        <v>5801</v>
+        <v>5800</v>
       </c>
       <c r="C995" s="3" t="s">
         <v>4</v>
@@ -35198,7 +35198,7 @@
         <v>448240</v>
       </c>
       <c r="B996" s="3" t="s">
-        <v>5802</v>
+        <v>5801</v>
       </c>
       <c r="C996" s="3" t="s">
         <v>4</v>
@@ -35249,7 +35249,7 @@
         <v>450437</v>
       </c>
       <c r="B999" s="3" t="s">
-        <v>5477</v>
+        <v>5476</v>
       </c>
       <c r="C999" s="3" t="s">
         <v>4</v>
@@ -35317,7 +35317,7 @@
         <v>452102</v>
       </c>
       <c r="B1003" s="3" t="s">
-        <v>5803</v>
+        <v>5802</v>
       </c>
       <c r="C1003" s="3" t="s">
         <v>4</v>
@@ -35334,7 +35334,7 @@
         <v>452862</v>
       </c>
       <c r="B1004" s="3" t="s">
-        <v>5478</v>
+        <v>5477</v>
       </c>
       <c r="C1004" s="3" t="s">
         <v>4</v>
@@ -35368,7 +35368,7 @@
         <v>454896</v>
       </c>
       <c r="B1006" s="3" t="s">
-        <v>5804</v>
+        <v>5803</v>
       </c>
       <c r="C1006" s="3" t="s">
         <v>4</v>
@@ -35487,7 +35487,7 @@
         <v>458226</v>
       </c>
       <c r="B1013" s="3" t="s">
-        <v>5479</v>
+        <v>5478</v>
       </c>
       <c r="C1013" s="3" t="s">
         <v>4</v>
@@ -35589,7 +35589,7 @@
         <v>462720</v>
       </c>
       <c r="B1019" s="3" t="s">
-        <v>5805</v>
+        <v>5804</v>
       </c>
       <c r="C1019" s="3" t="s">
         <v>4</v>
@@ -35742,7 +35742,7 @@
         <v>465657</v>
       </c>
       <c r="B1028" s="3" t="s">
-        <v>5480</v>
+        <v>5479</v>
       </c>
       <c r="C1028" s="3" t="s">
         <v>4</v>
@@ -35827,7 +35827,7 @@
         <v>467162</v>
       </c>
       <c r="B1033" s="3" t="s">
-        <v>5806</v>
+        <v>5805</v>
       </c>
       <c r="C1033" s="3" t="s">
         <v>4</v>
@@ -35895,7 +35895,7 @@
         <v>468937</v>
       </c>
       <c r="B1037" s="3" t="s">
-        <v>5807</v>
+        <v>5806</v>
       </c>
       <c r="C1037" s="3" t="s">
         <v>4</v>
@@ -35946,7 +35946,7 @@
         <v>470779</v>
       </c>
       <c r="B1040" s="3" t="s">
-        <v>5808</v>
+        <v>5807</v>
       </c>
       <c r="C1040" s="3" t="s">
         <v>4</v>
@@ -36031,7 +36031,7 @@
         <v>473152</v>
       </c>
       <c r="B1045" s="3" t="s">
-        <v>5481</v>
+        <v>5480</v>
       </c>
       <c r="C1045" s="3" t="s">
         <v>4</v>
@@ -36082,7 +36082,7 @@
         <v>474589</v>
       </c>
       <c r="B1048" s="3" t="s">
-        <v>5809</v>
+        <v>5808</v>
       </c>
       <c r="C1048" s="3" t="s">
         <v>4</v>
@@ -36099,7 +36099,7 @@
         <v>475153</v>
       </c>
       <c r="B1049" s="3" t="s">
-        <v>5810</v>
+        <v>5809</v>
       </c>
       <c r="C1049" s="3" t="s">
         <v>4</v>
@@ -36116,7 +36116,7 @@
         <v>475328</v>
       </c>
       <c r="B1050" s="3" t="s">
-        <v>5811</v>
+        <v>5810</v>
       </c>
       <c r="C1050" s="3" t="s">
         <v>4</v>
@@ -36150,7 +36150,7 @@
         <v>476145</v>
       </c>
       <c r="B1052" s="3" t="s">
-        <v>5482</v>
+        <v>5481</v>
       </c>
       <c r="C1052" s="3" t="s">
         <v>4</v>
@@ -36167,7 +36167,7 @@
         <v>476653</v>
       </c>
       <c r="B1053" s="3" t="s">
-        <v>5812</v>
+        <v>5811</v>
       </c>
       <c r="C1053" s="3" t="s">
         <v>4</v>
@@ -36184,7 +36184,7 @@
         <v>476769</v>
       </c>
       <c r="B1054" s="3" t="s">
-        <v>5483</v>
+        <v>5482</v>
       </c>
       <c r="C1054" s="3" t="s">
         <v>4</v>
@@ -36422,7 +36422,7 @@
         <v>482080</v>
       </c>
       <c r="B1068" s="3" t="s">
-        <v>5813</v>
+        <v>5812</v>
       </c>
       <c r="C1068" s="3" t="s">
         <v>4</v>
@@ -36643,7 +36643,7 @@
         <v>487092</v>
       </c>
       <c r="B1081" s="3" t="s">
-        <v>5484</v>
+        <v>5483</v>
       </c>
       <c r="C1081" s="3" t="s">
         <v>4</v>
@@ -36660,7 +36660,7 @@
         <v>487468</v>
       </c>
       <c r="B1082" s="3" t="s">
-        <v>5814</v>
+        <v>5813</v>
       </c>
       <c r="C1082" s="3" t="s">
         <v>4</v>
@@ -36711,7 +36711,7 @@
         <v>488040</v>
       </c>
       <c r="B1085" s="3" t="s">
-        <v>5485</v>
+        <v>5484</v>
       </c>
       <c r="C1085" s="3" t="s">
         <v>4</v>
@@ -36771,7 +36771,7 @@
         <v>2609</v>
       </c>
       <c r="E1088" s="3" t="s">
-        <v>5667</v>
+        <v>5666</v>
       </c>
     </row>
     <row r="1089" spans="1:5" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -36830,7 +36830,7 @@
         <v>493348</v>
       </c>
       <c r="B1092" s="3" t="s">
-        <v>5486</v>
+        <v>5485</v>
       </c>
       <c r="C1092" s="3" t="s">
         <v>4</v>
@@ -36966,7 +36966,7 @@
         <v>499105</v>
       </c>
       <c r="B1100" s="3" t="s">
-        <v>5487</v>
+        <v>5486</v>
       </c>
       <c r="C1100" s="3" t="s">
         <v>4</v>
@@ -37017,7 +37017,7 @@
         <v>500344</v>
       </c>
       <c r="B1103" s="3" t="s">
-        <v>5488</v>
+        <v>5487</v>
       </c>
       <c r="C1103" s="3" t="s">
         <v>4</v>
@@ -37085,7 +37085,7 @@
         <v>502358</v>
       </c>
       <c r="B1107" s="3" t="s">
-        <v>5489</v>
+        <v>5488</v>
       </c>
       <c r="C1107" s="3" t="s">
         <v>4</v>
@@ -37102,7 +37102,7 @@
         <v>502711</v>
       </c>
       <c r="B1108" s="3" t="s">
-        <v>5490</v>
+        <v>5489</v>
       </c>
       <c r="C1108" s="3" t="s">
         <v>4</v>
@@ -37187,7 +37187,7 @@
         <v>504519</v>
       </c>
       <c r="B1113" s="3" t="s">
-        <v>5815</v>
+        <v>5814</v>
       </c>
       <c r="C1113" s="3" t="s">
         <v>4</v>
@@ -37272,7 +37272,7 @@
         <v>505676</v>
       </c>
       <c r="B1118" s="3" t="s">
-        <v>5491</v>
+        <v>5490</v>
       </c>
       <c r="C1118" s="3" t="s">
         <v>4</v>
@@ -37340,7 +37340,7 @@
         <v>506343</v>
       </c>
       <c r="B1122" s="3" t="s">
-        <v>5492</v>
+        <v>5491</v>
       </c>
       <c r="C1122" s="3" t="s">
         <v>4</v>
@@ -37527,7 +37527,7 @@
         <v>509335</v>
       </c>
       <c r="B1133" s="3" t="s">
-        <v>5493</v>
+        <v>5492</v>
       </c>
       <c r="C1133" s="3" t="s">
         <v>4</v>
@@ -37646,7 +37646,7 @@
         <v>510555</v>
       </c>
       <c r="B1140" s="3" t="s">
-        <v>5494</v>
+        <v>5493</v>
       </c>
       <c r="C1140" s="3" t="s">
         <v>4</v>
@@ -37816,7 +37816,7 @@
         <v>515344</v>
       </c>
       <c r="B1150" s="3" t="s">
-        <v>5495</v>
+        <v>5494</v>
       </c>
       <c r="C1150" s="3" t="s">
         <v>4</v>
@@ -38088,7 +38088,7 @@
         <v>523966</v>
       </c>
       <c r="B1166" s="3" t="s">
-        <v>5816</v>
+        <v>5815</v>
       </c>
       <c r="C1166" s="3" t="s">
         <v>4</v>
@@ -38122,7 +38122,7 @@
         <v>525880</v>
       </c>
       <c r="B1168" s="3" t="s">
-        <v>5496</v>
+        <v>5495</v>
       </c>
       <c r="C1168" s="3" t="s">
         <v>4</v>
@@ -38173,7 +38173,7 @@
         <v>527287</v>
       </c>
       <c r="B1171" s="3" t="s">
-        <v>5817</v>
+        <v>5816</v>
       </c>
       <c r="C1171" s="3" t="s">
         <v>4</v>
@@ -38258,7 +38258,7 @@
         <v>529130</v>
       </c>
       <c r="B1176" s="3" t="s">
-        <v>5497</v>
+        <v>5496</v>
       </c>
       <c r="C1176" s="3" t="s">
         <v>4</v>
@@ -38292,7 +38292,7 @@
         <v>529899</v>
       </c>
       <c r="B1178" s="3" t="s">
-        <v>5818</v>
+        <v>5817</v>
       </c>
       <c r="C1178" s="3" t="s">
         <v>4</v>
@@ -38360,7 +38360,7 @@
         <v>530515</v>
       </c>
       <c r="B1182" s="3" t="s">
-        <v>5498</v>
+        <v>5497</v>
       </c>
       <c r="C1182" s="3" t="s">
         <v>4</v>
@@ -38377,7 +38377,7 @@
         <v>530968</v>
       </c>
       <c r="B1183" s="3" t="s">
-        <v>5819</v>
+        <v>5818</v>
       </c>
       <c r="C1183" s="3" t="s">
         <v>4</v>
@@ -38411,7 +38411,7 @@
         <v>532762</v>
       </c>
       <c r="B1185" s="3" t="s">
-        <v>5499</v>
+        <v>5498</v>
       </c>
       <c r="C1185" s="3" t="s">
         <v>4</v>
@@ -38615,7 +38615,7 @@
         <v>537706</v>
       </c>
       <c r="B1197" s="3" t="s">
-        <v>5820</v>
+        <v>5819</v>
       </c>
       <c r="C1197" s="3" t="s">
         <v>4</v>
@@ -38751,7 +38751,7 @@
         <v>539572</v>
       </c>
       <c r="B1205" s="3" t="s">
-        <v>5821</v>
+        <v>5820</v>
       </c>
       <c r="C1205" s="3" t="s">
         <v>4</v>
@@ -38836,7 +38836,7 @@
         <v>541309</v>
       </c>
       <c r="B1210" s="3" t="s">
-        <v>5500</v>
+        <v>5499</v>
       </c>
       <c r="C1210" s="3" t="s">
         <v>4</v>
@@ -38853,7 +38853,7 @@
         <v>541312</v>
       </c>
       <c r="B1211" s="3" t="s">
-        <v>5822</v>
+        <v>5821</v>
       </c>
       <c r="C1211" s="3" t="s">
         <v>4</v>
@@ -38887,7 +38887,7 @@
         <v>542670</v>
       </c>
       <c r="B1213" s="3" t="s">
-        <v>5501</v>
+        <v>5500</v>
       </c>
       <c r="C1213" s="3" t="s">
         <v>4</v>
@@ -39040,7 +39040,7 @@
         <v>544884</v>
       </c>
       <c r="B1222" s="3" t="s">
-        <v>5502</v>
+        <v>5501</v>
       </c>
       <c r="C1222" s="3" t="s">
         <v>4</v>
@@ -39074,7 +39074,7 @@
         <v>545039</v>
       </c>
       <c r="B1224" s="3" t="s">
-        <v>5503</v>
+        <v>5502</v>
       </c>
       <c r="C1224" s="3" t="s">
         <v>4</v>
@@ -39176,7 +39176,7 @@
         <v>546853</v>
       </c>
       <c r="B1230" s="3" t="s">
-        <v>5504</v>
+        <v>5503</v>
       </c>
       <c r="C1230" s="3" t="s">
         <v>4</v>
@@ -39346,7 +39346,7 @@
         <v>550167</v>
       </c>
       <c r="B1240" s="3" t="s">
-        <v>5505</v>
+        <v>5504</v>
       </c>
       <c r="C1240" s="3" t="s">
         <v>4</v>
@@ -39414,7 +39414,7 @@
         <v>552534</v>
       </c>
       <c r="B1244" s="3" t="s">
-        <v>5823</v>
+        <v>5822</v>
       </c>
       <c r="C1244" s="3" t="s">
         <v>4</v>
@@ -39465,7 +39465,7 @@
         <v>553935</v>
       </c>
       <c r="B1247" s="3" t="s">
-        <v>5506</v>
+        <v>5505</v>
       </c>
       <c r="C1247" s="3" t="s">
         <v>4</v>
@@ -39482,7 +39482,7 @@
         <v>554185</v>
       </c>
       <c r="B1248" s="3" t="s">
-        <v>5824</v>
+        <v>5823</v>
       </c>
       <c r="C1248" s="3" t="s">
         <v>4</v>
@@ -39533,7 +39533,7 @@
         <v>554929</v>
       </c>
       <c r="B1251" s="3" t="s">
-        <v>5825</v>
+        <v>5824</v>
       </c>
       <c r="C1251" s="3" t="s">
         <v>4</v>
@@ -39601,7 +39601,7 @@
         <v>555954</v>
       </c>
       <c r="B1255" s="3" t="s">
-        <v>5826</v>
+        <v>5825</v>
       </c>
       <c r="C1255" s="3" t="s">
         <v>4</v>
@@ -39618,7 +39618,7 @@
         <v>555959</v>
       </c>
       <c r="B1256" s="3" t="s">
-        <v>5827</v>
+        <v>5826</v>
       </c>
       <c r="C1256" s="3" t="s">
         <v>4</v>
@@ -39669,7 +39669,7 @@
         <v>558033</v>
       </c>
       <c r="B1259" s="3" t="s">
-        <v>5507</v>
+        <v>5506</v>
       </c>
       <c r="C1259" s="3" t="s">
         <v>4</v>
@@ -39720,7 +39720,7 @@
         <v>559580</v>
       </c>
       <c r="B1262" s="3" t="s">
-        <v>5828</v>
+        <v>5827</v>
       </c>
       <c r="C1262" s="3" t="s">
         <v>4</v>
@@ -39754,7 +39754,7 @@
         <v>559956</v>
       </c>
       <c r="B1264" s="3" t="s">
-        <v>5829</v>
+        <v>5828</v>
       </c>
       <c r="C1264" s="3" t="s">
         <v>4</v>
@@ -40179,7 +40179,7 @@
         <v>567118</v>
       </c>
       <c r="B1289" s="3" t="s">
-        <v>5830</v>
+        <v>5829</v>
       </c>
       <c r="C1289" s="3" t="s">
         <v>4</v>
@@ -40196,7 +40196,7 @@
         <v>567465</v>
       </c>
       <c r="B1290" s="3" t="s">
-        <v>5831</v>
+        <v>5830</v>
       </c>
       <c r="C1290" s="3" t="s">
         <v>4</v>
@@ -40230,7 +40230,7 @@
         <v>567772</v>
       </c>
       <c r="B1292" s="3" t="s">
-        <v>5832</v>
+        <v>5831</v>
       </c>
       <c r="C1292" s="3" t="s">
         <v>4</v>
@@ -40349,7 +40349,7 @@
         <v>570624</v>
       </c>
       <c r="B1299" s="3" t="s">
-        <v>5833</v>
+        <v>5832</v>
       </c>
       <c r="C1299" s="3" t="s">
         <v>4</v>
@@ -40434,7 +40434,7 @@
         <v>573335</v>
       </c>
       <c r="B1304" s="3" t="s">
-        <v>5508</v>
+        <v>5507</v>
       </c>
       <c r="C1304" s="3" t="s">
         <v>4</v>
@@ -40502,7 +40502,7 @@
         <v>577935</v>
       </c>
       <c r="B1308" s="3" t="s">
-        <v>5509</v>
+        <v>5508</v>
       </c>
       <c r="C1308" s="3" t="s">
         <v>4</v>
@@ -40519,7 +40519,7 @@
         <v>578095</v>
       </c>
       <c r="B1309" s="3" t="s">
-        <v>5510</v>
+        <v>5509</v>
       </c>
       <c r="C1309" s="3" t="s">
         <v>4</v>
@@ -40655,7 +40655,7 @@
         <v>581820</v>
       </c>
       <c r="B1317" s="3" t="s">
-        <v>5834</v>
+        <v>5833</v>
       </c>
       <c r="C1317" s="3" t="s">
         <v>4</v>
@@ -40876,7 +40876,7 @@
         <v>585234</v>
       </c>
       <c r="B1330" s="3" t="s">
-        <v>5835</v>
+        <v>5834</v>
       </c>
       <c r="C1330" s="3" t="s">
         <v>4</v>
@@ -40944,7 +40944,7 @@
         <v>585471</v>
       </c>
       <c r="B1334" s="3" t="s">
-        <v>5511</v>
+        <v>5510</v>
       </c>
       <c r="C1334" s="3" t="s">
         <v>4</v>
@@ -41148,7 +41148,7 @@
         <v>589917</v>
       </c>
       <c r="B1346" s="3" t="s">
-        <v>5512</v>
+        <v>5511</v>
       </c>
       <c r="C1346" s="3" t="s">
         <v>4</v>
@@ -41250,7 +41250,7 @@
         <v>593741</v>
       </c>
       <c r="B1352" s="3" t="s">
-        <v>5513</v>
+        <v>5512</v>
       </c>
       <c r="C1352" s="3" t="s">
         <v>4</v>
@@ -41301,7 +41301,7 @@
         <v>594675</v>
       </c>
       <c r="B1355" s="3" t="s">
-        <v>5836</v>
+        <v>5835</v>
       </c>
       <c r="C1355" s="3" t="s">
         <v>4</v>
@@ -41335,7 +41335,7 @@
         <v>595444</v>
       </c>
       <c r="B1357" s="3" t="s">
-        <v>5514</v>
+        <v>5513</v>
       </c>
       <c r="C1357" s="3" t="s">
         <v>4</v>
@@ -41624,7 +41624,7 @@
         <v>601844</v>
       </c>
       <c r="B1374" s="3" t="s">
-        <v>5837</v>
+        <v>5836</v>
       </c>
       <c r="C1374" s="3" t="s">
         <v>4</v>
@@ -41845,7 +41845,7 @@
         <v>606982</v>
       </c>
       <c r="B1387" s="3" t="s">
-        <v>5838</v>
+        <v>5837</v>
       </c>
       <c r="C1387" s="3" t="s">
         <v>4</v>
@@ -42100,7 +42100,7 @@
         <v>611217</v>
       </c>
       <c r="B1402" s="3" t="s">
-        <v>5515</v>
+        <v>5514</v>
       </c>
       <c r="C1402" s="3" t="s">
         <v>4</v>
@@ -42287,7 +42287,7 @@
         <v>613079</v>
       </c>
       <c r="B1413" s="3" t="s">
-        <v>5839</v>
+        <v>5838</v>
       </c>
       <c r="C1413" s="3" t="s">
         <v>4</v>
@@ -42321,7 +42321,7 @@
         <v>614449</v>
       </c>
       <c r="B1415" s="3" t="s">
-        <v>5840</v>
+        <v>5839</v>
       </c>
       <c r="C1415" s="3" t="s">
         <v>4</v>
@@ -42372,7 +42372,7 @@
         <v>615195</v>
       </c>
       <c r="B1418" s="3" t="s">
-        <v>5516</v>
+        <v>5515</v>
       </c>
       <c r="C1418" s="3" t="s">
         <v>4</v>
@@ -42559,7 +42559,7 @@
         <v>618730</v>
       </c>
       <c r="B1429" s="3" t="s">
-        <v>5517</v>
+        <v>5516</v>
       </c>
       <c r="C1429" s="3" t="s">
         <v>4</v>
@@ -42593,7 +42593,7 @@
         <v>619630</v>
       </c>
       <c r="B1431" s="3" t="s">
-        <v>5518</v>
+        <v>5517</v>
       </c>
       <c r="C1431" s="3" t="s">
         <v>4</v>
@@ -42704,7 +42704,7 @@
         <v>775</v>
       </c>
       <c r="E1437" s="3" t="s">
-        <v>5667</v>
+        <v>5666</v>
       </c>
     </row>
     <row r="1438" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
@@ -42746,7 +42746,7 @@
         <v>622404</v>
       </c>
       <c r="B1440" s="3" t="s">
-        <v>5519</v>
+        <v>5518</v>
       </c>
       <c r="C1440" s="3" t="s">
         <v>4</v>
@@ -42814,7 +42814,7 @@
         <v>624098</v>
       </c>
       <c r="B1444" s="3" t="s">
-        <v>5520</v>
+        <v>5519</v>
       </c>
       <c r="C1444" s="3" t="s">
         <v>4</v>
@@ -42865,7 +42865,7 @@
         <v>625027</v>
       </c>
       <c r="B1447" s="3" t="s">
-        <v>5521</v>
+        <v>5520</v>
       </c>
       <c r="C1447" s="3" t="s">
         <v>4</v>
@@ -43103,7 +43103,7 @@
         <v>631291</v>
       </c>
       <c r="B1461" s="3" t="s">
-        <v>5522</v>
+        <v>5521</v>
       </c>
       <c r="C1461" s="3" t="s">
         <v>4</v>
@@ -43256,7 +43256,7 @@
         <v>637472</v>
       </c>
       <c r="B1470" s="3" t="s">
-        <v>5523</v>
+        <v>5522</v>
       </c>
       <c r="C1470" s="3" t="s">
         <v>4</v>
@@ -43562,7 +43562,7 @@
         <v>641165</v>
       </c>
       <c r="B1488" s="3" t="s">
-        <v>5524</v>
+        <v>5523</v>
       </c>
       <c r="C1488" s="3" t="s">
         <v>4</v>
@@ -43596,7 +43596,7 @@
         <v>641451</v>
       </c>
       <c r="B1490" s="3" t="s">
-        <v>5525</v>
+        <v>5524</v>
       </c>
       <c r="C1490" s="3" t="s">
         <v>4</v>
@@ -43613,7 +43613,7 @@
         <v>641600</v>
       </c>
       <c r="B1491" s="3" t="s">
-        <v>5526</v>
+        <v>5525</v>
       </c>
       <c r="C1491" s="3" t="s">
         <v>4</v>
@@ -43715,7 +43715,7 @@
         <v>643238</v>
       </c>
       <c r="B1497" s="3" t="s">
-        <v>5527</v>
+        <v>5526</v>
       </c>
       <c r="C1497" s="3" t="s">
         <v>4</v>
@@ -43749,7 +43749,7 @@
         <v>644774</v>
       </c>
       <c r="B1499" s="3" t="s">
-        <v>5841</v>
+        <v>5840</v>
       </c>
       <c r="C1499" s="3" t="s">
         <v>4</v>
@@ -43766,7 +43766,7 @@
         <v>645456</v>
       </c>
       <c r="B1500" s="3" t="s">
-        <v>5842</v>
+        <v>5841</v>
       </c>
       <c r="C1500" s="3" t="s">
         <v>4</v>
@@ -43783,7 +43783,7 @@
         <v>646120</v>
       </c>
       <c r="B1501" s="3" t="s">
-        <v>5843</v>
+        <v>5842</v>
       </c>
       <c r="C1501" s="3" t="s">
         <v>4</v>
@@ -43885,7 +43885,7 @@
         <v>646636</v>
       </c>
       <c r="B1507" s="3" t="s">
-        <v>5844</v>
+        <v>5843</v>
       </c>
       <c r="C1507" s="3" t="s">
         <v>4</v>
@@ -43902,7 +43902,7 @@
         <v>646742</v>
       </c>
       <c r="B1508" s="3" t="s">
-        <v>5845</v>
+        <v>5844</v>
       </c>
       <c r="C1508" s="3" t="s">
         <v>4</v>
@@ -43936,7 +43936,7 @@
         <v>647191</v>
       </c>
       <c r="B1510" s="3" t="s">
-        <v>5846</v>
+        <v>5845</v>
       </c>
       <c r="C1510" s="3" t="s">
         <v>4</v>
@@ -44072,7 +44072,7 @@
         <v>650292</v>
       </c>
       <c r="B1518" s="3" t="s">
-        <v>5847</v>
+        <v>5846</v>
       </c>
       <c r="C1518" s="3" t="s">
         <v>4</v>
@@ -44123,7 +44123,7 @@
         <v>651066</v>
       </c>
       <c r="B1521" s="3" t="s">
-        <v>5848</v>
+        <v>5847</v>
       </c>
       <c r="C1521" s="3" t="s">
         <v>4</v>
@@ -44140,7 +44140,7 @@
         <v>651411</v>
       </c>
       <c r="B1522" s="3" t="s">
-        <v>5528</v>
+        <v>5527</v>
       </c>
       <c r="C1522" s="3" t="s">
         <v>4</v>
@@ -44225,7 +44225,7 @@
         <v>653059</v>
       </c>
       <c r="B1527" s="3" t="s">
-        <v>5529</v>
+        <v>5528</v>
       </c>
       <c r="C1527" s="3" t="s">
         <v>4</v>
@@ -44310,7 +44310,7 @@
         <v>655324</v>
       </c>
       <c r="B1532" s="3" t="s">
-        <v>5849</v>
+        <v>5848</v>
       </c>
       <c r="C1532" s="3" t="s">
         <v>4</v>
@@ -44327,7 +44327,7 @@
         <v>655654</v>
       </c>
       <c r="B1533" s="3" t="s">
-        <v>5850</v>
+        <v>5849</v>
       </c>
       <c r="C1533" s="3" t="s">
         <v>4</v>
@@ -44599,7 +44599,7 @@
         <v>660479</v>
       </c>
       <c r="B1549" s="3" t="s">
-        <v>5530</v>
+        <v>5529</v>
       </c>
       <c r="C1549" s="3" t="s">
         <v>4</v>
@@ -44616,7 +44616,7 @@
         <v>660480</v>
       </c>
       <c r="B1550" s="3" t="s">
-        <v>5531</v>
+        <v>5530</v>
       </c>
       <c r="C1550" s="3" t="s">
         <v>4</v>
@@ -44735,7 +44735,7 @@
         <v>662129</v>
       </c>
       <c r="B1557" s="3" t="s">
-        <v>5851</v>
+        <v>5850</v>
       </c>
       <c r="C1557" s="3" t="s">
         <v>4</v>
@@ -44786,7 +44786,7 @@
         <v>662387</v>
       </c>
       <c r="B1560" s="3" t="s">
-        <v>5532</v>
+        <v>5531</v>
       </c>
       <c r="C1560" s="3" t="s">
         <v>4</v>
@@ -44888,7 +44888,7 @@
         <v>663699</v>
       </c>
       <c r="B1566" s="3" t="s">
-        <v>5533</v>
+        <v>5532</v>
       </c>
       <c r="C1566" s="3" t="s">
         <v>4</v>
@@ -45279,7 +45279,7 @@
         <v>673034</v>
       </c>
       <c r="B1589" s="3" t="s">
-        <v>5852</v>
+        <v>5851</v>
       </c>
       <c r="C1589" s="3" t="s">
         <v>4</v>
@@ -45500,7 +45500,7 @@
         <v>677217</v>
       </c>
       <c r="B1602" s="3" t="s">
-        <v>5534</v>
+        <v>5533</v>
       </c>
       <c r="C1602" s="3" t="s">
         <v>4</v>
@@ -45687,7 +45687,7 @@
         <v>680269</v>
       </c>
       <c r="B1613" s="3" t="s">
-        <v>5535</v>
+        <v>5534</v>
       </c>
       <c r="C1613" s="3" t="s">
         <v>4</v>
@@ -45789,7 +45789,7 @@
         <v>681885</v>
       </c>
       <c r="B1619" s="3" t="s">
-        <v>5536</v>
+        <v>5535</v>
       </c>
       <c r="C1619" s="3" t="s">
         <v>4</v>
@@ -45874,7 +45874,7 @@
         <v>681890</v>
       </c>
       <c r="B1624" s="3" t="s">
-        <v>5537</v>
+        <v>5536</v>
       </c>
       <c r="C1624" s="3" t="s">
         <v>4</v>
@@ -45959,7 +45959,7 @@
         <v>682745</v>
       </c>
       <c r="B1629" s="3" t="s">
-        <v>5538</v>
+        <v>5537</v>
       </c>
       <c r="C1629" s="3" t="s">
         <v>4</v>
@@ -46078,7 +46078,7 @@
         <v>684053</v>
       </c>
       <c r="B1636" s="3" t="s">
-        <v>5853</v>
+        <v>5852</v>
       </c>
       <c r="C1636" s="3" t="s">
         <v>4</v>
@@ -46146,7 +46146,7 @@
         <v>684684</v>
       </c>
       <c r="B1640" s="3" t="s">
-        <v>5539</v>
+        <v>5538</v>
       </c>
       <c r="C1640" s="3" t="s">
         <v>4</v>
@@ -46180,7 +46180,7 @@
         <v>684967</v>
       </c>
       <c r="B1642" s="3" t="s">
-        <v>5854</v>
+        <v>5853</v>
       </c>
       <c r="C1642" s="3" t="s">
         <v>4</v>
@@ -46231,7 +46231,7 @@
         <v>685601</v>
       </c>
       <c r="B1645" s="3" t="s">
-        <v>5855</v>
+        <v>5854</v>
       </c>
       <c r="C1645" s="3" t="s">
         <v>4</v>
@@ -46265,7 +46265,7 @@
         <v>685739</v>
       </c>
       <c r="B1647" s="3" t="s">
-        <v>5540</v>
+        <v>5539</v>
       </c>
       <c r="C1647" s="3" t="s">
         <v>4</v>
@@ -46367,7 +46367,7 @@
         <v>686259</v>
       </c>
       <c r="B1653" s="3" t="s">
-        <v>5541</v>
+        <v>5540</v>
       </c>
       <c r="C1653" s="3" t="s">
         <v>4</v>
@@ -46401,7 +46401,7 @@
         <v>686336</v>
       </c>
       <c r="B1655" s="3" t="s">
-        <v>5542</v>
+        <v>5541</v>
       </c>
       <c r="C1655" s="3" t="s">
         <v>4</v>
@@ -46656,7 +46656,7 @@
         <v>688340</v>
       </c>
       <c r="B1670" s="3" t="s">
-        <v>5543</v>
+        <v>5542</v>
       </c>
       <c r="C1670" s="3" t="s">
         <v>4</v>
@@ -46707,7 +46707,7 @@
         <v>688809</v>
       </c>
       <c r="B1673" s="3" t="s">
-        <v>5544</v>
+        <v>5543</v>
       </c>
       <c r="C1673" s="3" t="s">
         <v>4</v>
@@ -46792,7 +46792,7 @@
         <v>689981</v>
       </c>
       <c r="B1678" s="3" t="s">
-        <v>5856</v>
+        <v>5855</v>
       </c>
       <c r="C1678" s="3" t="s">
         <v>4</v>
@@ -46928,7 +46928,7 @@
         <v>691484</v>
       </c>
       <c r="B1686" s="3" t="s">
-        <v>5545</v>
+        <v>5544</v>
       </c>
       <c r="C1686" s="3" t="s">
         <v>4</v>
@@ -46979,7 +46979,7 @@
         <v>694175</v>
       </c>
       <c r="B1689" s="3" t="s">
-        <v>5546</v>
+        <v>5545</v>
       </c>
       <c r="C1689" s="3" t="s">
         <v>4</v>
@@ -46996,7 +46996,7 @@
         <v>694547</v>
       </c>
       <c r="B1690" s="3" t="s">
-        <v>5547</v>
+        <v>5546</v>
       </c>
       <c r="C1690" s="3" t="s">
         <v>4</v>
@@ -47064,7 +47064,7 @@
         <v>695102</v>
       </c>
       <c r="B1694" s="3" t="s">
-        <v>5548</v>
+        <v>5547</v>
       </c>
       <c r="C1694" s="3" t="s">
         <v>4</v>
@@ -47081,7 +47081,7 @@
         <v>695239</v>
       </c>
       <c r="B1695" s="3" t="s">
-        <v>5857</v>
+        <v>5856</v>
       </c>
       <c r="C1695" s="3" t="s">
         <v>4</v>
@@ -47251,7 +47251,7 @@
         <v>699637</v>
       </c>
       <c r="B1705" s="3" t="s">
-        <v>5549</v>
+        <v>5548</v>
       </c>
       <c r="C1705" s="3" t="s">
         <v>4</v>
@@ -47285,7 +47285,7 @@
         <v>700137</v>
       </c>
       <c r="B1707" s="3" t="s">
-        <v>5550</v>
+        <v>5549</v>
       </c>
       <c r="C1707" s="3" t="s">
         <v>4</v>
@@ -47319,7 +47319,7 @@
         <v>700761</v>
       </c>
       <c r="B1709" s="3" t="s">
-        <v>5858</v>
+        <v>5857</v>
       </c>
       <c r="C1709" s="3" t="s">
         <v>4</v>
@@ -47438,7 +47438,7 @@
         <v>701527</v>
       </c>
       <c r="B1716" s="3" t="s">
-        <v>5551</v>
+        <v>5550</v>
       </c>
       <c r="C1716" s="3" t="s">
         <v>4</v>
@@ -47625,7 +47625,7 @@
         <v>808758</v>
       </c>
       <c r="B1727" s="3" t="s">
-        <v>5552</v>
+        <v>5551</v>
       </c>
       <c r="C1727" s="3" t="s">
         <v>4</v>
@@ -47846,7 +47846,7 @@
         <v>826937</v>
       </c>
       <c r="B1740" s="3" t="s">
-        <v>5859</v>
+        <v>5858</v>
       </c>
       <c r="C1740" s="3" t="s">
         <v>4</v>
@@ -48050,7 +48050,7 @@
         <v>836749</v>
       </c>
       <c r="B1752" s="3" t="s">
-        <v>5553</v>
+        <v>5552</v>
       </c>
       <c r="C1752" s="3" t="s">
         <v>4</v>
@@ -48220,7 +48220,7 @@
         <v>838965</v>
       </c>
       <c r="B1762" s="3" t="s">
-        <v>5860</v>
+        <v>5859</v>
       </c>
       <c r="C1762" s="3" t="s">
         <v>4</v>
@@ -48254,7 +48254,7 @@
         <v>841373</v>
       </c>
       <c r="B1764" s="3" t="s">
-        <v>5861</v>
+        <v>5860</v>
       </c>
       <c r="C1764" s="3" t="s">
         <v>4</v>
@@ -48322,7 +48322,7 @@
         <v>841528</v>
       </c>
       <c r="B1768" s="3" t="s">
-        <v>5862</v>
+        <v>5861</v>
       </c>
       <c r="C1768" s="3" t="s">
         <v>4</v>
@@ -48390,7 +48390,7 @@
         <v>841533</v>
       </c>
       <c r="B1772" s="3" t="s">
-        <v>5554</v>
+        <v>5553</v>
       </c>
       <c r="C1772" s="3" t="s">
         <v>4</v>
@@ -48526,7 +48526,7 @@
         <v>845513</v>
       </c>
       <c r="B1780" s="3" t="s">
-        <v>5863</v>
+        <v>5862</v>
       </c>
       <c r="C1780" s="3" t="s">
         <v>4</v>
@@ -48611,7 +48611,7 @@
         <v>848985</v>
       </c>
       <c r="B1785" s="3" t="s">
-        <v>5555</v>
+        <v>5554</v>
       </c>
       <c r="C1785" s="3" t="s">
         <v>4</v>
@@ -48696,7 +48696,7 @@
         <v>851990</v>
       </c>
       <c r="B1790" s="3" t="s">
-        <v>5864</v>
+        <v>5863</v>
       </c>
       <c r="C1790" s="3" t="s">
         <v>4</v>
@@ -48798,7 +48798,7 @@
         <v>857892</v>
       </c>
       <c r="B1796" s="3" t="s">
-        <v>5865</v>
+        <v>5864</v>
       </c>
       <c r="C1796" s="3" t="s">
         <v>4</v>
@@ -48866,7 +48866,7 @@
         <v>860533</v>
       </c>
       <c r="B1800" s="3" t="s">
-        <v>5866</v>
+        <v>5865</v>
       </c>
       <c r="C1800" s="3" t="s">
         <v>4</v>
@@ -49053,7 +49053,7 @@
         <v>868789</v>
       </c>
       <c r="B1811" s="3" t="s">
-        <v>5556</v>
+        <v>5555</v>
       </c>
       <c r="C1811" s="3" t="s">
         <v>4</v>
@@ -49121,7 +49121,7 @@
         <v>873623</v>
       </c>
       <c r="B1815" s="3" t="s">
-        <v>5557</v>
+        <v>5556</v>
       </c>
       <c r="C1815" s="3" t="s">
         <v>4</v>
@@ -49206,7 +49206,7 @@
         <v>878176</v>
       </c>
       <c r="B1820" s="3" t="s">
-        <v>5867</v>
+        <v>5866</v>
       </c>
       <c r="C1820" s="3" t="s">
         <v>4</v>
@@ -49240,7 +49240,7 @@
         <v>879568</v>
       </c>
       <c r="B1822" s="3" t="s">
-        <v>5558</v>
+        <v>5557</v>
       </c>
       <c r="C1822" s="3" t="s">
         <v>4</v>
@@ -49308,7 +49308,7 @@
         <v>888265</v>
       </c>
       <c r="B1826" s="3" t="s">
-        <v>5559</v>
+        <v>5558</v>
       </c>
       <c r="C1826" s="3" t="s">
         <v>4</v>
@@ -49801,7 +49801,7 @@
         <v>909009</v>
       </c>
       <c r="B1855" s="3" t="s">
-        <v>5560</v>
+        <v>5559</v>
       </c>
       <c r="C1855" s="3" t="s">
         <v>4</v>
@@ -49971,7 +49971,7 @@
         <v>924120</v>
       </c>
       <c r="B1865" s="3" t="s">
-        <v>5561</v>
+        <v>5560</v>
       </c>
       <c r="C1865" s="3" t="s">
         <v>4</v>
@@ -50039,7 +50039,7 @@
         <v>932362</v>
       </c>
       <c r="B1869" s="3" t="s">
-        <v>5562</v>
+        <v>5561</v>
       </c>
       <c r="C1869" s="3" t="s">
         <v>4</v>
@@ -50107,7 +50107,7 @@
         <v>937325</v>
       </c>
       <c r="B1873" s="3" t="s">
-        <v>5563</v>
+        <v>5562</v>
       </c>
       <c r="C1873" s="3" t="s">
         <v>4</v>
@@ -50158,7 +50158,7 @@
         <v>939901</v>
       </c>
       <c r="B1876" s="3" t="s">
-        <v>5868</v>
+        <v>5867</v>
       </c>
       <c r="C1876" s="3" t="s">
         <v>4</v>
@@ -50260,7 +50260,7 @@
         <v>947155</v>
       </c>
       <c r="B1882" s="3" t="s">
-        <v>5564</v>
+        <v>5563</v>
       </c>
       <c r="C1882" s="3" t="s">
         <v>4</v>
@@ -50498,7 +50498,7 @@
         <v>956445</v>
       </c>
       <c r="B1896" s="3" t="s">
-        <v>5869</v>
+        <v>5868</v>
       </c>
       <c r="C1896" s="3" t="s">
         <v>4</v>
@@ -50600,7 +50600,7 @@
         <v>960578</v>
       </c>
       <c r="B1902" s="3" t="s">
-        <v>5870</v>
+        <v>5869</v>
       </c>
       <c r="C1902" s="3" t="s">
         <v>4</v>
@@ -50651,7 +50651,7 @@
         <v>962282</v>
       </c>
       <c r="B1905" s="3" t="s">
-        <v>5871</v>
+        <v>5870</v>
       </c>
       <c r="C1905" s="3" t="s">
         <v>4</v>
@@ -50719,7 +50719,7 @@
         <v>963991</v>
       </c>
       <c r="B1909" s="3" t="s">
-        <v>5872</v>
+        <v>5871</v>
       </c>
       <c r="C1909" s="3" t="s">
         <v>4</v>
@@ -50838,7 +50838,7 @@
         <v>976272</v>
       </c>
       <c r="B1916" s="3" t="s">
-        <v>5565</v>
+        <v>5564</v>
       </c>
       <c r="C1916" s="3" t="s">
         <v>4</v>
@@ -50855,7 +50855,7 @@
         <v>976274</v>
       </c>
       <c r="B1917" s="3" t="s">
-        <v>5873</v>
+        <v>5872</v>
       </c>
       <c r="C1917" s="3" t="s">
         <v>4</v>
@@ -50991,7 +50991,7 @@
         <v>980825</v>
       </c>
       <c r="B1925" s="3" t="s">
-        <v>5498</v>
+        <v>5497</v>
       </c>
       <c r="C1925" s="3" t="s">
         <v>4</v>
@@ -51059,7 +51059,7 @@
         <v>985161</v>
       </c>
       <c r="B1929" s="3" t="s">
-        <v>5566</v>
+        <v>5565</v>
       </c>
       <c r="C1929" s="3" t="s">
         <v>4</v>
@@ -51093,7 +51093,7 @@
         <v>986735</v>
       </c>
       <c r="B1931" s="3" t="s">
-        <v>5874</v>
+        <v>5873</v>
       </c>
       <c r="C1931" s="3" t="s">
         <v>4</v>
@@ -51110,7 +51110,7 @@
         <v>987620</v>
       </c>
       <c r="B1932" s="3" t="s">
-        <v>5567</v>
+        <v>5566</v>
       </c>
       <c r="C1932" s="3" t="s">
         <v>4</v>
@@ -51280,7 +51280,7 @@
         <v>994764</v>
       </c>
       <c r="B1942" s="3" t="s">
-        <v>5568</v>
+        <v>5567</v>
       </c>
       <c r="C1942" s="3" t="s">
         <v>4</v>
@@ -51297,7 +51297,7 @@
         <v>994840</v>
       </c>
       <c r="B1943" s="3" t="s">
-        <v>5569</v>
+        <v>5568</v>
       </c>
       <c r="C1943" s="3" t="s">
         <v>4</v>
@@ -51314,7 +51314,7 @@
         <v>994932</v>
       </c>
       <c r="B1944" s="3" t="s">
-        <v>5875</v>
+        <v>5874</v>
       </c>
       <c r="C1944" s="3" t="s">
         <v>4</v>
@@ -51586,7 +51586,7 @@
         <v>1009758</v>
       </c>
       <c r="B1960" s="3" t="s">
-        <v>5570</v>
+        <v>5569</v>
       </c>
       <c r="C1960" s="3" t="s">
         <v>4</v>
@@ -51688,7 +51688,7 @@
         <v>1011533</v>
       </c>
       <c r="B1966" s="3" t="s">
-        <v>5876</v>
+        <v>5875</v>
       </c>
       <c r="C1966" s="3" t="s">
         <v>4</v>
@@ -51756,7 +51756,7 @@
         <v>1012491</v>
       </c>
       <c r="B1970" s="3" t="s">
-        <v>5877</v>
+        <v>5876</v>
       </c>
       <c r="C1970" s="3" t="s">
         <v>4</v>
@@ -51790,7 +51790,7 @@
         <v>1013869</v>
       </c>
       <c r="B1972" s="3" t="s">
-        <v>5878</v>
+        <v>5877</v>
       </c>
       <c r="C1972" s="3" t="s">
         <v>4</v>
@@ -51841,7 +51841,7 @@
         <v>1016541</v>
       </c>
       <c r="B1975" s="3" t="s">
-        <v>5879</v>
+        <v>5878</v>
       </c>
       <c r="C1975" s="3" t="s">
         <v>4</v>
@@ -51858,7 +51858,7 @@
         <v>1018117</v>
       </c>
       <c r="B1976" s="3" t="s">
-        <v>5880</v>
+        <v>5879</v>
       </c>
       <c r="C1976" s="3" t="s">
         <v>4</v>
@@ -51875,7 +51875,7 @@
         <v>1018638</v>
       </c>
       <c r="B1977" s="3" t="s">
-        <v>5881</v>
+        <v>5880</v>
       </c>
       <c r="C1977" s="3" t="s">
         <v>4</v>
@@ -51943,7 +51943,7 @@
         <v>1021214</v>
       </c>
       <c r="B1981" s="3" t="s">
-        <v>5882</v>
+        <v>5881</v>
       </c>
       <c r="C1981" s="3" t="s">
         <v>4</v>
@@ -51977,7 +51977,7 @@
         <v>1024377</v>
       </c>
       <c r="B1983" s="3" t="s">
-        <v>5883</v>
+        <v>5882</v>
       </c>
       <c r="C1983" s="3" t="s">
         <v>4</v>
@@ -52011,7 +52011,7 @@
         <v>1026143</v>
       </c>
       <c r="B1985" s="3" t="s">
-        <v>5571</v>
+        <v>5570</v>
       </c>
       <c r="C1985" s="3" t="s">
         <v>4</v>
@@ -52079,7 +52079,7 @@
         <v>1028997</v>
       </c>
       <c r="B1989" s="3" t="s">
-        <v>5572</v>
+        <v>5571</v>
       </c>
       <c r="C1989" s="3" t="s">
         <v>4</v>
@@ -52113,7 +52113,7 @@
         <v>1031747</v>
       </c>
       <c r="B1991" s="3" t="s">
-        <v>5884</v>
+        <v>5883</v>
       </c>
       <c r="C1991" s="3" t="s">
         <v>4</v>
@@ -52198,7 +52198,7 @@
         <v>1037645</v>
       </c>
       <c r="B1996" s="3" t="s">
-        <v>5573</v>
+        <v>5572</v>
       </c>
       <c r="C1996" s="3" t="s">
         <v>4</v>
@@ -52232,7 +52232,7 @@
         <v>1039852</v>
       </c>
       <c r="B1998" s="3" t="s">
-        <v>5574</v>
+        <v>5573</v>
       </c>
       <c r="C1998" s="3" t="s">
         <v>4</v>
@@ -52317,7 +52317,7 @@
         <v>1046931</v>
       </c>
       <c r="B2003" s="3" t="s">
-        <v>5575</v>
+        <v>5574</v>
       </c>
       <c r="C2003" s="3" t="s">
         <v>4</v>
@@ -52351,7 +52351,7 @@
         <v>1048745</v>
       </c>
       <c r="B2005" s="3" t="s">
-        <v>5885</v>
+        <v>5884</v>
       </c>
       <c r="C2005" s="3" t="s">
         <v>4</v>
@@ -52453,7 +52453,7 @@
         <v>1050566</v>
       </c>
       <c r="B2011" s="3" t="s">
-        <v>5576</v>
+        <v>5575</v>
       </c>
       <c r="C2011" s="3" t="s">
         <v>4</v>
@@ -52538,7 +52538,7 @@
         <v>1052686</v>
       </c>
       <c r="B2016" s="3" t="s">
-        <v>5577</v>
+        <v>5576</v>
       </c>
       <c r="C2016" s="3" t="s">
         <v>4</v>
@@ -52606,7 +52606,7 @@
         <v>1056353</v>
       </c>
       <c r="B2020" s="3" t="s">
-        <v>5886</v>
+        <v>5885</v>
       </c>
       <c r="C2020" s="3" t="s">
         <v>4</v>
@@ -52657,7 +52657,7 @@
         <v>1059131</v>
       </c>
       <c r="B2023" s="3" t="s">
-        <v>5578</v>
+        <v>5577</v>
       </c>
       <c r="C2023" s="3" t="s">
         <v>4</v>
@@ -52674,7 +52674,7 @@
         <v>1060800</v>
       </c>
       <c r="B2024" s="3" t="s">
-        <v>5579</v>
+        <v>5578</v>
       </c>
       <c r="C2024" s="3" t="s">
         <v>4</v>
@@ -52776,7 +52776,7 @@
         <v>1068978</v>
       </c>
       <c r="B2030" s="3" t="s">
-        <v>5887</v>
+        <v>5886</v>
       </c>
       <c r="C2030" s="3" t="s">
         <v>4</v>
@@ -52810,7 +52810,7 @@
         <v>1071021</v>
       </c>
       <c r="B2032" s="3" t="s">
-        <v>5580</v>
+        <v>5579</v>
       </c>
       <c r="C2032" s="3" t="s">
         <v>4</v>
@@ -52878,7 +52878,7 @@
         <v>1073213</v>
       </c>
       <c r="B2036" s="3" t="s">
-        <v>5888</v>
+        <v>5887</v>
       </c>
       <c r="C2036" s="3" t="s">
         <v>4</v>
@@ -52895,7 +52895,7 @@
         <v>1073948</v>
       </c>
       <c r="B2037" s="3" t="s">
-        <v>5581</v>
+        <v>5580</v>
       </c>
       <c r="C2037" s="3" t="s">
         <v>4</v>
@@ -52929,7 +52929,7 @@
         <v>1074228</v>
       </c>
       <c r="B2039" s="3" t="s">
-        <v>5889</v>
+        <v>5888</v>
       </c>
       <c r="C2039" s="3" t="s">
         <v>4</v>
@@ -53031,7 +53031,7 @@
         <v>1078485</v>
       </c>
       <c r="B2045" s="3" t="s">
-        <v>5890</v>
+        <v>5889</v>
       </c>
       <c r="C2045" s="3" t="s">
         <v>4</v>
@@ -53167,7 +53167,7 @@
         <v>1084345</v>
       </c>
       <c r="B2053" s="3" t="s">
-        <v>5891</v>
+        <v>5890</v>
       </c>
       <c r="C2053" s="3" t="s">
         <v>4</v>
@@ -53320,7 +53320,7 @@
         <v>1091726</v>
       </c>
       <c r="B2062" s="3" t="s">
-        <v>5582</v>
+        <v>5581</v>
       </c>
       <c r="C2062" s="3" t="s">
         <v>4</v>
@@ -53456,7 +53456,7 @@
         <v>1099041</v>
       </c>
       <c r="B2070" s="3" t="s">
-        <v>5583</v>
+        <v>5582</v>
       </c>
       <c r="C2070" s="3" t="s">
         <v>4</v>
@@ -53507,7 +53507,7 @@
         <v>1101870</v>
       </c>
       <c r="B2073" s="3" t="s">
-        <v>5892</v>
+        <v>5891</v>
       </c>
       <c r="C2073" s="3" t="s">
         <v>4</v>
@@ -53524,7 +53524,7 @@
         <v>1102128</v>
       </c>
       <c r="B2074" s="3" t="s">
-        <v>5584</v>
+        <v>5583</v>
       </c>
       <c r="C2074" s="3" t="s">
         <v>4</v>
@@ -53779,7 +53779,7 @@
         <v>1112419</v>
       </c>
       <c r="B2089" s="3" t="s">
-        <v>5893</v>
+        <v>5892</v>
       </c>
       <c r="C2089" s="3" t="s">
         <v>4</v>
@@ -53898,7 +53898,7 @@
         <v>1123804</v>
       </c>
       <c r="B2096" s="3" t="s">
-        <v>5585</v>
+        <v>5584</v>
       </c>
       <c r="C2096" s="3" t="s">
         <v>4</v>
@@ -54017,7 +54017,7 @@
         <v>1128085</v>
       </c>
       <c r="B2103" s="3" t="s">
-        <v>5586</v>
+        <v>5585</v>
       </c>
       <c r="C2103" s="3" t="s">
         <v>4</v>
@@ -54034,7 +54034,7 @@
         <v>1128680</v>
       </c>
       <c r="B2104" s="3" t="s">
-        <v>5894</v>
+        <v>5893</v>
       </c>
       <c r="C2104" s="3" t="s">
         <v>4</v>
@@ -54119,7 +54119,7 @@
         <v>1131013</v>
       </c>
       <c r="B2109" s="3" t="s">
-        <v>5895</v>
+        <v>5894</v>
       </c>
       <c r="C2109" s="3" t="s">
         <v>4</v>
@@ -54153,7 +54153,7 @@
         <v>1133475</v>
       </c>
       <c r="B2111" s="3" t="s">
-        <v>5587</v>
+        <v>5586</v>
       </c>
       <c r="C2111" s="3" t="s">
         <v>4</v>
@@ -54289,7 +54289,7 @@
         <v>1140377</v>
       </c>
       <c r="B2119" s="3" t="s">
-        <v>5588</v>
+        <v>5587</v>
       </c>
       <c r="C2119" s="3" t="s">
         <v>4</v>
@@ -54374,7 +54374,7 @@
         <v>1143864</v>
       </c>
       <c r="B2124" s="3" t="s">
-        <v>5896</v>
+        <v>5895</v>
       </c>
       <c r="C2124" s="3" t="s">
         <v>4</v>
@@ -54527,7 +54527,7 @@
         <v>1151083</v>
       </c>
       <c r="B2133" s="3" t="s">
-        <v>5589</v>
+        <v>5588</v>
       </c>
       <c r="C2133" s="3" t="s">
         <v>4</v>
@@ -54969,7 +54969,7 @@
         <v>1197166</v>
       </c>
       <c r="B2159" s="3" t="s">
-        <v>5590</v>
+        <v>5589</v>
       </c>
       <c r="C2159" s="3" t="s">
         <v>4</v>
@@ -55003,7 +55003,7 @@
         <v>1199451</v>
       </c>
       <c r="B2161" s="3" t="s">
-        <v>5897</v>
+        <v>5896</v>
       </c>
       <c r="C2161" s="3" t="s">
         <v>4</v>
@@ -55190,7 +55190,7 @@
         <v>1204446</v>
       </c>
       <c r="B2172" s="3" t="s">
-        <v>5591</v>
+        <v>5590</v>
       </c>
       <c r="C2172" s="3" t="s">
         <v>4</v>
@@ -55275,7 +55275,7 @@
         <v>1208680</v>
       </c>
       <c r="B2177" s="3" t="s">
-        <v>5592</v>
+        <v>5591</v>
       </c>
       <c r="C2177" s="3" t="s">
         <v>4</v>
@@ -55411,7 +55411,7 @@
         <v>1217078</v>
       </c>
       <c r="B2185" s="3" t="s">
-        <v>5898</v>
+        <v>5897</v>
       </c>
       <c r="C2185" s="3" t="s">
         <v>4</v>
@@ -55428,7 +55428,7 @@
         <v>1218167</v>
       </c>
       <c r="B2186" s="3" t="s">
-        <v>5593</v>
+        <v>5592</v>
       </c>
       <c r="C2186" s="3" t="s">
         <v>4</v>
@@ -55445,7 +55445,7 @@
         <v>1218658</v>
       </c>
       <c r="B2187" s="3" t="s">
-        <v>5594</v>
+        <v>5593</v>
       </c>
       <c r="C2187" s="3" t="s">
         <v>4</v>
@@ -55479,7 +55479,7 @@
         <v>1219803</v>
       </c>
       <c r="B2189" s="3" t="s">
-        <v>5899</v>
+        <v>5898</v>
       </c>
       <c r="C2189" s="3" t="s">
         <v>4</v>
@@ -55547,7 +55547,7 @@
         <v>1225266</v>
       </c>
       <c r="B2193" s="3" t="s">
-        <v>5900</v>
+        <v>5899</v>
       </c>
       <c r="C2193" s="3" t="s">
         <v>4</v>
@@ -55683,7 +55683,7 @@
         <v>1236427</v>
       </c>
       <c r="B2201" s="3" t="s">
-        <v>5901</v>
+        <v>5900</v>
       </c>
       <c r="C2201" s="3" t="s">
         <v>4</v>
@@ -55717,7 +55717,7 @@
         <v>1239005</v>
       </c>
       <c r="B2203" s="3" t="s">
-        <v>5902</v>
+        <v>5901</v>
       </c>
       <c r="C2203" s="3" t="s">
         <v>4</v>
@@ -55870,7 +55870,7 @@
         <v>1245373</v>
       </c>
       <c r="B2212" s="3" t="s">
-        <v>5903</v>
+        <v>5902</v>
       </c>
       <c r="C2212" s="3" t="s">
         <v>4</v>
@@ -55887,7 +55887,7 @@
         <v>1246547</v>
       </c>
       <c r="B2213" s="3" t="s">
-        <v>5904</v>
+        <v>5903</v>
       </c>
       <c r="C2213" s="3" t="s">
         <v>4</v>
@@ -55972,7 +55972,7 @@
         <v>1253912</v>
       </c>
       <c r="B2218" s="3" t="s">
-        <v>5595</v>
+        <v>5594</v>
       </c>
       <c r="C2218" s="3" t="s">
         <v>4</v>
@@ -56074,7 +56074,7 @@
         <v>1257253</v>
       </c>
       <c r="B2224" s="3" t="s">
-        <v>5905</v>
+        <v>5904</v>
       </c>
       <c r="C2224" s="3" t="s">
         <v>4</v>
@@ -56142,7 +56142,7 @@
         <v>1260769</v>
       </c>
       <c r="B2228" s="3" t="s">
-        <v>5906</v>
+        <v>5905</v>
       </c>
       <c r="C2228" s="3" t="s">
         <v>4</v>
@@ -56176,7 +56176,7 @@
         <v>1261859</v>
       </c>
       <c r="B2230" s="3" t="s">
-        <v>5596</v>
+        <v>5595</v>
       </c>
       <c r="C2230" s="3" t="s">
         <v>4</v>
@@ -56295,7 +56295,7 @@
         <v>1274405</v>
       </c>
       <c r="B2237" s="3" t="s">
-        <v>5907</v>
+        <v>5906</v>
       </c>
       <c r="C2237" s="3" t="s">
         <v>4</v>
@@ -56431,7 +56431,7 @@
         <v>1285695</v>
       </c>
       <c r="B2245" s="3" t="s">
-        <v>5597</v>
+        <v>5596</v>
       </c>
       <c r="C2245" s="3" t="s">
         <v>4</v>
@@ -56652,7 +56652,7 @@
         <v>1304324</v>
       </c>
       <c r="B2258" s="3" t="s">
-        <v>5598</v>
+        <v>5597</v>
       </c>
       <c r="C2258" s="3" t="s">
         <v>4</v>
@@ -56805,7 +56805,7 @@
         <v>1312513</v>
       </c>
       <c r="B2267" s="3" t="s">
-        <v>5908</v>
+        <v>5907</v>
       </c>
       <c r="C2267" s="3" t="s">
         <v>4</v>
@@ -56822,7 +56822,7 @@
         <v>1312635</v>
       </c>
       <c r="B2268" s="3" t="s">
-        <v>5599</v>
+        <v>5598</v>
       </c>
       <c r="C2268" s="3" t="s">
         <v>4</v>
@@ -56873,7 +56873,7 @@
         <v>1317946</v>
       </c>
       <c r="B2271" s="3" t="s">
-        <v>5600</v>
+        <v>5599</v>
       </c>
       <c r="C2271" s="3" t="s">
         <v>4</v>
@@ -57077,7 +57077,7 @@
         <v>1335418</v>
       </c>
       <c r="B2283" s="3" t="s">
-        <v>5601</v>
+        <v>5600</v>
       </c>
       <c r="C2283" s="3" t="s">
         <v>4</v>
@@ -57111,7 +57111,7 @@
         <v>1336417</v>
       </c>
       <c r="B2285" s="3" t="s">
-        <v>5909</v>
+        <v>5908</v>
       </c>
       <c r="C2285" s="3" t="s">
         <v>4</v>
@@ -57349,7 +57349,7 @@
         <v>1350483</v>
       </c>
       <c r="B2299" s="3" t="s">
-        <v>5602</v>
+        <v>5601</v>
       </c>
       <c r="C2299" s="3" t="s">
         <v>4</v>
@@ -57383,7 +57383,7 @@
         <v>1351666</v>
       </c>
       <c r="B2301" s="3" t="s">
-        <v>5603</v>
+        <v>5602</v>
       </c>
       <c r="C2301" s="3" t="s">
         <v>4</v>
@@ -57740,7 +57740,7 @@
         <v>1385822</v>
       </c>
       <c r="B2322" s="3" t="s">
-        <v>5910</v>
+        <v>5909</v>
       </c>
       <c r="C2322" s="3" t="s">
         <v>4</v>
@@ -57825,7 +57825,7 @@
         <v>1390207</v>
       </c>
       <c r="B2327" s="3" t="s">
-        <v>5604</v>
+        <v>5603</v>
       </c>
       <c r="C2327" s="3" t="s">
         <v>4</v>
@@ -57944,7 +57944,7 @@
         <v>1397375</v>
       </c>
       <c r="B2334" s="3" t="s">
-        <v>5911</v>
+        <v>5910</v>
       </c>
       <c r="C2334" s="3" t="s">
         <v>4</v>
@@ -58063,7 +58063,7 @@
         <v>1409685</v>
       </c>
       <c r="B2341" s="3" t="s">
-        <v>5605</v>
+        <v>5604</v>
       </c>
       <c r="C2341" s="3" t="s">
         <v>4</v>
@@ -58216,7 +58216,7 @@
         <v>1419661</v>
       </c>
       <c r="B2350" s="3" t="s">
-        <v>5606</v>
+        <v>5605</v>
       </c>
       <c r="C2350" s="3" t="s">
         <v>4</v>
@@ -58301,7 +58301,7 @@
         <v>1422247</v>
       </c>
       <c r="B2355" s="3" t="s">
-        <v>5607</v>
+        <v>5606</v>
       </c>
       <c r="C2355" s="3" t="s">
         <v>4</v>
@@ -58352,7 +58352,7 @@
         <v>1422846</v>
       </c>
       <c r="B2358" s="3" t="s">
-        <v>5912</v>
+        <v>5911</v>
       </c>
       <c r="C2358" s="3" t="s">
         <v>4</v>
@@ -58386,7 +58386,7 @@
         <v>1423880</v>
       </c>
       <c r="B2360" s="3" t="s">
-        <v>5608</v>
+        <v>5607</v>
       </c>
       <c r="C2360" s="3" t="s">
         <v>4</v>
@@ -58539,7 +58539,7 @@
         <v>1429968</v>
       </c>
       <c r="B2369" s="3" t="s">
-        <v>5609</v>
+        <v>5608</v>
       </c>
       <c r="C2369" s="3" t="s">
         <v>4</v>
@@ -58692,7 +58692,7 @@
         <v>1442654</v>
       </c>
       <c r="B2378" s="3" t="s">
-        <v>5913</v>
+        <v>5912</v>
       </c>
       <c r="C2378" s="3" t="s">
         <v>4</v>
@@ -58743,7 +58743,7 @@
         <v>1447752</v>
       </c>
       <c r="B2381" s="3" t="s">
-        <v>5914</v>
+        <v>5913</v>
       </c>
       <c r="C2381" s="3" t="s">
         <v>4</v>
@@ -58845,7 +58845,7 @@
         <v>1452913</v>
       </c>
       <c r="B2387" s="3" t="s">
-        <v>5610</v>
+        <v>5609</v>
       </c>
       <c r="C2387" s="3" t="s">
         <v>4</v>
@@ -59015,7 +59015,7 @@
         <v>1465959</v>
       </c>
       <c r="B2397" s="3" t="s">
-        <v>5611</v>
+        <v>5610</v>
       </c>
       <c r="C2397" s="3" t="s">
         <v>4</v>
@@ -59134,7 +59134,7 @@
         <v>1474089</v>
       </c>
       <c r="B2404" s="3" t="s">
-        <v>5612</v>
+        <v>5611</v>
       </c>
       <c r="C2404" s="3" t="s">
         <v>4</v>
@@ -59321,7 +59321,7 @@
         <v>1481741</v>
       </c>
       <c r="B2415" s="3" t="s">
-        <v>5915</v>
+        <v>5914</v>
       </c>
       <c r="C2415" s="3" t="s">
         <v>4</v>
@@ -59355,7 +59355,7 @@
         <v>1482046</v>
       </c>
       <c r="B2417" s="3" t="s">
-        <v>5613</v>
+        <v>5612</v>
       </c>
       <c r="C2417" s="3" t="s">
         <v>4</v>
@@ -59644,7 +59644,7 @@
         <v>1516688</v>
       </c>
       <c r="B2434" s="3" t="s">
-        <v>5614</v>
+        <v>5613</v>
       </c>
       <c r="C2434" s="3" t="s">
         <v>4</v>
@@ -59678,7 +59678,7 @@
         <v>1516796</v>
       </c>
       <c r="B2436" s="3" t="s">
-        <v>5615</v>
+        <v>5614</v>
       </c>
       <c r="C2436" s="3" t="s">
         <v>4</v>
@@ -59695,7 +59695,7 @@
         <v>1517415</v>
       </c>
       <c r="B2437" s="3" t="s">
-        <v>5616</v>
+        <v>5615</v>
       </c>
       <c r="C2437" s="3" t="s">
         <v>4</v>
@@ -59746,7 +59746,7 @@
         <v>1522681</v>
       </c>
       <c r="B2440" s="3" t="s">
-        <v>5617</v>
+        <v>5616</v>
       </c>
       <c r="C2440" s="3" t="s">
         <v>4</v>
@@ -59916,7 +59916,7 @@
         <v>1530118</v>
       </c>
       <c r="B2450" s="3" t="s">
-        <v>5916</v>
+        <v>5915</v>
       </c>
       <c r="C2450" s="3" t="s">
         <v>4</v>
@@ -60273,7 +60273,7 @@
         <v>1563243</v>
       </c>
       <c r="B2471" s="3" t="s">
-        <v>5917</v>
+        <v>5916</v>
       </c>
       <c r="C2471" s="3" t="s">
         <v>4</v>
@@ -60494,7 +60494,7 @@
         <v>1578153</v>
       </c>
       <c r="B2484" s="3" t="s">
-        <v>5918</v>
+        <v>5917</v>
       </c>
       <c r="C2484" s="3" t="s">
         <v>4</v>
@@ -60511,7 +60511,7 @@
         <v>1578200</v>
       </c>
       <c r="B2485" s="3" t="s">
-        <v>5618</v>
+        <v>5617</v>
       </c>
       <c r="C2485" s="3" t="s">
         <v>4</v>
@@ -60545,7 +60545,7 @@
         <v>1583807</v>
       </c>
       <c r="B2487" s="3" t="s">
-        <v>5619</v>
+        <v>5618</v>
       </c>
       <c r="C2487" s="3" t="s">
         <v>4</v>
@@ -60715,7 +60715,7 @@
         <v>1593477</v>
       </c>
       <c r="B2497" s="3" t="s">
-        <v>5919</v>
+        <v>5918</v>
       </c>
       <c r="C2497" s="3" t="s">
         <v>4</v>
@@ -60902,7 +60902,7 @@
         <v>1603362</v>
       </c>
       <c r="B2508" s="3" t="s">
-        <v>5920</v>
+        <v>5919</v>
       </c>
       <c r="C2508" s="3" t="s">
         <v>4</v>
@@ -60936,7 +60936,7 @@
         <v>1605525</v>
       </c>
       <c r="B2510" s="3" t="s">
-        <v>5921</v>
+        <v>5920</v>
       </c>
       <c r="C2510" s="3" t="s">
         <v>4</v>
@@ -61004,7 +61004,7 @@
         <v>1606578</v>
       </c>
       <c r="B2514" s="3" t="s">
-        <v>5922</v>
+        <v>5921</v>
       </c>
       <c r="C2514" s="3" t="s">
         <v>4</v>
@@ -61089,7 +61089,7 @@
         <v>1608791</v>
       </c>
       <c r="B2519" s="3" t="s">
-        <v>5620</v>
+        <v>5619</v>
       </c>
       <c r="C2519" s="3" t="s">
         <v>4</v>
@@ -61106,7 +61106,7 @@
         <v>1611527</v>
       </c>
       <c r="B2520" s="3" t="s">
-        <v>5621</v>
+        <v>5620</v>
       </c>
       <c r="C2520" s="3" t="s">
         <v>4</v>
@@ -61378,7 +61378,7 @@
         <v>1625129</v>
       </c>
       <c r="B2536" s="3" t="s">
-        <v>5622</v>
+        <v>5621</v>
       </c>
       <c r="C2536" s="3" t="s">
         <v>4</v>
@@ -61973,7 +61973,7 @@
         <v>1657935</v>
       </c>
       <c r="B2571" s="3" t="s">
-        <v>5623</v>
+        <v>5622</v>
       </c>
       <c r="C2571" s="3" t="s">
         <v>4</v>
@@ -62109,7 +62109,7 @@
         <v>1665231</v>
       </c>
       <c r="B2579" s="3" t="s">
-        <v>5624</v>
+        <v>5623</v>
       </c>
       <c r="C2579" s="3" t="s">
         <v>4</v>
@@ -62211,7 +62211,7 @@
         <v>1671262</v>
       </c>
       <c r="B2585" s="3" t="s">
-        <v>5923</v>
+        <v>5922</v>
       </c>
       <c r="C2585" s="3" t="s">
         <v>4</v>
@@ -62636,7 +62636,7 @@
         <v>1699443</v>
       </c>
       <c r="B2610" s="3" t="s">
-        <v>5924</v>
+        <v>5923</v>
       </c>
       <c r="C2610" s="3" t="s">
         <v>4</v>
@@ -62704,7 +62704,7 @@
         <v>1701693</v>
       </c>
       <c r="B2614" s="3" t="s">
-        <v>5625</v>
+        <v>5624</v>
       </c>
       <c r="C2614" s="3" t="s">
         <v>4</v>
@@ -62755,7 +62755,7 @@
         <v>1707533</v>
       </c>
       <c r="B2617" s="3" t="s">
-        <v>5925</v>
+        <v>5924</v>
       </c>
       <c r="C2617" s="3" t="s">
         <v>4</v>
@@ -62772,7 +62772,7 @@
         <v>1709011</v>
       </c>
       <c r="B2618" s="3" t="s">
-        <v>5926</v>
+        <v>5925</v>
       </c>
       <c r="C2618" s="3" t="s">
         <v>4</v>
@@ -62789,7 +62789,7 @@
         <v>1709744</v>
       </c>
       <c r="B2619" s="3" t="s">
-        <v>5626</v>
+        <v>5625</v>
       </c>
       <c r="C2619" s="3" t="s">
         <v>4</v>
@@ -62857,7 +62857,7 @@
         <v>1713978</v>
       </c>
       <c r="B2623" s="3" t="s">
-        <v>5627</v>
+        <v>5626</v>
       </c>
       <c r="C2623" s="3" t="s">
         <v>4</v>
@@ -62976,7 +62976,7 @@
         <v>1716746</v>
       </c>
       <c r="B2630" s="3" t="s">
-        <v>5927</v>
+        <v>5926</v>
       </c>
       <c r="C2630" s="3" t="s">
         <v>4</v>
@@ -63231,7 +63231,7 @@
         <v>1730428</v>
       </c>
       <c r="B2645" s="3" t="s">
-        <v>5628</v>
+        <v>5627</v>
       </c>
       <c r="C2645" s="3" t="s">
         <v>4</v>
@@ -63503,7 +63503,7 @@
         <v>1741495</v>
       </c>
       <c r="B2661" s="3" t="s">
-        <v>5629</v>
+        <v>5628</v>
       </c>
       <c r="C2661" s="3" t="s">
         <v>4</v>
@@ -63690,7 +63690,7 @@
         <v>1760183</v>
       </c>
       <c r="B2672" s="3" t="s">
-        <v>5630</v>
+        <v>5629</v>
       </c>
       <c r="C2672" s="3" t="s">
         <v>4</v>
@@ -63809,7 +63809,7 @@
         <v>1774566</v>
       </c>
       <c r="B2679" s="3" t="s">
-        <v>5928</v>
+        <v>5927</v>
       </c>
       <c r="C2679" s="3" t="s">
         <v>4</v>
@@ -63928,7 +63928,7 @@
         <v>1784838</v>
       </c>
       <c r="B2686" s="3" t="s">
-        <v>5631</v>
+        <v>5630</v>
       </c>
       <c r="C2686" s="3" t="s">
         <v>4</v>
@@ -63945,7 +63945,7 @@
         <v>1785221</v>
       </c>
       <c r="B2687" s="3" t="s">
-        <v>5632</v>
+        <v>5631</v>
       </c>
       <c r="C2687" s="3" t="s">
         <v>4</v>
@@ -63979,7 +63979,7 @@
         <v>1788095</v>
       </c>
       <c r="B2689" s="3" t="s">
-        <v>5929</v>
+        <v>5928</v>
       </c>
       <c r="C2689" s="3" t="s">
         <v>4</v>
@@ -63996,7 +63996,7 @@
         <v>1788387</v>
       </c>
       <c r="B2690" s="3" t="s">
-        <v>5633</v>
+        <v>5632</v>
       </c>
       <c r="C2690" s="3" t="s">
         <v>4</v>
@@ -64251,7 +64251,7 @@
         <v>1799298</v>
       </c>
       <c r="B2705" s="3" t="s">
-        <v>5930</v>
+        <v>5929</v>
       </c>
       <c r="C2705" s="3" t="s">
         <v>4</v>
@@ -64438,7 +64438,7 @@
         <v>1817438</v>
       </c>
       <c r="B2716" s="3" t="s">
-        <v>5634</v>
+        <v>5633</v>
       </c>
       <c r="C2716" s="3" t="s">
         <v>4</v>
@@ -64472,7 +64472,7 @@
         <v>1824240</v>
       </c>
       <c r="B2718" s="3" t="s">
-        <v>5931</v>
+        <v>5930</v>
       </c>
       <c r="C2718" s="3" t="s">
         <v>4</v>
@@ -64489,7 +64489,7 @@
         <v>1828587</v>
       </c>
       <c r="B2719" s="3" t="s">
-        <v>5932</v>
+        <v>5931</v>
       </c>
       <c r="C2719" s="3" t="s">
         <v>4</v>
@@ -64557,7 +64557,7 @@
         <v>1836903</v>
       </c>
       <c r="B2723" s="3" t="s">
-        <v>5933</v>
+        <v>5932</v>
       </c>
       <c r="C2723" s="3" t="s">
         <v>4</v>
@@ -64931,7 +64931,7 @@
         <v>1853556</v>
       </c>
       <c r="B2745" s="3" t="s">
-        <v>5635</v>
+        <v>5634</v>
       </c>
       <c r="C2745" s="3" t="s">
         <v>4</v>
@@ -65084,7 +65084,7 @@
         <v>1864820</v>
       </c>
       <c r="B2754" s="3" t="s">
-        <v>5636</v>
+        <v>5635</v>
       </c>
       <c r="C2754" s="3" t="s">
         <v>4</v>
@@ -65118,7 +65118,7 @@
         <v>1871096</v>
       </c>
       <c r="B2756" s="3" t="s">
-        <v>5637</v>
+        <v>5636</v>
       </c>
       <c r="C2756" s="3" t="s">
         <v>4</v>
@@ -65169,7 +65169,7 @@
         <v>1876106</v>
       </c>
       <c r="B2759" s="3" t="s">
-        <v>5638</v>
+        <v>5637</v>
       </c>
       <c r="C2759" s="3" t="s">
         <v>4</v>
@@ -65203,7 +65203,7 @@
         <v>1877654</v>
       </c>
       <c r="B2761" s="3" t="s">
-        <v>5639</v>
+        <v>5638</v>
       </c>
       <c r="C2761" s="3" t="s">
         <v>4</v>
@@ -65254,7 +65254,7 @@
         <v>1885837</v>
       </c>
       <c r="B2764" s="3" t="s">
-        <v>5640</v>
+        <v>5639</v>
       </c>
       <c r="C2764" s="3" t="s">
         <v>4</v>
@@ -65390,7 +65390,7 @@
         <v>1894218</v>
       </c>
       <c r="B2772" s="3" t="s">
-        <v>5641</v>
+        <v>5640</v>
       </c>
       <c r="C2772" s="3" t="s">
         <v>4</v>
@@ -65441,7 +65441,7 @@
         <v>1897397</v>
       </c>
       <c r="B2775" s="3" t="s">
-        <v>5642</v>
+        <v>5641</v>
       </c>
       <c r="C2775" s="3" t="s">
         <v>4</v>
@@ -65509,7 +65509,7 @@
         <v>1902089</v>
       </c>
       <c r="B2779" s="3" t="s">
-        <v>5643</v>
+        <v>5642</v>
       </c>
       <c r="C2779" s="3" t="s">
         <v>4</v>
@@ -65594,7 +65594,7 @@
         <v>1912440</v>
       </c>
       <c r="B2784" s="3" t="s">
-        <v>5644</v>
+        <v>5643</v>
       </c>
       <c r="C2784" s="3" t="s">
         <v>4</v>
@@ -65696,7 +65696,7 @@
         <v>1922769</v>
       </c>
       <c r="B2790" s="3" t="s">
-        <v>5934</v>
+        <v>5933</v>
       </c>
       <c r="C2790" s="3" t="s">
         <v>4</v>
@@ -65730,7 +65730,7 @@
         <v>1924572</v>
       </c>
       <c r="B2792" s="3" t="s">
-        <v>5645</v>
+        <v>5644</v>
       </c>
       <c r="C2792" s="3" t="s">
         <v>4</v>
@@ -65747,7 +65747,7 @@
         <v>1925698</v>
       </c>
       <c r="B2793" s="3" t="s">
-        <v>5935</v>
+        <v>5934</v>
       </c>
       <c r="C2793" s="3" t="s">
         <v>4</v>
@@ -65968,7 +65968,7 @@
         <v>1936005</v>
       </c>
       <c r="B2806" s="3" t="s">
-        <v>5936</v>
+        <v>5935</v>
       </c>
       <c r="C2806" s="3" t="s">
         <v>4</v>
@@ -65985,7 +65985,7 @@
         <v>1936921</v>
       </c>
       <c r="B2807" s="3" t="s">
-        <v>5646</v>
+        <v>5645</v>
       </c>
       <c r="C2807" s="3" t="s">
         <v>4</v>
@@ -66121,7 +66121,7 @@
         <v>1945526</v>
       </c>
       <c r="B2815" s="3" t="s">
-        <v>5647</v>
+        <v>5646</v>
       </c>
       <c r="C2815" s="3" t="s">
         <v>4</v>
@@ -66138,7 +66138,7 @@
         <v>1945782</v>
       </c>
       <c r="B2816" s="3" t="s">
-        <v>5648</v>
+        <v>5647</v>
       </c>
       <c r="C2816" s="3" t="s">
         <v>4</v>
@@ -66189,7 +66189,7 @@
         <v>1947939</v>
       </c>
       <c r="B2819" s="3" t="s">
-        <v>5937</v>
+        <v>5936</v>
       </c>
       <c r="C2819" s="3" t="s">
         <v>4</v>
@@ -66206,7 +66206,7 @@
         <v>1948863</v>
       </c>
       <c r="B2820" s="3" t="s">
-        <v>5938</v>
+        <v>5937</v>
       </c>
       <c r="C2820" s="3" t="s">
         <v>4</v>
@@ -66223,7 +66223,7 @@
         <v>1949059</v>
       </c>
       <c r="B2821" s="3" t="s">
-        <v>5649</v>
+        <v>5648</v>
       </c>
       <c r="C2821" s="3" t="s">
         <v>4</v>
@@ -66546,7 +66546,7 @@
         <v>1968563</v>
       </c>
       <c r="B2840" s="3" t="s">
-        <v>5650</v>
+        <v>5649</v>
       </c>
       <c r="C2840" s="3" t="s">
         <v>4</v>
@@ -66580,7 +66580,7 @@
         <v>1970348</v>
       </c>
       <c r="B2842" s="3" t="s">
-        <v>5651</v>
+        <v>5650</v>
       </c>
       <c r="C2842" s="3" t="s">
         <v>4</v>
@@ -66614,7 +66614,7 @@
         <v>1977273</v>
       </c>
       <c r="B2844" s="3" t="s">
-        <v>5939</v>
+        <v>5938</v>
       </c>
       <c r="C2844" s="3" t="s">
         <v>4</v>
@@ -66631,7 +66631,7 @@
         <v>1981639</v>
       </c>
       <c r="B2845" s="3" t="s">
-        <v>5940</v>
+        <v>5939</v>
       </c>
       <c r="C2845" s="3" t="s">
         <v>4</v>
@@ -66818,7 +66818,7 @@
         <v>2004435</v>
       </c>
       <c r="B2856" s="3" t="s">
-        <v>5652</v>
+        <v>5651</v>
       </c>
       <c r="C2856" s="3" t="s">
         <v>4</v>
@@ -66835,7 +66835,7 @@
         <v>2005460</v>
       </c>
       <c r="B2857" s="3" t="s">
-        <v>5653</v>
+        <v>5652</v>
       </c>
       <c r="C2857" s="3" t="s">
         <v>4</v>
@@ -66869,7 +66869,7 @@
         <v>2006759</v>
       </c>
       <c r="B2859" s="3" t="s">
-        <v>5941</v>
+        <v>5940</v>
       </c>
       <c r="C2859" s="3" t="s">
         <v>4</v>
@@ -66903,7 +66903,7 @@
         <v>2007122</v>
       </c>
       <c r="B2861" s="3" t="s">
-        <v>5654</v>
+        <v>5653</v>
       </c>
       <c r="C2861" s="3" t="s">
         <v>4</v>
@@ -67022,7 +67022,7 @@
         <v>2015755</v>
       </c>
       <c r="B2868" s="3" t="s">
-        <v>5655</v>
+        <v>5654</v>
       </c>
       <c r="C2868" s="3" t="s">
         <v>4</v>
@@ -67209,7 +67209,7 @@
         <v>2031153</v>
       </c>
       <c r="B2879" s="3" t="s">
-        <v>5942</v>
+        <v>5941</v>
       </c>
       <c r="C2879" s="3" t="s">
         <v>4</v>
@@ -67294,7 +67294,7 @@
         <v>2035055</v>
       </c>
       <c r="B2884" s="3" t="s">
-        <v>5656</v>
+        <v>5655</v>
       </c>
       <c r="C2884" s="3" t="s">
         <v>4</v>
@@ -67345,7 +67345,7 @@
         <v>2039927</v>
       </c>
       <c r="B2887" s="3" t="s">
-        <v>5657</v>
+        <v>5656</v>
       </c>
       <c r="C2887" s="3" t="s">
         <v>4</v>
@@ -67821,7 +67821,7 @@
         <v>2067751</v>
       </c>
       <c r="B2915" s="3" t="s">
-        <v>5658</v>
+        <v>5657</v>
       </c>
       <c r="C2915" s="3" t="s">
         <v>4</v>
@@ -67889,7 +67889,7 @@
         <v>2071331</v>
       </c>
       <c r="B2919" s="3" t="s">
-        <v>5659</v>
+        <v>5658</v>
       </c>
       <c r="C2919" s="3" t="s">
         <v>4</v>
@@ -67923,7 +67923,7 @@
         <v>2072627</v>
       </c>
       <c r="B2921" s="3" t="s">
-        <v>5943</v>
+        <v>5942</v>
       </c>
       <c r="C2921" s="3" t="s">
         <v>4</v>
@@ -67957,7 +67957,7 @@
         <v>2078387</v>
       </c>
       <c r="B2923" s="3" t="s">
-        <v>5660</v>
+        <v>5659</v>
       </c>
       <c r="C2923" s="3" t="s">
         <v>4</v>
@@ -67974,7 +67974,7 @@
         <v>2079588</v>
       </c>
       <c r="B2924" s="3" t="s">
-        <v>5944</v>
+        <v>5943</v>
       </c>
       <c r="C2924" s="3" t="s">
         <v>4</v>
@@ -68008,7 +68008,7 @@
         <v>2082859</v>
       </c>
       <c r="B2926" s="3" t="s">
-        <v>5945</v>
+        <v>5944</v>
       </c>
       <c r="C2926" s="3" t="s">
         <v>4</v>
@@ -68246,7 +68246,7 @@
         <v>2093311</v>
       </c>
       <c r="B2940" s="3" t="s">
-        <v>5661</v>
+        <v>5660</v>
       </c>
       <c r="C2940" s="3" t="s">
         <v>4</v>
@@ -68450,7 +68450,7 @@
         <v>2102652</v>
       </c>
       <c r="B2952" s="3" t="s">
-        <v>5662</v>
+        <v>5661</v>
       </c>
       <c r="C2952" s="3" t="s">
         <v>4</v>
@@ -68484,7 +68484,7 @@
         <v>2102961</v>
       </c>
       <c r="B2954" s="3" t="s">
-        <v>5663</v>
+        <v>5662</v>
       </c>
       <c r="C2954" s="3" t="s">
         <v>4</v>
@@ -68518,7 +68518,7 @@
         <v>2107643</v>
       </c>
       <c r="B2956" s="3" t="s">
-        <v>5946</v>
+        <v>5945</v>
       </c>
       <c r="C2956" s="3" t="s">
         <v>4</v>
@@ -68688,7 +68688,7 @@
         <v>2118160</v>
       </c>
       <c r="B2966" s="3" t="s">
-        <v>5664</v>
+        <v>5663</v>
       </c>
       <c r="C2966" s="3" t="s">
         <v>4</v>
@@ -68705,7 +68705,7 @@
         <v>2120883</v>
       </c>
       <c r="B2967" s="3" t="s">
-        <v>5665</v>
+        <v>5664</v>
       </c>
       <c r="C2967" s="3" t="s">
         <v>4</v>
@@ -68807,7 +68807,7 @@
         <v>2124341</v>
       </c>
       <c r="B2973" s="3" t="s">
-        <v>5666</v>
+        <v>5665</v>
       </c>
       <c r="C2973" s="3" t="s">
         <v>4</v>

</xml_diff>

<commit_message>
--IMPLEMENTACION DE LOGICA PARA PROCESAR FACTURAS DE LA EMPRESA EDESAL
</commit_message>
<xml_diff>
--- a/Control de Facturas/Assets/Plantillas/BENEFICIARIOS AGUA, GAS Y LUZ.xlsx
+++ b/Control de Facturas/Assets/Plantillas/BENEFICIARIOS AGUA, GAS Y LUZ.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Programa Servicios Basicos\Control de Facturas\Assets\Plantillas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB55AD5F-80B6-4EAF-A9DF-EE2AB27E39AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1CEEFB0-5C39-4BF9-A456-EFFB817FC441}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{82731452-31CB-4A50-BC16-E3FD7323D481}"/>
   </bookViews>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11896" uniqueCount="5948">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11896" uniqueCount="5949">
   <si>
     <t>Número</t>
   </si>
@@ -17873,6 +17873,9 @@
   </si>
   <si>
     <t>EPEC</t>
+  </si>
+  <si>
+    <t>EDESAL</t>
   </si>
 </sst>
 </file>
@@ -25850,8 +25853,8 @@
       <c r="A446" s="2">
         <v>127673</v>
       </c>
-      <c r="B446" s="3" t="s">
-        <v>2999</v>
+      <c r="B446" s="5" t="s">
+        <v>5948</v>
       </c>
       <c r="C446" s="3" t="s">
         <v>3</v>

</xml_diff>

<commit_message>
--IMPLEMENTACION DE LOGICA DE NEGOCIO PARA LA EMPRESA EDEN DE ELECTRICIDAD
</commit_message>
<xml_diff>
--- a/Control de Facturas/Assets/Plantillas/BENEFICIARIOS AGUA, GAS Y LUZ.xlsx
+++ b/Control de Facturas/Assets/Plantillas/BENEFICIARIOS AGUA, GAS Y LUZ.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Programa Servicios Basicos\Control de Facturas\Assets\Plantillas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{312ADE00-7C8A-4A8B-83B5-FD2E4C427868}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30E6A506-91EE-40AF-B750-2B7DBD440AB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{82731452-31CB-4A50-BC16-E3FD7323D481}"/>
   </bookViews>
@@ -16264,9 +16264,6 @@
     <t>NORBERTOL.GARCIA</t>
   </si>
   <si>
-    <t>EMPRESADIST.DEENERGIANORTES.A.(E.D.E.N.S.A.)</t>
-  </si>
-  <si>
     <t>COOP.DEELECTRICIDADYSERV.ANEXOSDEALTAMIRANOLTDA.</t>
   </si>
   <si>
@@ -17876,6 +17873,9 @@
   </si>
   <si>
     <t>AGUAS DE CATAMARCA</t>
+  </si>
+  <si>
+    <t>EDEN</t>
   </si>
 </sst>
 </file>
@@ -18408,7 +18408,7 @@
         <v>1202</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>5665</v>
+        <v>5664</v>
       </c>
       <c r="C8" s="3" t="s">
         <v>3</v>
@@ -18459,7 +18459,7 @@
         <v>1325</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>5666</v>
+        <v>5665</v>
       </c>
       <c r="C11" s="3" t="s">
         <v>3</v>
@@ -18476,7 +18476,7 @@
         <v>1357</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>5943</v>
+        <v>5942</v>
       </c>
       <c r="C12" s="3" t="s">
         <v>3</v>
@@ -18629,7 +18629,7 @@
         <v>2603</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>5667</v>
+        <v>5666</v>
       </c>
       <c r="C21" s="3" t="s">
         <v>3</v>
@@ -18680,7 +18680,7 @@
         <v>3814</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>5668</v>
+        <v>5667</v>
       </c>
       <c r="C24" s="3" t="s">
         <v>3</v>
@@ -18731,7 +18731,7 @@
         <v>3937</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>5669</v>
+        <v>5668</v>
       </c>
       <c r="C27" s="3" t="s">
         <v>3</v>
@@ -18901,7 +18901,7 @@
         <v>4876</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>5670</v>
+        <v>5669</v>
       </c>
       <c r="C37" s="3" t="s">
         <v>3</v>
@@ -19105,7 +19105,7 @@
         <v>5331</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>5671</v>
+        <v>5670</v>
       </c>
       <c r="C49" s="3" t="s">
         <v>3</v>
@@ -19275,7 +19275,7 @@
         <v>6255</v>
       </c>
       <c r="B59" s="3" t="s">
-        <v>5672</v>
+        <v>5671</v>
       </c>
       <c r="C59" s="3" t="s">
         <v>3</v>
@@ -19292,7 +19292,7 @@
         <v>6298</v>
       </c>
       <c r="B60" s="3" t="s">
-        <v>5673</v>
+        <v>5672</v>
       </c>
       <c r="C60" s="3" t="s">
         <v>3</v>
@@ -19309,7 +19309,7 @@
         <v>7007</v>
       </c>
       <c r="B61" s="3" t="s">
-        <v>5674</v>
+        <v>5673</v>
       </c>
       <c r="C61" s="3" t="s">
         <v>3</v>
@@ -19581,7 +19581,7 @@
         <v>7561</v>
       </c>
       <c r="B77" s="3" t="s">
-        <v>5675</v>
+        <v>5674</v>
       </c>
       <c r="C77" s="3" t="s">
         <v>3</v>
@@ -19615,7 +19615,7 @@
         <v>7571</v>
       </c>
       <c r="B79" s="3" t="s">
-        <v>5676</v>
+        <v>5675</v>
       </c>
       <c r="C79" s="3" t="s">
         <v>3</v>
@@ -19632,7 +19632,7 @@
         <v>7572</v>
       </c>
       <c r="B80" s="3" t="s">
-        <v>5677</v>
+        <v>5676</v>
       </c>
       <c r="C80" s="3" t="s">
         <v>3</v>
@@ -19666,7 +19666,7 @@
         <v>7578</v>
       </c>
       <c r="B82" s="3" t="s">
-        <v>5678</v>
+        <v>5677</v>
       </c>
       <c r="C82" s="3" t="s">
         <v>3</v>
@@ -19683,7 +19683,7 @@
         <v>7605</v>
       </c>
       <c r="B83" s="3" t="s">
-        <v>5679</v>
+        <v>5678</v>
       </c>
       <c r="C83" s="3" t="s">
         <v>3</v>
@@ -19904,7 +19904,7 @@
         <v>8469</v>
       </c>
       <c r="B96" s="3" t="s">
-        <v>5680</v>
+        <v>5679</v>
       </c>
       <c r="C96" s="3" t="s">
         <v>3</v>
@@ -19921,7 +19921,7 @@
         <v>8567</v>
       </c>
       <c r="B97" s="3" t="s">
-        <v>5681</v>
+        <v>5680</v>
       </c>
       <c r="C97" s="3" t="s">
         <v>3</v>
@@ -20125,7 +20125,7 @@
         <v>9028</v>
       </c>
       <c r="B109" s="3" t="s">
-        <v>5682</v>
+        <v>5681</v>
       </c>
       <c r="C109" s="3" t="s">
         <v>3</v>
@@ -20176,7 +20176,7 @@
         <v>9733</v>
       </c>
       <c r="B112" s="3" t="s">
-        <v>5683</v>
+        <v>5682</v>
       </c>
       <c r="C112" s="3" t="s">
         <v>3</v>
@@ -20244,7 +20244,7 @@
         <v>9969</v>
       </c>
       <c r="B116" s="3" t="s">
-        <v>5684</v>
+        <v>5683</v>
       </c>
       <c r="C116" s="3" t="s">
         <v>3</v>
@@ -20346,7 +20346,7 @@
         <v>10627</v>
       </c>
       <c r="B122" s="3" t="s">
-        <v>5685</v>
+        <v>5684</v>
       </c>
       <c r="C122" s="3" t="s">
         <v>3</v>
@@ -20363,7 +20363,7 @@
         <v>10646</v>
       </c>
       <c r="B123" s="3" t="s">
-        <v>5686</v>
+        <v>5685</v>
       </c>
       <c r="C123" s="3" t="s">
         <v>3</v>
@@ -20533,7 +20533,7 @@
         <v>10888</v>
       </c>
       <c r="B133" s="3" t="s">
-        <v>5687</v>
+        <v>5686</v>
       </c>
       <c r="C133" s="3" t="s">
         <v>3</v>
@@ -20601,7 +20601,7 @@
         <v>10943</v>
       </c>
       <c r="B137" s="3" t="s">
-        <v>5688</v>
+        <v>5687</v>
       </c>
       <c r="C137" s="3" t="s">
         <v>3</v>
@@ -20686,7 +20686,7 @@
         <v>11003</v>
       </c>
       <c r="B142" s="3" t="s">
-        <v>5689</v>
+        <v>5688</v>
       </c>
       <c r="C142" s="3" t="s">
         <v>3</v>
@@ -20941,7 +20941,7 @@
         <v>12357</v>
       </c>
       <c r="B157" s="3" t="s">
-        <v>5690</v>
+        <v>5689</v>
       </c>
       <c r="C157" s="3" t="s">
         <v>3</v>
@@ -21026,7 +21026,7 @@
         <v>12580</v>
       </c>
       <c r="B162" s="3" t="s">
-        <v>5691</v>
+        <v>5690</v>
       </c>
       <c r="C162" s="3" t="s">
         <v>3</v>
@@ -21196,7 +21196,7 @@
         <v>12863</v>
       </c>
       <c r="B172" s="3" t="s">
-        <v>5692</v>
+        <v>5691</v>
       </c>
       <c r="C172" s="3" t="s">
         <v>3</v>
@@ -21213,7 +21213,7 @@
         <v>12864</v>
       </c>
       <c r="B173" s="3" t="s">
-        <v>5693</v>
+        <v>5692</v>
       </c>
       <c r="C173" s="3" t="s">
         <v>3</v>
@@ -21366,7 +21366,7 @@
         <v>14181</v>
       </c>
       <c r="B182" s="3" t="s">
-        <v>5694</v>
+        <v>5693</v>
       </c>
       <c r="C182" s="3" t="s">
         <v>3</v>
@@ -21434,7 +21434,7 @@
         <v>14626</v>
       </c>
       <c r="B186" s="5" t="s">
-        <v>5947</v>
+        <v>5946</v>
       </c>
       <c r="C186" s="3" t="s">
         <v>3</v>
@@ -21570,7 +21570,7 @@
         <v>17805</v>
       </c>
       <c r="B194" s="3" t="s">
-        <v>5695</v>
+        <v>5694</v>
       </c>
       <c r="C194" s="3" t="s">
         <v>3</v>
@@ -21672,7 +21672,7 @@
         <v>20477</v>
       </c>
       <c r="B200" s="3" t="s">
-        <v>5696</v>
+        <v>5695</v>
       </c>
       <c r="C200" s="3" t="s">
         <v>3</v>
@@ -21910,7 +21910,7 @@
         <v>26156</v>
       </c>
       <c r="B214" s="3" t="s">
-        <v>5697</v>
+        <v>5696</v>
       </c>
       <c r="C214" s="3" t="s">
         <v>3</v>
@@ -22165,7 +22165,7 @@
         <v>33533</v>
       </c>
       <c r="B229" s="3" t="s">
-        <v>5698</v>
+        <v>5697</v>
       </c>
       <c r="C229" s="3" t="s">
         <v>3</v>
@@ -22318,7 +22318,7 @@
         <v>35750</v>
       </c>
       <c r="B238" s="3" t="s">
-        <v>5699</v>
+        <v>5698</v>
       </c>
       <c r="C238" s="3" t="s">
         <v>3</v>
@@ -22862,7 +22862,7 @@
         <v>46145</v>
       </c>
       <c r="B270" s="3" t="s">
-        <v>5700</v>
+        <v>5699</v>
       </c>
       <c r="C270" s="3" t="s">
         <v>3</v>
@@ -22913,7 +22913,7 @@
         <v>48338</v>
       </c>
       <c r="B273" s="3" t="s">
-        <v>5701</v>
+        <v>5700</v>
       </c>
       <c r="C273" s="3" t="s">
         <v>3</v>
@@ -22964,7 +22964,7 @@
         <v>48805</v>
       </c>
       <c r="B276" s="3" t="s">
-        <v>5702</v>
+        <v>5701</v>
       </c>
       <c r="C276" s="3" t="s">
         <v>3</v>
@@ -23083,7 +23083,7 @@
         <v>49829</v>
       </c>
       <c r="B283" s="3" t="s">
-        <v>5703</v>
+        <v>5702</v>
       </c>
       <c r="C283" s="3" t="s">
         <v>3</v>
@@ -23236,7 +23236,7 @@
         <v>57520</v>
       </c>
       <c r="B292" s="3" t="s">
-        <v>5704</v>
+        <v>5703</v>
       </c>
       <c r="C292" s="3" t="s">
         <v>3</v>
@@ -23355,7 +23355,7 @@
         <v>58737</v>
       </c>
       <c r="B299" s="3" t="s">
-        <v>5705</v>
+        <v>5704</v>
       </c>
       <c r="C299" s="3" t="s">
         <v>3</v>
@@ -23524,8 +23524,8 @@
       <c r="A309" s="2">
         <v>67354</v>
       </c>
-      <c r="B309" s="3" t="s">
-        <v>5411</v>
+      <c r="B309" s="5" t="s">
+        <v>5948</v>
       </c>
       <c r="C309" s="3" t="s">
         <v>3</v>
@@ -23542,7 +23542,7 @@
         <v>67776</v>
       </c>
       <c r="B310" s="5" t="s">
-        <v>5945</v>
+        <v>5944</v>
       </c>
       <c r="C310" s="3" t="s">
         <v>3</v>
@@ -23576,7 +23576,7 @@
         <v>68602</v>
       </c>
       <c r="B312" s="3" t="s">
-        <v>5706</v>
+        <v>5705</v>
       </c>
       <c r="C312" s="3" t="s">
         <v>3</v>
@@ -23695,7 +23695,7 @@
         <v>75448</v>
       </c>
       <c r="B319" s="3" t="s">
-        <v>5412</v>
+        <v>5411</v>
       </c>
       <c r="C319" s="3" t="s">
         <v>3</v>
@@ -24035,7 +24035,7 @@
         <v>82472</v>
       </c>
       <c r="B339" s="3" t="s">
-        <v>5707</v>
+        <v>5706</v>
       </c>
       <c r="C339" s="3" t="s">
         <v>3</v>
@@ -24069,7 +24069,7 @@
         <v>82772</v>
       </c>
       <c r="B341" s="3" t="s">
-        <v>5708</v>
+        <v>5707</v>
       </c>
       <c r="C341" s="3" t="s">
         <v>3</v>
@@ -24154,7 +24154,7 @@
         <v>85154</v>
       </c>
       <c r="B346" s="3" t="s">
-        <v>5413</v>
+        <v>5412</v>
       </c>
       <c r="C346" s="3" t="s">
         <v>3</v>
@@ -24324,7 +24324,7 @@
         <v>89047</v>
       </c>
       <c r="B356" s="3" t="s">
-        <v>5414</v>
+        <v>5413</v>
       </c>
       <c r="C356" s="3" t="s">
         <v>3</v>
@@ -24426,7 +24426,7 @@
         <v>92681</v>
       </c>
       <c r="B362" s="3" t="s">
-        <v>5709</v>
+        <v>5708</v>
       </c>
       <c r="C362" s="3" t="s">
         <v>3</v>
@@ -24613,7 +24613,7 @@
         <v>99451</v>
       </c>
       <c r="B373" s="3" t="s">
-        <v>5710</v>
+        <v>5709</v>
       </c>
       <c r="C373" s="3" t="s">
         <v>3</v>
@@ -24630,7 +24630,7 @@
         <v>99598</v>
       </c>
       <c r="B374" s="3" t="s">
-        <v>5711</v>
+        <v>5710</v>
       </c>
       <c r="C374" s="3" t="s">
         <v>3</v>
@@ -25038,7 +25038,7 @@
         <v>110674</v>
       </c>
       <c r="B398" s="3" t="s">
-        <v>5712</v>
+        <v>5711</v>
       </c>
       <c r="C398" s="3" t="s">
         <v>3</v>
@@ -25055,7 +25055,7 @@
         <v>111078</v>
       </c>
       <c r="B399" s="3" t="s">
-        <v>5713</v>
+        <v>5712</v>
       </c>
       <c r="C399" s="3" t="s">
         <v>3</v>
@@ -25106,7 +25106,7 @@
         <v>111715</v>
       </c>
       <c r="B402" s="3" t="s">
-        <v>5714</v>
+        <v>5713</v>
       </c>
       <c r="C402" s="3" t="s">
         <v>3</v>
@@ -25276,7 +25276,7 @@
         <v>116470</v>
       </c>
       <c r="B412" s="3" t="s">
-        <v>5415</v>
+        <v>5414</v>
       </c>
       <c r="C412" s="3" t="s">
         <v>3</v>
@@ -25327,7 +25327,7 @@
         <v>118049</v>
       </c>
       <c r="B415" s="3" t="s">
-        <v>5416</v>
+        <v>5415</v>
       </c>
       <c r="C415" s="3" t="s">
         <v>3</v>
@@ -25344,7 +25344,7 @@
         <v>118398</v>
       </c>
       <c r="B416" s="3" t="s">
-        <v>5417</v>
+        <v>5416</v>
       </c>
       <c r="C416" s="3" t="s">
         <v>3</v>
@@ -25463,7 +25463,7 @@
         <v>122357</v>
       </c>
       <c r="B423" s="3" t="s">
-        <v>5715</v>
+        <v>5714</v>
       </c>
       <c r="C423" s="3" t="s">
         <v>3</v>
@@ -25497,7 +25497,7 @@
         <v>122551</v>
       </c>
       <c r="B425" s="3" t="s">
-        <v>5418</v>
+        <v>5417</v>
       </c>
       <c r="C425" s="3" t="s">
         <v>3</v>
@@ -25565,7 +25565,7 @@
         <v>122860</v>
       </c>
       <c r="B429" s="3" t="s">
-        <v>5419</v>
+        <v>5418</v>
       </c>
       <c r="C429" s="3" t="s">
         <v>3</v>
@@ -25667,7 +25667,7 @@
         <v>124361</v>
       </c>
       <c r="B435" s="3" t="s">
-        <v>5716</v>
+        <v>5715</v>
       </c>
       <c r="C435" s="3" t="s">
         <v>3</v>
@@ -25701,7 +25701,7 @@
         <v>124976</v>
       </c>
       <c r="B437" s="3" t="s">
-        <v>5420</v>
+        <v>5419</v>
       </c>
       <c r="C437" s="3" t="s">
         <v>3</v>
@@ -25786,7 +25786,7 @@
         <v>125649</v>
       </c>
       <c r="B442" s="3" t="s">
-        <v>5717</v>
+        <v>5716</v>
       </c>
       <c r="C442" s="3" t="s">
         <v>3</v>
@@ -25803,7 +25803,7 @@
         <v>125851</v>
       </c>
       <c r="B443" s="3" t="s">
-        <v>5718</v>
+        <v>5717</v>
       </c>
       <c r="C443" s="3" t="s">
         <v>3</v>
@@ -25854,7 +25854,7 @@
         <v>127673</v>
       </c>
       <c r="B446" s="5" t="s">
-        <v>5944</v>
+        <v>5943</v>
       </c>
       <c r="C446" s="3" t="s">
         <v>3</v>
@@ -25956,7 +25956,7 @@
         <v>129590</v>
       </c>
       <c r="B452" s="3" t="s">
-        <v>5421</v>
+        <v>5420</v>
       </c>
       <c r="C452" s="3" t="s">
         <v>3</v>
@@ -26041,7 +26041,7 @@
         <v>132364</v>
       </c>
       <c r="B457" s="3" t="s">
-        <v>5719</v>
+        <v>5718</v>
       </c>
       <c r="C457" s="3" t="s">
         <v>3</v>
@@ -26245,7 +26245,7 @@
         <v>142996</v>
       </c>
       <c r="B469" s="3" t="s">
-        <v>5422</v>
+        <v>5421</v>
       </c>
       <c r="C469" s="3" t="s">
         <v>3</v>
@@ -26449,7 +26449,7 @@
         <v>153315</v>
       </c>
       <c r="B481" s="3" t="s">
-        <v>5423</v>
+        <v>5422</v>
       </c>
       <c r="C481" s="3" t="s">
         <v>3</v>
@@ -26483,7 +26483,7 @@
         <v>155870</v>
       </c>
       <c r="B483" s="3" t="s">
-        <v>5424</v>
+        <v>5423</v>
       </c>
       <c r="C483" s="3" t="s">
         <v>3</v>
@@ -26534,7 +26534,7 @@
         <v>158689</v>
       </c>
       <c r="B486" s="3" t="s">
-        <v>5720</v>
+        <v>5719</v>
       </c>
       <c r="C486" s="3" t="s">
         <v>3</v>
@@ -26687,7 +26687,7 @@
         <v>168013</v>
       </c>
       <c r="B495" s="3" t="s">
-        <v>5425</v>
+        <v>5424</v>
       </c>
       <c r="C495" s="3" t="s">
         <v>3</v>
@@ -26755,7 +26755,7 @@
         <v>171813</v>
       </c>
       <c r="B499" s="3" t="s">
-        <v>5721</v>
+        <v>5720</v>
       </c>
       <c r="C499" s="3" t="s">
         <v>3</v>
@@ -26959,7 +26959,7 @@
         <v>178027</v>
       </c>
       <c r="B511" s="3" t="s">
-        <v>5722</v>
+        <v>5721</v>
       </c>
       <c r="C511" s="3" t="s">
         <v>3</v>
@@ -27129,7 +27129,7 @@
         <v>189468</v>
       </c>
       <c r="B521" s="3" t="s">
-        <v>5723</v>
+        <v>5722</v>
       </c>
       <c r="C521" s="3" t="s">
         <v>3</v>
@@ -27333,7 +27333,7 @@
         <v>190418</v>
       </c>
       <c r="B533" s="3" t="s">
-        <v>5426</v>
+        <v>5425</v>
       </c>
       <c r="C533" s="3" t="s">
         <v>3</v>
@@ -27435,7 +27435,7 @@
         <v>190454</v>
       </c>
       <c r="B539" s="3" t="s">
-        <v>5427</v>
+        <v>5426</v>
       </c>
       <c r="C539" s="3" t="s">
         <v>3</v>
@@ -27622,7 +27622,7 @@
         <v>190514</v>
       </c>
       <c r="B550" s="3" t="s">
-        <v>5428</v>
+        <v>5427</v>
       </c>
       <c r="C550" s="3" t="s">
         <v>3</v>
@@ -27707,7 +27707,7 @@
         <v>190558</v>
       </c>
       <c r="B555" s="3" t="s">
-        <v>5724</v>
+        <v>5723</v>
       </c>
       <c r="C555" s="3" t="s">
         <v>3</v>
@@ -27775,7 +27775,7 @@
         <v>191311</v>
       </c>
       <c r="B559" s="3" t="s">
-        <v>5725</v>
+        <v>5724</v>
       </c>
       <c r="C559" s="3" t="s">
         <v>3</v>
@@ -27826,7 +27826,7 @@
         <v>191951</v>
       </c>
       <c r="B562" s="3" t="s">
-        <v>5726</v>
+        <v>5725</v>
       </c>
       <c r="C562" s="3" t="s">
         <v>3</v>
@@ -27843,7 +27843,7 @@
         <v>192881</v>
       </c>
       <c r="B563" s="3" t="s">
-        <v>5727</v>
+        <v>5726</v>
       </c>
       <c r="C563" s="3" t="s">
         <v>3</v>
@@ -27860,7 +27860,7 @@
         <v>193054</v>
       </c>
       <c r="B564" s="3" t="s">
-        <v>5728</v>
+        <v>5727</v>
       </c>
       <c r="C564" s="3" t="s">
         <v>3</v>
@@ -28013,7 +28013,7 @@
         <v>197127</v>
       </c>
       <c r="B573" s="3" t="s">
-        <v>5729</v>
+        <v>5728</v>
       </c>
       <c r="C573" s="3" t="s">
         <v>3</v>
@@ -28166,7 +28166,7 @@
         <v>202738</v>
       </c>
       <c r="B582" s="3" t="s">
-        <v>5730</v>
+        <v>5729</v>
       </c>
       <c r="C582" s="3" t="s">
         <v>3</v>
@@ -28251,7 +28251,7 @@
         <v>204941</v>
       </c>
       <c r="B587" s="3" t="s">
-        <v>5731</v>
+        <v>5730</v>
       </c>
       <c r="C587" s="3" t="s">
         <v>3</v>
@@ -28404,7 +28404,7 @@
         <v>219118</v>
       </c>
       <c r="B596" s="3" t="s">
-        <v>5732</v>
+        <v>5731</v>
       </c>
       <c r="C596" s="3" t="s">
         <v>3</v>
@@ -28591,7 +28591,7 @@
         <v>224861</v>
       </c>
       <c r="B607" s="3" t="s">
-        <v>5429</v>
+        <v>5428</v>
       </c>
       <c r="C607" s="3" t="s">
         <v>3</v>
@@ -28608,7 +28608,7 @@
         <v>225470</v>
       </c>
       <c r="B608" s="3" t="s">
-        <v>5430</v>
+        <v>5429</v>
       </c>
       <c r="C608" s="3" t="s">
         <v>3</v>
@@ -28625,7 +28625,7 @@
         <v>226297</v>
       </c>
       <c r="B609" s="3" t="s">
-        <v>5733</v>
+        <v>5732</v>
       </c>
       <c r="C609" s="3" t="s">
         <v>3</v>
@@ -28642,7 +28642,7 @@
         <v>226401</v>
       </c>
       <c r="B610" s="3" t="s">
-        <v>5734</v>
+        <v>5733</v>
       </c>
       <c r="C610" s="3" t="s">
         <v>3</v>
@@ -28744,7 +28744,7 @@
         <v>230376</v>
       </c>
       <c r="B616" s="3" t="s">
-        <v>5735</v>
+        <v>5734</v>
       </c>
       <c r="C616" s="3" t="s">
         <v>3</v>
@@ -28778,7 +28778,7 @@
         <v>232246</v>
       </c>
       <c r="B618" s="3" t="s">
-        <v>5736</v>
+        <v>5735</v>
       </c>
       <c r="C618" s="3" t="s">
         <v>3</v>
@@ -28795,7 +28795,7 @@
         <v>232630</v>
       </c>
       <c r="B619" s="3" t="s">
-        <v>5431</v>
+        <v>5430</v>
       </c>
       <c r="C619" s="3" t="s">
         <v>3</v>
@@ -28897,7 +28897,7 @@
         <v>235510</v>
       </c>
       <c r="B625" s="3" t="s">
-        <v>5737</v>
+        <v>5736</v>
       </c>
       <c r="C625" s="3" t="s">
         <v>3</v>
@@ -28914,7 +28914,7 @@
         <v>235512</v>
       </c>
       <c r="B626" s="3" t="s">
-        <v>5738</v>
+        <v>5737</v>
       </c>
       <c r="C626" s="3" t="s">
         <v>3</v>
@@ -28931,7 +28931,7 @@
         <v>235513</v>
       </c>
       <c r="B627" s="3" t="s">
-        <v>5739</v>
+        <v>5738</v>
       </c>
       <c r="C627" s="3" t="s">
         <v>3</v>
@@ -28982,7 +28982,7 @@
         <v>235622</v>
       </c>
       <c r="B630" s="3" t="s">
-        <v>5740</v>
+        <v>5739</v>
       </c>
       <c r="C630" s="3" t="s">
         <v>3</v>
@@ -29016,7 +29016,7 @@
         <v>236048</v>
       </c>
       <c r="B632" s="3" t="s">
-        <v>5741</v>
+        <v>5740</v>
       </c>
       <c r="C632" s="3" t="s">
         <v>3</v>
@@ -29033,7 +29033,7 @@
         <v>236636</v>
       </c>
       <c r="B633" s="3" t="s">
-        <v>5742</v>
+        <v>5741</v>
       </c>
       <c r="C633" s="3" t="s">
         <v>3</v>
@@ -29152,7 +29152,7 @@
         <v>239815</v>
       </c>
       <c r="B640" s="3" t="s">
-        <v>5432</v>
+        <v>5431</v>
       </c>
       <c r="C640" s="3" t="s">
         <v>3</v>
@@ -29237,7 +29237,7 @@
         <v>240433</v>
       </c>
       <c r="B645" s="3" t="s">
-        <v>5433</v>
+        <v>5432</v>
       </c>
       <c r="C645" s="3" t="s">
         <v>3</v>
@@ -29254,7 +29254,7 @@
         <v>240657</v>
       </c>
       <c r="B646" s="3" t="s">
-        <v>5743</v>
+        <v>5742</v>
       </c>
       <c r="C646" s="3" t="s">
         <v>3</v>
@@ -29322,7 +29322,7 @@
         <v>241576</v>
       </c>
       <c r="B650" s="3" t="s">
-        <v>5744</v>
+        <v>5743</v>
       </c>
       <c r="C650" s="3" t="s">
         <v>3</v>
@@ -29339,7 +29339,7 @@
         <v>241577</v>
       </c>
       <c r="B651" s="3" t="s">
-        <v>5745</v>
+        <v>5744</v>
       </c>
       <c r="C651" s="3" t="s">
         <v>3</v>
@@ -29458,7 +29458,7 @@
         <v>243126</v>
       </c>
       <c r="B658" s="3" t="s">
-        <v>5746</v>
+        <v>5745</v>
       </c>
       <c r="C658" s="3" t="s">
         <v>3</v>
@@ -29543,7 +29543,7 @@
         <v>245475</v>
       </c>
       <c r="B663" s="3" t="s">
-        <v>5434</v>
+        <v>5433</v>
       </c>
       <c r="C663" s="3" t="s">
         <v>3</v>
@@ -29577,7 +29577,7 @@
         <v>245569</v>
       </c>
       <c r="B665" s="3" t="s">
-        <v>5435</v>
+        <v>5434</v>
       </c>
       <c r="C665" s="3" t="s">
         <v>3</v>
@@ -29594,7 +29594,7 @@
         <v>245792</v>
       </c>
       <c r="B666" s="3" t="s">
-        <v>5747</v>
+        <v>5746</v>
       </c>
       <c r="C666" s="3" t="s">
         <v>3</v>
@@ -29628,7 +29628,7 @@
         <v>246010</v>
       </c>
       <c r="B668" s="3" t="s">
-        <v>5748</v>
+        <v>5747</v>
       </c>
       <c r="C668" s="3" t="s">
         <v>3</v>
@@ -29696,7 +29696,7 @@
         <v>250244</v>
       </c>
       <c r="B672" s="3" t="s">
-        <v>5436</v>
+        <v>5435</v>
       </c>
       <c r="C672" s="3" t="s">
         <v>3</v>
@@ -29832,7 +29832,7 @@
         <v>253700</v>
       </c>
       <c r="B680" s="3" t="s">
-        <v>5437</v>
+        <v>5436</v>
       </c>
       <c r="C680" s="3" t="s">
         <v>3</v>
@@ -29883,7 +29883,7 @@
         <v>255046</v>
       </c>
       <c r="B683" s="3" t="s">
-        <v>5749</v>
+        <v>5748</v>
       </c>
       <c r="C683" s="3" t="s">
         <v>3</v>
@@ -29951,7 +29951,7 @@
         <v>256609</v>
       </c>
       <c r="B687" s="3" t="s">
-        <v>5750</v>
+        <v>5749</v>
       </c>
       <c r="C687" s="3" t="s">
         <v>3</v>
@@ -30053,7 +30053,7 @@
         <v>260696</v>
       </c>
       <c r="B693" s="3" t="s">
-        <v>5751</v>
+        <v>5750</v>
       </c>
       <c r="C693" s="3" t="s">
         <v>3</v>
@@ -30138,7 +30138,7 @@
         <v>262595</v>
       </c>
       <c r="B698" s="3" t="s">
-        <v>5752</v>
+        <v>5751</v>
       </c>
       <c r="C698" s="3" t="s">
         <v>3</v>
@@ -30189,7 +30189,7 @@
         <v>262648</v>
       </c>
       <c r="B701" s="3" t="s">
-        <v>5753</v>
+        <v>5752</v>
       </c>
       <c r="C701" s="3" t="s">
         <v>3</v>
@@ -30240,7 +30240,7 @@
         <v>266798</v>
       </c>
       <c r="B704" s="3" t="s">
-        <v>5438</v>
+        <v>5437</v>
       </c>
       <c r="C704" s="3" t="s">
         <v>3</v>
@@ -30308,7 +30308,7 @@
         <v>269554</v>
       </c>
       <c r="B708" s="3" t="s">
-        <v>5754</v>
+        <v>5753</v>
       </c>
       <c r="C708" s="3" t="s">
         <v>3</v>
@@ -30495,7 +30495,7 @@
         <v>276933</v>
       </c>
       <c r="B719" s="3" t="s">
-        <v>5755</v>
+        <v>5754</v>
       </c>
       <c r="C719" s="3" t="s">
         <v>3</v>
@@ -30563,7 +30563,7 @@
         <v>278058</v>
       </c>
       <c r="B723" s="3" t="s">
-        <v>5756</v>
+        <v>5755</v>
       </c>
       <c r="C723" s="3" t="s">
         <v>3</v>
@@ -30631,7 +30631,7 @@
         <v>281556</v>
       </c>
       <c r="B727" s="3" t="s">
-        <v>5757</v>
+        <v>5756</v>
       </c>
       <c r="C727" s="3" t="s">
         <v>3</v>
@@ -30716,7 +30716,7 @@
         <v>285507</v>
       </c>
       <c r="B732" s="3" t="s">
-        <v>5758</v>
+        <v>5757</v>
       </c>
       <c r="C732" s="3" t="s">
         <v>3</v>
@@ -30767,7 +30767,7 @@
         <v>287431</v>
       </c>
       <c r="B735" s="3" t="s">
-        <v>5439</v>
+        <v>5438</v>
       </c>
       <c r="C735" s="3" t="s">
         <v>3</v>
@@ -30801,7 +30801,7 @@
         <v>287851</v>
       </c>
       <c r="B737" s="3" t="s">
-        <v>5759</v>
+        <v>5758</v>
       </c>
       <c r="C737" s="3" t="s">
         <v>3</v>
@@ -30937,7 +30937,7 @@
         <v>291978</v>
       </c>
       <c r="B745" s="3" t="s">
-        <v>5760</v>
+        <v>5759</v>
       </c>
       <c r="C745" s="3" t="s">
         <v>3</v>
@@ -30971,7 +30971,7 @@
         <v>295086</v>
       </c>
       <c r="B747" s="3" t="s">
-        <v>5761</v>
+        <v>5760</v>
       </c>
       <c r="C747" s="3" t="s">
         <v>3</v>
@@ -30988,7 +30988,7 @@
         <v>297792</v>
       </c>
       <c r="B748" s="3" t="s">
-        <v>5762</v>
+        <v>5761</v>
       </c>
       <c r="C748" s="3" t="s">
         <v>3</v>
@@ -31005,7 +31005,7 @@
         <v>298556</v>
       </c>
       <c r="B749" s="3" t="s">
-        <v>5763</v>
+        <v>5762</v>
       </c>
       <c r="C749" s="3" t="s">
         <v>3</v>
@@ -31056,7 +31056,7 @@
         <v>299682</v>
       </c>
       <c r="B752" s="3" t="s">
-        <v>5440</v>
+        <v>5439</v>
       </c>
       <c r="C752" s="3" t="s">
         <v>3</v>
@@ -31073,7 +31073,7 @@
         <v>300800</v>
       </c>
       <c r="B753" s="3" t="s">
-        <v>5764</v>
+        <v>5763</v>
       </c>
       <c r="C753" s="3" t="s">
         <v>3</v>
@@ -31090,7 +31090,7 @@
         <v>301705</v>
       </c>
       <c r="B754" s="3" t="s">
-        <v>5765</v>
+        <v>5764</v>
       </c>
       <c r="C754" s="3" t="s">
         <v>3</v>
@@ -31124,7 +31124,7 @@
         <v>307867</v>
       </c>
       <c r="B756" s="3" t="s">
-        <v>5766</v>
+        <v>5765</v>
       </c>
       <c r="C756" s="3" t="s">
         <v>3</v>
@@ -31209,7 +31209,7 @@
         <v>316725</v>
       </c>
       <c r="B761" s="5" t="s">
-        <v>5948</v>
+        <v>5947</v>
       </c>
       <c r="C761" s="3" t="s">
         <v>3</v>
@@ -31379,7 +31379,7 @@
         <v>324503</v>
       </c>
       <c r="B771" s="3" t="s">
-        <v>5767</v>
+        <v>5766</v>
       </c>
       <c r="C771" s="3" t="s">
         <v>3</v>
@@ -31396,7 +31396,7 @@
         <v>324977</v>
       </c>
       <c r="B772" s="3" t="s">
-        <v>5768</v>
+        <v>5767</v>
       </c>
       <c r="C772" s="3" t="s">
         <v>3</v>
@@ -31481,7 +31481,7 @@
         <v>327658</v>
       </c>
       <c r="B777" s="3" t="s">
-        <v>5769</v>
+        <v>5768</v>
       </c>
       <c r="C777" s="3" t="s">
         <v>3</v>
@@ -31498,7 +31498,7 @@
         <v>328124</v>
       </c>
       <c r="B778" s="3" t="s">
-        <v>5770</v>
+        <v>5769</v>
       </c>
       <c r="C778" s="3" t="s">
         <v>3</v>
@@ -31532,7 +31532,7 @@
         <v>331486</v>
       </c>
       <c r="B780" s="3" t="s">
-        <v>5441</v>
+        <v>5440</v>
       </c>
       <c r="C780" s="3" t="s">
         <v>3</v>
@@ -31583,7 +31583,7 @@
         <v>332307</v>
       </c>
       <c r="B783" s="3" t="s">
-        <v>5442</v>
+        <v>5441</v>
       </c>
       <c r="C783" s="3" t="s">
         <v>3</v>
@@ -31651,7 +31651,7 @@
         <v>335317</v>
       </c>
       <c r="B787" s="3" t="s">
-        <v>5443</v>
+        <v>5442</v>
       </c>
       <c r="C787" s="3" t="s">
         <v>3</v>
@@ -31668,7 +31668,7 @@
         <v>335786</v>
       </c>
       <c r="B788" s="3" t="s">
-        <v>5444</v>
+        <v>5443</v>
       </c>
       <c r="C788" s="3" t="s">
         <v>3</v>
@@ -31736,7 +31736,7 @@
         <v>336865</v>
       </c>
       <c r="B792" s="3" t="s">
-        <v>5445</v>
+        <v>5444</v>
       </c>
       <c r="C792" s="3" t="s">
         <v>3</v>
@@ -31838,7 +31838,7 @@
         <v>343290</v>
       </c>
       <c r="B798" s="3" t="s">
-        <v>5771</v>
+        <v>5770</v>
       </c>
       <c r="C798" s="3" t="s">
         <v>3</v>
@@ -31923,7 +31923,7 @@
         <v>345453</v>
       </c>
       <c r="B803" s="3" t="s">
-        <v>5772</v>
+        <v>5771</v>
       </c>
       <c r="C803" s="3" t="s">
         <v>3</v>
@@ -31940,7 +31940,7 @@
         <v>346087</v>
       </c>
       <c r="B804" s="3" t="s">
-        <v>5446</v>
+        <v>5445</v>
       </c>
       <c r="C804" s="3" t="s">
         <v>3</v>
@@ -31957,7 +31957,7 @@
         <v>346199</v>
       </c>
       <c r="B805" s="3" t="s">
-        <v>5447</v>
+        <v>5446</v>
       </c>
       <c r="C805" s="3" t="s">
         <v>3</v>
@@ -32008,7 +32008,7 @@
         <v>347739</v>
       </c>
       <c r="B808" s="3" t="s">
-        <v>5773</v>
+        <v>5772</v>
       </c>
       <c r="C808" s="3" t="s">
         <v>3</v>
@@ -32042,7 +32042,7 @@
         <v>349673</v>
       </c>
       <c r="B810" s="3" t="s">
-        <v>5448</v>
+        <v>5447</v>
       </c>
       <c r="C810" s="3" t="s">
         <v>3</v>
@@ -32076,7 +32076,7 @@
         <v>350234</v>
       </c>
       <c r="B812" s="3" t="s">
-        <v>5774</v>
+        <v>5773</v>
       </c>
       <c r="C812" s="3" t="s">
         <v>3</v>
@@ -32144,7 +32144,7 @@
         <v>352365</v>
       </c>
       <c r="B816" s="3" t="s">
-        <v>5449</v>
+        <v>5448</v>
       </c>
       <c r="C816" s="3" t="s">
         <v>3</v>
@@ -32178,7 +32178,7 @@
         <v>354314</v>
       </c>
       <c r="B818" s="3" t="s">
-        <v>5450</v>
+        <v>5449</v>
       </c>
       <c r="C818" s="3" t="s">
         <v>3</v>
@@ -32246,7 +32246,7 @@
         <v>355329</v>
       </c>
       <c r="B822" s="3" t="s">
-        <v>5451</v>
+        <v>5450</v>
       </c>
       <c r="C822" s="3" t="s">
         <v>3</v>
@@ -32263,7 +32263,7 @@
         <v>357514</v>
       </c>
       <c r="B823" s="3" t="s">
-        <v>5452</v>
+        <v>5451</v>
       </c>
       <c r="C823" s="3" t="s">
         <v>3</v>
@@ -32348,7 +32348,7 @@
         <v>360931</v>
       </c>
       <c r="B828" s="3" t="s">
-        <v>5453</v>
+        <v>5452</v>
       </c>
       <c r="C828" s="3" t="s">
         <v>3</v>
@@ -32433,7 +32433,7 @@
         <v>365326</v>
       </c>
       <c r="B833" s="3" t="s">
-        <v>5454</v>
+        <v>5453</v>
       </c>
       <c r="C833" s="3" t="s">
         <v>3</v>
@@ -32450,7 +32450,7 @@
         <v>365501</v>
       </c>
       <c r="B834" s="3" t="s">
-        <v>5775</v>
+        <v>5774</v>
       </c>
       <c r="C834" s="3" t="s">
         <v>3</v>
@@ -32535,7 +32535,7 @@
         <v>368363</v>
       </c>
       <c r="B839" s="3" t="s">
-        <v>5455</v>
+        <v>5454</v>
       </c>
       <c r="C839" s="3" t="s">
         <v>3</v>
@@ -32569,7 +32569,7 @@
         <v>368986</v>
       </c>
       <c r="B841" s="3" t="s">
-        <v>5456</v>
+        <v>5455</v>
       </c>
       <c r="C841" s="3" t="s">
         <v>3</v>
@@ -32620,7 +32620,7 @@
         <v>370379</v>
       </c>
       <c r="B844" s="3" t="s">
-        <v>5457</v>
+        <v>5456</v>
       </c>
       <c r="C844" s="3" t="s">
         <v>3</v>
@@ -32637,7 +32637,7 @@
         <v>370761</v>
       </c>
       <c r="B845" s="3" t="s">
-        <v>5458</v>
+        <v>5457</v>
       </c>
       <c r="C845" s="3" t="s">
         <v>3</v>
@@ -32722,7 +32722,7 @@
         <v>372272</v>
       </c>
       <c r="B850" s="3" t="s">
-        <v>5776</v>
+        <v>5775</v>
       </c>
       <c r="C850" s="3" t="s">
         <v>3</v>
@@ -32739,7 +32739,7 @@
         <v>372443</v>
       </c>
       <c r="B851" s="3" t="s">
-        <v>5777</v>
+        <v>5776</v>
       </c>
       <c r="C851" s="3" t="s">
         <v>3</v>
@@ -32756,7 +32756,7 @@
         <v>372530</v>
       </c>
       <c r="B852" s="3" t="s">
-        <v>5459</v>
+        <v>5458</v>
       </c>
       <c r="C852" s="3" t="s">
         <v>3</v>
@@ -32841,7 +32841,7 @@
         <v>373863</v>
       </c>
       <c r="B857" s="3" t="s">
-        <v>5778</v>
+        <v>5777</v>
       </c>
       <c r="C857" s="3" t="s">
         <v>3</v>
@@ -32960,7 +32960,7 @@
         <v>376974</v>
       </c>
       <c r="B864" s="3" t="s">
-        <v>5460</v>
+        <v>5459</v>
       </c>
       <c r="C864" s="3" t="s">
         <v>3</v>
@@ -33079,7 +33079,7 @@
         <v>383882</v>
       </c>
       <c r="B871" s="3" t="s">
-        <v>5461</v>
+        <v>5460</v>
       </c>
       <c r="C871" s="3" t="s">
         <v>3</v>
@@ -33096,7 +33096,7 @@
         <v>384192</v>
       </c>
       <c r="B872" s="3" t="s">
-        <v>5779</v>
+        <v>5778</v>
       </c>
       <c r="C872" s="3" t="s">
         <v>3</v>
@@ -33300,7 +33300,7 @@
         <v>388346</v>
       </c>
       <c r="B884" s="3" t="s">
-        <v>5462</v>
+        <v>5461</v>
       </c>
       <c r="C884" s="3" t="s">
         <v>3</v>
@@ -33334,7 +33334,7 @@
         <v>389701</v>
       </c>
       <c r="B886" s="3" t="s">
-        <v>5780</v>
+        <v>5779</v>
       </c>
       <c r="C886" s="3" t="s">
         <v>3</v>
@@ -33368,7 +33368,7 @@
         <v>392098</v>
       </c>
       <c r="B888" s="3" t="s">
-        <v>5781</v>
+        <v>5780</v>
       </c>
       <c r="C888" s="3" t="s">
         <v>3</v>
@@ -33453,7 +33453,7 @@
         <v>394655</v>
       </c>
       <c r="B893" s="3" t="s">
-        <v>5782</v>
+        <v>5781</v>
       </c>
       <c r="C893" s="3" t="s">
         <v>3</v>
@@ -33470,7 +33470,7 @@
         <v>394709</v>
       </c>
       <c r="B894" s="3" t="s">
-        <v>5783</v>
+        <v>5782</v>
       </c>
       <c r="C894" s="3" t="s">
         <v>3</v>
@@ -33487,7 +33487,7 @@
         <v>394861</v>
       </c>
       <c r="B895" s="3" t="s">
-        <v>5784</v>
+        <v>5783</v>
       </c>
       <c r="C895" s="3" t="s">
         <v>3</v>
@@ -33521,7 +33521,7 @@
         <v>395525</v>
       </c>
       <c r="B897" s="3" t="s">
-        <v>5785</v>
+        <v>5784</v>
       </c>
       <c r="C897" s="3" t="s">
         <v>3</v>
@@ -33538,7 +33538,7 @@
         <v>395560</v>
       </c>
       <c r="B898" s="3" t="s">
-        <v>5463</v>
+        <v>5462</v>
       </c>
       <c r="C898" s="3" t="s">
         <v>3</v>
@@ -33589,7 +33589,7 @@
         <v>397509</v>
       </c>
       <c r="B901" s="3" t="s">
-        <v>5786</v>
+        <v>5785</v>
       </c>
       <c r="C901" s="3" t="s">
         <v>3</v>
@@ -33708,7 +33708,7 @@
         <v>401447</v>
       </c>
       <c r="B908" s="3" t="s">
-        <v>5464</v>
+        <v>5463</v>
       </c>
       <c r="C908" s="3" t="s">
         <v>3</v>
@@ -33827,7 +33827,7 @@
         <v>406298</v>
       </c>
       <c r="B915" s="3" t="s">
-        <v>5465</v>
+        <v>5464</v>
       </c>
       <c r="C915" s="3" t="s">
         <v>3</v>
@@ -33895,7 +33895,7 @@
         <v>409909</v>
       </c>
       <c r="B919" s="3" t="s">
-        <v>5787</v>
+        <v>5786</v>
       </c>
       <c r="C919" s="3" t="s">
         <v>3</v>
@@ -33997,7 +33997,7 @@
         <v>412340</v>
       </c>
       <c r="B925" s="3" t="s">
-        <v>5466</v>
+        <v>5465</v>
       </c>
       <c r="C925" s="3" t="s">
         <v>3</v>
@@ -34133,7 +34133,7 @@
         <v>413789</v>
       </c>
       <c r="B933" s="3" t="s">
-        <v>5788</v>
+        <v>5787</v>
       </c>
       <c r="C933" s="3" t="s">
         <v>3</v>
@@ -34150,7 +34150,7 @@
         <v>414649</v>
       </c>
       <c r="B934" s="3" t="s">
-        <v>5467</v>
+        <v>5466</v>
       </c>
       <c r="C934" s="3" t="s">
         <v>3</v>
@@ -34167,7 +34167,7 @@
         <v>415197</v>
       </c>
       <c r="B935" s="3" t="s">
-        <v>5789</v>
+        <v>5788</v>
       </c>
       <c r="C935" s="3" t="s">
         <v>3</v>
@@ -34456,7 +34456,7 @@
         <v>423286</v>
       </c>
       <c r="B952" s="3" t="s">
-        <v>5468</v>
+        <v>5467</v>
       </c>
       <c r="C952" s="3" t="s">
         <v>3</v>
@@ -34609,7 +34609,7 @@
         <v>429725</v>
       </c>
       <c r="B961" s="3" t="s">
-        <v>5790</v>
+        <v>5789</v>
       </c>
       <c r="C961" s="3" t="s">
         <v>3</v>
@@ -34643,7 +34643,7 @@
         <v>430464</v>
       </c>
       <c r="B963" s="3" t="s">
-        <v>5469</v>
+        <v>5468</v>
       </c>
       <c r="C963" s="3" t="s">
         <v>3</v>
@@ -34694,7 +34694,7 @@
         <v>431885</v>
       </c>
       <c r="B966" s="3" t="s">
-        <v>5791</v>
+        <v>5790</v>
       </c>
       <c r="C966" s="3" t="s">
         <v>3</v>
@@ -34728,7 +34728,7 @@
         <v>432712</v>
       </c>
       <c r="B968" s="3" t="s">
-        <v>5792</v>
+        <v>5791</v>
       </c>
       <c r="C968" s="3" t="s">
         <v>3</v>
@@ -34847,7 +34847,7 @@
         <v>436912</v>
       </c>
       <c r="B975" s="3" t="s">
-        <v>5793</v>
+        <v>5792</v>
       </c>
       <c r="C975" s="3" t="s">
         <v>3</v>
@@ -35000,7 +35000,7 @@
         <v>441476</v>
       </c>
       <c r="B984" s="3" t="s">
-        <v>5470</v>
+        <v>5469</v>
       </c>
       <c r="C984" s="3" t="s">
         <v>3</v>
@@ -35017,7 +35017,7 @@
         <v>441593</v>
       </c>
       <c r="B985" s="3" t="s">
-        <v>5794</v>
+        <v>5793</v>
       </c>
       <c r="C985" s="3" t="s">
         <v>3</v>
@@ -35034,7 +35034,7 @@
         <v>441873</v>
       </c>
       <c r="B986" s="3" t="s">
-        <v>5795</v>
+        <v>5794</v>
       </c>
       <c r="C986" s="3" t="s">
         <v>3</v>
@@ -35085,7 +35085,7 @@
         <v>443033</v>
       </c>
       <c r="B989" s="3" t="s">
-        <v>5471</v>
+        <v>5470</v>
       </c>
       <c r="C989" s="3" t="s">
         <v>3</v>
@@ -35102,7 +35102,7 @@
         <v>443358</v>
       </c>
       <c r="B990" s="3" t="s">
-        <v>5472</v>
+        <v>5471</v>
       </c>
       <c r="C990" s="3" t="s">
         <v>3</v>
@@ -35187,7 +35187,7 @@
         <v>445141</v>
       </c>
       <c r="B995" s="3" t="s">
-        <v>5796</v>
+        <v>5795</v>
       </c>
       <c r="C995" s="3" t="s">
         <v>3</v>
@@ -35204,7 +35204,7 @@
         <v>448194</v>
       </c>
       <c r="B996" s="3" t="s">
-        <v>5797</v>
+        <v>5796</v>
       </c>
       <c r="C996" s="3" t="s">
         <v>3</v>
@@ -35221,7 +35221,7 @@
         <v>448240</v>
       </c>
       <c r="B997" s="3" t="s">
-        <v>5798</v>
+        <v>5797</v>
       </c>
       <c r="C997" s="3" t="s">
         <v>3</v>
@@ -35272,7 +35272,7 @@
         <v>450437</v>
       </c>
       <c r="B1000" s="3" t="s">
-        <v>5473</v>
+        <v>5472</v>
       </c>
       <c r="C1000" s="3" t="s">
         <v>3</v>
@@ -35340,7 +35340,7 @@
         <v>452102</v>
       </c>
       <c r="B1004" s="3" t="s">
-        <v>5799</v>
+        <v>5798</v>
       </c>
       <c r="C1004" s="3" t="s">
         <v>3</v>
@@ -35357,7 +35357,7 @@
         <v>452862</v>
       </c>
       <c r="B1005" s="3" t="s">
-        <v>5474</v>
+        <v>5473</v>
       </c>
       <c r="C1005" s="3" t="s">
         <v>3</v>
@@ -35391,7 +35391,7 @@
         <v>454896</v>
       </c>
       <c r="B1007" s="3" t="s">
-        <v>5800</v>
+        <v>5799</v>
       </c>
       <c r="C1007" s="3" t="s">
         <v>3</v>
@@ -35510,7 +35510,7 @@
         <v>458226</v>
       </c>
       <c r="B1014" s="3" t="s">
-        <v>5475</v>
+        <v>5474</v>
       </c>
       <c r="C1014" s="3" t="s">
         <v>3</v>
@@ -35612,7 +35612,7 @@
         <v>462720</v>
       </c>
       <c r="B1020" s="3" t="s">
-        <v>5801</v>
+        <v>5800</v>
       </c>
       <c r="C1020" s="3" t="s">
         <v>3</v>
@@ -35765,7 +35765,7 @@
         <v>465657</v>
       </c>
       <c r="B1029" s="3" t="s">
-        <v>5476</v>
+        <v>5475</v>
       </c>
       <c r="C1029" s="3" t="s">
         <v>3</v>
@@ -35850,7 +35850,7 @@
         <v>467162</v>
       </c>
       <c r="B1034" s="3" t="s">
-        <v>5802</v>
+        <v>5801</v>
       </c>
       <c r="C1034" s="3" t="s">
         <v>3</v>
@@ -35918,7 +35918,7 @@
         <v>468937</v>
       </c>
       <c r="B1038" s="3" t="s">
-        <v>5803</v>
+        <v>5802</v>
       </c>
       <c r="C1038" s="3" t="s">
         <v>3</v>
@@ -35969,7 +35969,7 @@
         <v>470779</v>
       </c>
       <c r="B1041" s="3" t="s">
-        <v>5804</v>
+        <v>5803</v>
       </c>
       <c r="C1041" s="3" t="s">
         <v>3</v>
@@ -36054,7 +36054,7 @@
         <v>473152</v>
       </c>
       <c r="B1046" s="3" t="s">
-        <v>5477</v>
+        <v>5476</v>
       </c>
       <c r="C1046" s="3" t="s">
         <v>3</v>
@@ -36105,7 +36105,7 @@
         <v>474589</v>
       </c>
       <c r="B1049" s="3" t="s">
-        <v>5805</v>
+        <v>5804</v>
       </c>
       <c r="C1049" s="3" t="s">
         <v>3</v>
@@ -36122,7 +36122,7 @@
         <v>475153</v>
       </c>
       <c r="B1050" s="3" t="s">
-        <v>5806</v>
+        <v>5805</v>
       </c>
       <c r="C1050" s="3" t="s">
         <v>3</v>
@@ -36139,7 +36139,7 @@
         <v>475328</v>
       </c>
       <c r="B1051" s="3" t="s">
-        <v>5807</v>
+        <v>5806</v>
       </c>
       <c r="C1051" s="3" t="s">
         <v>3</v>
@@ -36173,7 +36173,7 @@
         <v>476145</v>
       </c>
       <c r="B1053" s="3" t="s">
-        <v>5478</v>
+        <v>5477</v>
       </c>
       <c r="C1053" s="3" t="s">
         <v>3</v>
@@ -36190,7 +36190,7 @@
         <v>476653</v>
       </c>
       <c r="B1054" s="3" t="s">
-        <v>5808</v>
+        <v>5807</v>
       </c>
       <c r="C1054" s="3" t="s">
         <v>3</v>
@@ -36207,7 +36207,7 @@
         <v>476769</v>
       </c>
       <c r="B1055" s="3" t="s">
-        <v>5479</v>
+        <v>5478</v>
       </c>
       <c r="C1055" s="3" t="s">
         <v>3</v>
@@ -36445,7 +36445,7 @@
         <v>482080</v>
       </c>
       <c r="B1069" s="3" t="s">
-        <v>5809</v>
+        <v>5808</v>
       </c>
       <c r="C1069" s="3" t="s">
         <v>3</v>
@@ -36615,7 +36615,7 @@
         <v>485612</v>
       </c>
       <c r="B1079" s="5" t="s">
-        <v>5946</v>
+        <v>5945</v>
       </c>
       <c r="C1079" s="3" t="s">
         <v>3</v>
@@ -36666,7 +36666,7 @@
         <v>487092</v>
       </c>
       <c r="B1082" s="3" t="s">
-        <v>5480</v>
+        <v>5479</v>
       </c>
       <c r="C1082" s="3" t="s">
         <v>3</v>
@@ -36683,7 +36683,7 @@
         <v>487468</v>
       </c>
       <c r="B1083" s="3" t="s">
-        <v>5810</v>
+        <v>5809</v>
       </c>
       <c r="C1083" s="3" t="s">
         <v>3</v>
@@ -36734,7 +36734,7 @@
         <v>488040</v>
       </c>
       <c r="B1086" s="3" t="s">
-        <v>5481</v>
+        <v>5480</v>
       </c>
       <c r="C1086" s="3" t="s">
         <v>3</v>
@@ -36853,7 +36853,7 @@
         <v>493348</v>
       </c>
       <c r="B1093" s="3" t="s">
-        <v>5482</v>
+        <v>5481</v>
       </c>
       <c r="C1093" s="3" t="s">
         <v>3</v>
@@ -36904,7 +36904,7 @@
         <v>495138</v>
       </c>
       <c r="B1096" s="3" t="s">
-        <v>5483</v>
+        <v>5482</v>
       </c>
       <c r="C1096" s="3" t="s">
         <v>3</v>
@@ -36989,7 +36989,7 @@
         <v>499105</v>
       </c>
       <c r="B1101" s="3" t="s">
-        <v>5484</v>
+        <v>5483</v>
       </c>
       <c r="C1101" s="3" t="s">
         <v>3</v>
@@ -37040,7 +37040,7 @@
         <v>500344</v>
       </c>
       <c r="B1104" s="3" t="s">
-        <v>5485</v>
+        <v>5484</v>
       </c>
       <c r="C1104" s="3" t="s">
         <v>3</v>
@@ -37108,7 +37108,7 @@
         <v>502358</v>
       </c>
       <c r="B1108" s="3" t="s">
-        <v>5486</v>
+        <v>5485</v>
       </c>
       <c r="C1108" s="3" t="s">
         <v>3</v>
@@ -37125,7 +37125,7 @@
         <v>502711</v>
       </c>
       <c r="B1109" s="3" t="s">
-        <v>5487</v>
+        <v>5486</v>
       </c>
       <c r="C1109" s="3" t="s">
         <v>3</v>
@@ -37210,7 +37210,7 @@
         <v>504519</v>
       </c>
       <c r="B1114" s="3" t="s">
-        <v>5811</v>
+        <v>5810</v>
       </c>
       <c r="C1114" s="3" t="s">
         <v>3</v>
@@ -37295,7 +37295,7 @@
         <v>505676</v>
       </c>
       <c r="B1119" s="3" t="s">
-        <v>5488</v>
+        <v>5487</v>
       </c>
       <c r="C1119" s="3" t="s">
         <v>3</v>
@@ -37363,7 +37363,7 @@
         <v>506343</v>
       </c>
       <c r="B1123" s="3" t="s">
-        <v>5489</v>
+        <v>5488</v>
       </c>
       <c r="C1123" s="3" t="s">
         <v>3</v>
@@ -37550,7 +37550,7 @@
         <v>509335</v>
       </c>
       <c r="B1134" s="3" t="s">
-        <v>5490</v>
+        <v>5489</v>
       </c>
       <c r="C1134" s="3" t="s">
         <v>3</v>
@@ -37669,7 +37669,7 @@
         <v>510555</v>
       </c>
       <c r="B1141" s="3" t="s">
-        <v>5491</v>
+        <v>5490</v>
       </c>
       <c r="C1141" s="3" t="s">
         <v>3</v>
@@ -37839,7 +37839,7 @@
         <v>515344</v>
       </c>
       <c r="B1151" s="3" t="s">
-        <v>5492</v>
+        <v>5491</v>
       </c>
       <c r="C1151" s="3" t="s">
         <v>3</v>
@@ -38111,7 +38111,7 @@
         <v>523966</v>
       </c>
       <c r="B1167" s="3" t="s">
-        <v>5812</v>
+        <v>5811</v>
       </c>
       <c r="C1167" s="3" t="s">
         <v>3</v>
@@ -38145,7 +38145,7 @@
         <v>525880</v>
       </c>
       <c r="B1169" s="3" t="s">
-        <v>5493</v>
+        <v>5492</v>
       </c>
       <c r="C1169" s="3" t="s">
         <v>3</v>
@@ -38196,7 +38196,7 @@
         <v>527287</v>
       </c>
       <c r="B1172" s="3" t="s">
-        <v>5813</v>
+        <v>5812</v>
       </c>
       <c r="C1172" s="3" t="s">
         <v>3</v>
@@ -38281,7 +38281,7 @@
         <v>529130</v>
       </c>
       <c r="B1177" s="3" t="s">
-        <v>5494</v>
+        <v>5493</v>
       </c>
       <c r="C1177" s="3" t="s">
         <v>3</v>
@@ -38315,7 +38315,7 @@
         <v>529899</v>
       </c>
       <c r="B1179" s="3" t="s">
-        <v>5814</v>
+        <v>5813</v>
       </c>
       <c r="C1179" s="3" t="s">
         <v>3</v>
@@ -38383,7 +38383,7 @@
         <v>530515</v>
       </c>
       <c r="B1183" s="3" t="s">
-        <v>5495</v>
+        <v>5494</v>
       </c>
       <c r="C1183" s="3" t="s">
         <v>3</v>
@@ -38400,7 +38400,7 @@
         <v>530968</v>
       </c>
       <c r="B1184" s="3" t="s">
-        <v>5815</v>
+        <v>5814</v>
       </c>
       <c r="C1184" s="3" t="s">
         <v>3</v>
@@ -38434,7 +38434,7 @@
         <v>532762</v>
       </c>
       <c r="B1186" s="3" t="s">
-        <v>5496</v>
+        <v>5495</v>
       </c>
       <c r="C1186" s="3" t="s">
         <v>3</v>
@@ -38638,7 +38638,7 @@
         <v>537706</v>
       </c>
       <c r="B1198" s="3" t="s">
-        <v>5816</v>
+        <v>5815</v>
       </c>
       <c r="C1198" s="3" t="s">
         <v>3</v>
@@ -38774,7 +38774,7 @@
         <v>539572</v>
       </c>
       <c r="B1206" s="3" t="s">
-        <v>5817</v>
+        <v>5816</v>
       </c>
       <c r="C1206" s="3" t="s">
         <v>3</v>
@@ -38859,7 +38859,7 @@
         <v>541309</v>
       </c>
       <c r="B1211" s="3" t="s">
-        <v>5497</v>
+        <v>5496</v>
       </c>
       <c r="C1211" s="3" t="s">
         <v>3</v>
@@ -38876,7 +38876,7 @@
         <v>541312</v>
       </c>
       <c r="B1212" s="3" t="s">
-        <v>5818</v>
+        <v>5817</v>
       </c>
       <c r="C1212" s="3" t="s">
         <v>3</v>
@@ -38910,7 +38910,7 @@
         <v>542670</v>
       </c>
       <c r="B1214" s="3" t="s">
-        <v>5498</v>
+        <v>5497</v>
       </c>
       <c r="C1214" s="3" t="s">
         <v>3</v>
@@ -39063,7 +39063,7 @@
         <v>544884</v>
       </c>
       <c r="B1223" s="3" t="s">
-        <v>5499</v>
+        <v>5498</v>
       </c>
       <c r="C1223" s="3" t="s">
         <v>3</v>
@@ -39097,7 +39097,7 @@
         <v>545039</v>
       </c>
       <c r="B1225" s="3" t="s">
-        <v>5500</v>
+        <v>5499</v>
       </c>
       <c r="C1225" s="3" t="s">
         <v>3</v>
@@ -39199,7 +39199,7 @@
         <v>546853</v>
       </c>
       <c r="B1231" s="3" t="s">
-        <v>5501</v>
+        <v>5500</v>
       </c>
       <c r="C1231" s="3" t="s">
         <v>3</v>
@@ -39369,7 +39369,7 @@
         <v>550167</v>
       </c>
       <c r="B1241" s="3" t="s">
-        <v>5502</v>
+        <v>5501</v>
       </c>
       <c r="C1241" s="3" t="s">
         <v>3</v>
@@ -39437,7 +39437,7 @@
         <v>552534</v>
       </c>
       <c r="B1245" s="3" t="s">
-        <v>5819</v>
+        <v>5818</v>
       </c>
       <c r="C1245" s="3" t="s">
         <v>3</v>
@@ -39488,7 +39488,7 @@
         <v>553935</v>
       </c>
       <c r="B1248" s="3" t="s">
-        <v>5503</v>
+        <v>5502</v>
       </c>
       <c r="C1248" s="3" t="s">
         <v>3</v>
@@ -39505,7 +39505,7 @@
         <v>554185</v>
       </c>
       <c r="B1249" s="3" t="s">
-        <v>5820</v>
+        <v>5819</v>
       </c>
       <c r="C1249" s="3" t="s">
         <v>3</v>
@@ -39556,7 +39556,7 @@
         <v>554929</v>
       </c>
       <c r="B1252" s="3" t="s">
-        <v>5821</v>
+        <v>5820</v>
       </c>
       <c r="C1252" s="3" t="s">
         <v>3</v>
@@ -39624,7 +39624,7 @@
         <v>555954</v>
       </c>
       <c r="B1256" s="3" t="s">
-        <v>5822</v>
+        <v>5821</v>
       </c>
       <c r="C1256" s="3" t="s">
         <v>3</v>
@@ -39641,7 +39641,7 @@
         <v>555959</v>
       </c>
       <c r="B1257" s="3" t="s">
-        <v>5823</v>
+        <v>5822</v>
       </c>
       <c r="C1257" s="3" t="s">
         <v>3</v>
@@ -39692,7 +39692,7 @@
         <v>558033</v>
       </c>
       <c r="B1260" s="3" t="s">
-        <v>5504</v>
+        <v>5503</v>
       </c>
       <c r="C1260" s="3" t="s">
         <v>3</v>
@@ -39743,7 +39743,7 @@
         <v>559580</v>
       </c>
       <c r="B1263" s="3" t="s">
-        <v>5824</v>
+        <v>5823</v>
       </c>
       <c r="C1263" s="3" t="s">
         <v>3</v>
@@ -39777,7 +39777,7 @@
         <v>559956</v>
       </c>
       <c r="B1265" s="3" t="s">
-        <v>5825</v>
+        <v>5824</v>
       </c>
       <c r="C1265" s="3" t="s">
         <v>3</v>
@@ -40202,7 +40202,7 @@
         <v>567118</v>
       </c>
       <c r="B1290" s="3" t="s">
-        <v>5826</v>
+        <v>5825</v>
       </c>
       <c r="C1290" s="3" t="s">
         <v>3</v>
@@ -40219,7 +40219,7 @@
         <v>567465</v>
       </c>
       <c r="B1291" s="3" t="s">
-        <v>5827</v>
+        <v>5826</v>
       </c>
       <c r="C1291" s="3" t="s">
         <v>3</v>
@@ -40236,7 +40236,7 @@
         <v>567627</v>
       </c>
       <c r="B1292" s="3" t="s">
-        <v>5505</v>
+        <v>5504</v>
       </c>
       <c r="C1292" s="3" t="s">
         <v>3</v>
@@ -40253,7 +40253,7 @@
         <v>567772</v>
       </c>
       <c r="B1293" s="3" t="s">
-        <v>5828</v>
+        <v>5827</v>
       </c>
       <c r="C1293" s="3" t="s">
         <v>3</v>
@@ -40372,7 +40372,7 @@
         <v>570624</v>
       </c>
       <c r="B1300" s="3" t="s">
-        <v>5829</v>
+        <v>5828</v>
       </c>
       <c r="C1300" s="3" t="s">
         <v>3</v>
@@ -40457,7 +40457,7 @@
         <v>573335</v>
       </c>
       <c r="B1305" s="3" t="s">
-        <v>5506</v>
+        <v>5505</v>
       </c>
       <c r="C1305" s="3" t="s">
         <v>3</v>
@@ -40525,7 +40525,7 @@
         <v>577935</v>
       </c>
       <c r="B1309" s="3" t="s">
-        <v>5507</v>
+        <v>5506</v>
       </c>
       <c r="C1309" s="3" t="s">
         <v>3</v>
@@ -40542,7 +40542,7 @@
         <v>578095</v>
       </c>
       <c r="B1310" s="3" t="s">
-        <v>5508</v>
+        <v>5507</v>
       </c>
       <c r="C1310" s="3" t="s">
         <v>3</v>
@@ -40678,7 +40678,7 @@
         <v>581820</v>
       </c>
       <c r="B1318" s="3" t="s">
-        <v>5830</v>
+        <v>5829</v>
       </c>
       <c r="C1318" s="3" t="s">
         <v>3</v>
@@ -40899,7 +40899,7 @@
         <v>585234</v>
       </c>
       <c r="B1331" s="3" t="s">
-        <v>5831</v>
+        <v>5830</v>
       </c>
       <c r="C1331" s="3" t="s">
         <v>3</v>
@@ -40967,7 +40967,7 @@
         <v>585471</v>
       </c>
       <c r="B1335" s="3" t="s">
-        <v>5509</v>
+        <v>5508</v>
       </c>
       <c r="C1335" s="3" t="s">
         <v>3</v>
@@ -41171,7 +41171,7 @@
         <v>589917</v>
       </c>
       <c r="B1347" s="3" t="s">
-        <v>5510</v>
+        <v>5509</v>
       </c>
       <c r="C1347" s="3" t="s">
         <v>3</v>
@@ -41273,7 +41273,7 @@
         <v>593741</v>
       </c>
       <c r="B1353" s="3" t="s">
-        <v>5511</v>
+        <v>5510</v>
       </c>
       <c r="C1353" s="3" t="s">
         <v>3</v>
@@ -41324,7 +41324,7 @@
         <v>594675</v>
       </c>
       <c r="B1356" s="3" t="s">
-        <v>5832</v>
+        <v>5831</v>
       </c>
       <c r="C1356" s="3" t="s">
         <v>3</v>
@@ -41358,7 +41358,7 @@
         <v>595444</v>
       </c>
       <c r="B1358" s="3" t="s">
-        <v>5512</v>
+        <v>5511</v>
       </c>
       <c r="C1358" s="3" t="s">
         <v>3</v>
@@ -41647,7 +41647,7 @@
         <v>601844</v>
       </c>
       <c r="B1375" s="3" t="s">
-        <v>5833</v>
+        <v>5832</v>
       </c>
       <c r="C1375" s="3" t="s">
         <v>3</v>
@@ -41868,7 +41868,7 @@
         <v>606982</v>
       </c>
       <c r="B1388" s="3" t="s">
-        <v>5834</v>
+        <v>5833</v>
       </c>
       <c r="C1388" s="3" t="s">
         <v>3</v>
@@ -42123,7 +42123,7 @@
         <v>611217</v>
       </c>
       <c r="B1403" s="3" t="s">
-        <v>5513</v>
+        <v>5512</v>
       </c>
       <c r="C1403" s="3" t="s">
         <v>3</v>
@@ -42310,7 +42310,7 @@
         <v>613079</v>
       </c>
       <c r="B1414" s="3" t="s">
-        <v>5835</v>
+        <v>5834</v>
       </c>
       <c r="C1414" s="3" t="s">
         <v>3</v>
@@ -42344,7 +42344,7 @@
         <v>614449</v>
       </c>
       <c r="B1416" s="3" t="s">
-        <v>5836</v>
+        <v>5835</v>
       </c>
       <c r="C1416" s="3" t="s">
         <v>3</v>
@@ -42395,7 +42395,7 @@
         <v>615195</v>
       </c>
       <c r="B1419" s="3" t="s">
-        <v>5514</v>
+        <v>5513</v>
       </c>
       <c r="C1419" s="3" t="s">
         <v>3</v>
@@ -42582,7 +42582,7 @@
         <v>618730</v>
       </c>
       <c r="B1430" s="3" t="s">
-        <v>5515</v>
+        <v>5514</v>
       </c>
       <c r="C1430" s="3" t="s">
         <v>3</v>
@@ -42616,7 +42616,7 @@
         <v>619630</v>
       </c>
       <c r="B1432" s="3" t="s">
-        <v>5516</v>
+        <v>5515</v>
       </c>
       <c r="C1432" s="3" t="s">
         <v>3</v>
@@ -42769,7 +42769,7 @@
         <v>622404</v>
       </c>
       <c r="B1441" s="3" t="s">
-        <v>5517</v>
+        <v>5516</v>
       </c>
       <c r="C1441" s="3" t="s">
         <v>3</v>
@@ -42837,7 +42837,7 @@
         <v>624098</v>
       </c>
       <c r="B1445" s="3" t="s">
-        <v>5518</v>
+        <v>5517</v>
       </c>
       <c r="C1445" s="3" t="s">
         <v>3</v>
@@ -42888,7 +42888,7 @@
         <v>625027</v>
       </c>
       <c r="B1448" s="3" t="s">
-        <v>5519</v>
+        <v>5518</v>
       </c>
       <c r="C1448" s="3" t="s">
         <v>3</v>
@@ -43126,7 +43126,7 @@
         <v>631291</v>
       </c>
       <c r="B1462" s="3" t="s">
-        <v>5520</v>
+        <v>5519</v>
       </c>
       <c r="C1462" s="3" t="s">
         <v>3</v>
@@ -43279,7 +43279,7 @@
         <v>637472</v>
       </c>
       <c r="B1471" s="3" t="s">
-        <v>5521</v>
+        <v>5520</v>
       </c>
       <c r="C1471" s="3" t="s">
         <v>3</v>
@@ -43585,7 +43585,7 @@
         <v>641165</v>
       </c>
       <c r="B1489" s="3" t="s">
-        <v>5522</v>
+        <v>5521</v>
       </c>
       <c r="C1489" s="3" t="s">
         <v>3</v>
@@ -43619,7 +43619,7 @@
         <v>641451</v>
       </c>
       <c r="B1491" s="3" t="s">
-        <v>5523</v>
+        <v>5522</v>
       </c>
       <c r="C1491" s="3" t="s">
         <v>3</v>
@@ -43636,7 +43636,7 @@
         <v>641600</v>
       </c>
       <c r="B1492" s="3" t="s">
-        <v>5524</v>
+        <v>5523</v>
       </c>
       <c r="C1492" s="3" t="s">
         <v>3</v>
@@ -43738,7 +43738,7 @@
         <v>643238</v>
       </c>
       <c r="B1498" s="3" t="s">
-        <v>5525</v>
+        <v>5524</v>
       </c>
       <c r="C1498" s="3" t="s">
         <v>3</v>
@@ -43772,7 +43772,7 @@
         <v>644774</v>
       </c>
       <c r="B1500" s="3" t="s">
-        <v>5837</v>
+        <v>5836</v>
       </c>
       <c r="C1500" s="3" t="s">
         <v>3</v>
@@ -43789,7 +43789,7 @@
         <v>645456</v>
       </c>
       <c r="B1501" s="3" t="s">
-        <v>5838</v>
+        <v>5837</v>
       </c>
       <c r="C1501" s="3" t="s">
         <v>3</v>
@@ -43806,7 +43806,7 @@
         <v>646120</v>
       </c>
       <c r="B1502" s="3" t="s">
-        <v>5839</v>
+        <v>5838</v>
       </c>
       <c r="C1502" s="3" t="s">
         <v>3</v>
@@ -43908,7 +43908,7 @@
         <v>646636</v>
       </c>
       <c r="B1508" s="3" t="s">
-        <v>5840</v>
+        <v>5839</v>
       </c>
       <c r="C1508" s="3" t="s">
         <v>3</v>
@@ -43925,7 +43925,7 @@
         <v>646742</v>
       </c>
       <c r="B1509" s="3" t="s">
-        <v>5841</v>
+        <v>5840</v>
       </c>
       <c r="C1509" s="3" t="s">
         <v>3</v>
@@ -43959,7 +43959,7 @@
         <v>647191</v>
       </c>
       <c r="B1511" s="3" t="s">
-        <v>5842</v>
+        <v>5841</v>
       </c>
       <c r="C1511" s="3" t="s">
         <v>3</v>
@@ -44095,7 +44095,7 @@
         <v>650292</v>
       </c>
       <c r="B1519" s="3" t="s">
-        <v>5843</v>
+        <v>5842</v>
       </c>
       <c r="C1519" s="3" t="s">
         <v>3</v>
@@ -44146,7 +44146,7 @@
         <v>651066</v>
       </c>
       <c r="B1522" s="3" t="s">
-        <v>5844</v>
+        <v>5843</v>
       </c>
       <c r="C1522" s="3" t="s">
         <v>3</v>
@@ -44163,7 +44163,7 @@
         <v>651411</v>
       </c>
       <c r="B1523" s="3" t="s">
-        <v>5526</v>
+        <v>5525</v>
       </c>
       <c r="C1523" s="3" t="s">
         <v>3</v>
@@ -44248,7 +44248,7 @@
         <v>653059</v>
       </c>
       <c r="B1528" s="3" t="s">
-        <v>5527</v>
+        <v>5526</v>
       </c>
       <c r="C1528" s="3" t="s">
         <v>3</v>
@@ -44333,7 +44333,7 @@
         <v>655324</v>
       </c>
       <c r="B1533" s="3" t="s">
-        <v>5845</v>
+        <v>5844</v>
       </c>
       <c r="C1533" s="3" t="s">
         <v>3</v>
@@ -44350,7 +44350,7 @@
         <v>655654</v>
       </c>
       <c r="B1534" s="3" t="s">
-        <v>5846</v>
+        <v>5845</v>
       </c>
       <c r="C1534" s="3" t="s">
         <v>3</v>
@@ -44622,7 +44622,7 @@
         <v>660479</v>
       </c>
       <c r="B1550" s="3" t="s">
-        <v>5528</v>
+        <v>5527</v>
       </c>
       <c r="C1550" s="3" t="s">
         <v>3</v>
@@ -44639,7 +44639,7 @@
         <v>660480</v>
       </c>
       <c r="B1551" s="3" t="s">
-        <v>5529</v>
+        <v>5528</v>
       </c>
       <c r="C1551" s="3" t="s">
         <v>3</v>
@@ -44758,7 +44758,7 @@
         <v>662129</v>
       </c>
       <c r="B1558" s="3" t="s">
-        <v>5847</v>
+        <v>5846</v>
       </c>
       <c r="C1558" s="3" t="s">
         <v>3</v>
@@ -44809,7 +44809,7 @@
         <v>662387</v>
       </c>
       <c r="B1561" s="3" t="s">
-        <v>5530</v>
+        <v>5529</v>
       </c>
       <c r="C1561" s="3" t="s">
         <v>3</v>
@@ -44911,7 +44911,7 @@
         <v>663699</v>
       </c>
       <c r="B1567" s="3" t="s">
-        <v>5531</v>
+        <v>5530</v>
       </c>
       <c r="C1567" s="3" t="s">
         <v>3</v>
@@ -45302,7 +45302,7 @@
         <v>673034</v>
       </c>
       <c r="B1590" s="3" t="s">
-        <v>5848</v>
+        <v>5847</v>
       </c>
       <c r="C1590" s="3" t="s">
         <v>3</v>
@@ -45523,7 +45523,7 @@
         <v>677217</v>
       </c>
       <c r="B1603" s="3" t="s">
-        <v>5532</v>
+        <v>5531</v>
       </c>
       <c r="C1603" s="3" t="s">
         <v>3</v>
@@ -45710,7 +45710,7 @@
         <v>680269</v>
       </c>
       <c r="B1614" s="3" t="s">
-        <v>5533</v>
+        <v>5532</v>
       </c>
       <c r="C1614" s="3" t="s">
         <v>3</v>
@@ -45812,7 +45812,7 @@
         <v>681885</v>
       </c>
       <c r="B1620" s="3" t="s">
-        <v>5534</v>
+        <v>5533</v>
       </c>
       <c r="C1620" s="3" t="s">
         <v>3</v>
@@ -45897,7 +45897,7 @@
         <v>681890</v>
       </c>
       <c r="B1625" s="3" t="s">
-        <v>5535</v>
+        <v>5534</v>
       </c>
       <c r="C1625" s="3" t="s">
         <v>3</v>
@@ -45982,7 +45982,7 @@
         <v>682745</v>
       </c>
       <c r="B1630" s="3" t="s">
-        <v>5536</v>
+        <v>5535</v>
       </c>
       <c r="C1630" s="3" t="s">
         <v>3</v>
@@ -46101,7 +46101,7 @@
         <v>684053</v>
       </c>
       <c r="B1637" s="3" t="s">
-        <v>5849</v>
+        <v>5848</v>
       </c>
       <c r="C1637" s="3" t="s">
         <v>3</v>
@@ -46169,7 +46169,7 @@
         <v>684684</v>
       </c>
       <c r="B1641" s="3" t="s">
-        <v>5537</v>
+        <v>5536</v>
       </c>
       <c r="C1641" s="3" t="s">
         <v>3</v>
@@ -46203,7 +46203,7 @@
         <v>684967</v>
       </c>
       <c r="B1643" s="3" t="s">
-        <v>5850</v>
+        <v>5849</v>
       </c>
       <c r="C1643" s="3" t="s">
         <v>3</v>
@@ -46254,7 +46254,7 @@
         <v>685601</v>
       </c>
       <c r="B1646" s="3" t="s">
-        <v>5851</v>
+        <v>5850</v>
       </c>
       <c r="C1646" s="3" t="s">
         <v>3</v>
@@ -46288,7 +46288,7 @@
         <v>685739</v>
       </c>
       <c r="B1648" s="3" t="s">
-        <v>5538</v>
+        <v>5537</v>
       </c>
       <c r="C1648" s="3" t="s">
         <v>3</v>
@@ -46390,7 +46390,7 @@
         <v>686259</v>
       </c>
       <c r="B1654" s="3" t="s">
-        <v>5539</v>
+        <v>5538</v>
       </c>
       <c r="C1654" s="3" t="s">
         <v>3</v>
@@ -46424,7 +46424,7 @@
         <v>686336</v>
       </c>
       <c r="B1656" s="3" t="s">
-        <v>5540</v>
+        <v>5539</v>
       </c>
       <c r="C1656" s="3" t="s">
         <v>3</v>
@@ -46679,7 +46679,7 @@
         <v>688340</v>
       </c>
       <c r="B1671" s="3" t="s">
-        <v>5541</v>
+        <v>5540</v>
       </c>
       <c r="C1671" s="3" t="s">
         <v>3</v>
@@ -46730,7 +46730,7 @@
         <v>688809</v>
       </c>
       <c r="B1674" s="3" t="s">
-        <v>5542</v>
+        <v>5541</v>
       </c>
       <c r="C1674" s="3" t="s">
         <v>3</v>
@@ -46815,7 +46815,7 @@
         <v>689981</v>
       </c>
       <c r="B1679" s="3" t="s">
-        <v>5852</v>
+        <v>5851</v>
       </c>
       <c r="C1679" s="3" t="s">
         <v>3</v>
@@ -46951,7 +46951,7 @@
         <v>691484</v>
       </c>
       <c r="B1687" s="3" t="s">
-        <v>5543</v>
+        <v>5542</v>
       </c>
       <c r="C1687" s="3" t="s">
         <v>3</v>
@@ -47002,7 +47002,7 @@
         <v>694175</v>
       </c>
       <c r="B1690" s="3" t="s">
-        <v>5544</v>
+        <v>5543</v>
       </c>
       <c r="C1690" s="3" t="s">
         <v>3</v>
@@ -47019,7 +47019,7 @@
         <v>694547</v>
       </c>
       <c r="B1691" s="3" t="s">
-        <v>5545</v>
+        <v>5544</v>
       </c>
       <c r="C1691" s="3" t="s">
         <v>3</v>
@@ -47087,7 +47087,7 @@
         <v>695102</v>
       </c>
       <c r="B1695" s="3" t="s">
-        <v>5546</v>
+        <v>5545</v>
       </c>
       <c r="C1695" s="3" t="s">
         <v>3</v>
@@ -47104,7 +47104,7 @@
         <v>695239</v>
       </c>
       <c r="B1696" s="3" t="s">
-        <v>5853</v>
+        <v>5852</v>
       </c>
       <c r="C1696" s="3" t="s">
         <v>3</v>
@@ -47274,7 +47274,7 @@
         <v>699637</v>
       </c>
       <c r="B1706" s="3" t="s">
-        <v>5547</v>
+        <v>5546</v>
       </c>
       <c r="C1706" s="3" t="s">
         <v>3</v>
@@ -47308,7 +47308,7 @@
         <v>700137</v>
       </c>
       <c r="B1708" s="3" t="s">
-        <v>5548</v>
+        <v>5547</v>
       </c>
       <c r="C1708" s="3" t="s">
         <v>3</v>
@@ -47342,7 +47342,7 @@
         <v>700761</v>
       </c>
       <c r="B1710" s="3" t="s">
-        <v>5854</v>
+        <v>5853</v>
       </c>
       <c r="C1710" s="3" t="s">
         <v>3</v>
@@ -47461,7 +47461,7 @@
         <v>701527</v>
       </c>
       <c r="B1717" s="3" t="s">
-        <v>5549</v>
+        <v>5548</v>
       </c>
       <c r="C1717" s="3" t="s">
         <v>3</v>
@@ -47648,7 +47648,7 @@
         <v>808758</v>
       </c>
       <c r="B1728" s="3" t="s">
-        <v>5550</v>
+        <v>5549</v>
       </c>
       <c r="C1728" s="3" t="s">
         <v>3</v>
@@ -47869,7 +47869,7 @@
         <v>826937</v>
       </c>
       <c r="B1741" s="3" t="s">
-        <v>5855</v>
+        <v>5854</v>
       </c>
       <c r="C1741" s="3" t="s">
         <v>3</v>
@@ -48073,7 +48073,7 @@
         <v>836749</v>
       </c>
       <c r="B1753" s="3" t="s">
-        <v>5551</v>
+        <v>5550</v>
       </c>
       <c r="C1753" s="3" t="s">
         <v>3</v>
@@ -48243,7 +48243,7 @@
         <v>838965</v>
       </c>
       <c r="B1763" s="3" t="s">
-        <v>5856</v>
+        <v>5855</v>
       </c>
       <c r="C1763" s="3" t="s">
         <v>3</v>
@@ -48277,7 +48277,7 @@
         <v>841373</v>
       </c>
       <c r="B1765" s="3" t="s">
-        <v>5857</v>
+        <v>5856</v>
       </c>
       <c r="C1765" s="3" t="s">
         <v>3</v>
@@ -48345,7 +48345,7 @@
         <v>841528</v>
       </c>
       <c r="B1769" s="3" t="s">
-        <v>5858</v>
+        <v>5857</v>
       </c>
       <c r="C1769" s="3" t="s">
         <v>3</v>
@@ -48413,7 +48413,7 @@
         <v>841533</v>
       </c>
       <c r="B1773" s="3" t="s">
-        <v>5552</v>
+        <v>5551</v>
       </c>
       <c r="C1773" s="3" t="s">
         <v>3</v>
@@ -48549,7 +48549,7 @@
         <v>845513</v>
       </c>
       <c r="B1781" s="3" t="s">
-        <v>5859</v>
+        <v>5858</v>
       </c>
       <c r="C1781" s="3" t="s">
         <v>3</v>
@@ -48634,7 +48634,7 @@
         <v>848985</v>
       </c>
       <c r="B1786" s="3" t="s">
-        <v>5553</v>
+        <v>5552</v>
       </c>
       <c r="C1786" s="3" t="s">
         <v>3</v>
@@ -48719,7 +48719,7 @@
         <v>851990</v>
       </c>
       <c r="B1791" s="3" t="s">
-        <v>5860</v>
+        <v>5859</v>
       </c>
       <c r="C1791" s="3" t="s">
         <v>3</v>
@@ -48821,7 +48821,7 @@
         <v>857892</v>
       </c>
       <c r="B1797" s="3" t="s">
-        <v>5861</v>
+        <v>5860</v>
       </c>
       <c r="C1797" s="3" t="s">
         <v>3</v>
@@ -48889,7 +48889,7 @@
         <v>860533</v>
       </c>
       <c r="B1801" s="3" t="s">
-        <v>5862</v>
+        <v>5861</v>
       </c>
       <c r="C1801" s="3" t="s">
         <v>3</v>
@@ -49076,7 +49076,7 @@
         <v>868789</v>
       </c>
       <c r="B1812" s="3" t="s">
-        <v>5554</v>
+        <v>5553</v>
       </c>
       <c r="C1812" s="3" t="s">
         <v>3</v>
@@ -49144,7 +49144,7 @@
         <v>873623</v>
       </c>
       <c r="B1816" s="3" t="s">
-        <v>5555</v>
+        <v>5554</v>
       </c>
       <c r="C1816" s="3" t="s">
         <v>3</v>
@@ -49229,7 +49229,7 @@
         <v>878176</v>
       </c>
       <c r="B1821" s="3" t="s">
-        <v>5863</v>
+        <v>5862</v>
       </c>
       <c r="C1821" s="3" t="s">
         <v>3</v>
@@ -49263,7 +49263,7 @@
         <v>879568</v>
       </c>
       <c r="B1823" s="3" t="s">
-        <v>5556</v>
+        <v>5555</v>
       </c>
       <c r="C1823" s="3" t="s">
         <v>3</v>
@@ -49331,7 +49331,7 @@
         <v>888265</v>
       </c>
       <c r="B1827" s="3" t="s">
-        <v>5557</v>
+        <v>5556</v>
       </c>
       <c r="C1827" s="3" t="s">
         <v>3</v>
@@ -49824,7 +49824,7 @@
         <v>909009</v>
       </c>
       <c r="B1856" s="3" t="s">
-        <v>5558</v>
+        <v>5557</v>
       </c>
       <c r="C1856" s="3" t="s">
         <v>3</v>
@@ -49994,7 +49994,7 @@
         <v>924120</v>
       </c>
       <c r="B1866" s="3" t="s">
-        <v>5559</v>
+        <v>5558</v>
       </c>
       <c r="C1866" s="3" t="s">
         <v>3</v>
@@ -50062,7 +50062,7 @@
         <v>932362</v>
       </c>
       <c r="B1870" s="3" t="s">
-        <v>5560</v>
+        <v>5559</v>
       </c>
       <c r="C1870" s="3" t="s">
         <v>3</v>
@@ -50130,7 +50130,7 @@
         <v>937325</v>
       </c>
       <c r="B1874" s="3" t="s">
-        <v>5561</v>
+        <v>5560</v>
       </c>
       <c r="C1874" s="3" t="s">
         <v>3</v>
@@ -50181,7 +50181,7 @@
         <v>939901</v>
       </c>
       <c r="B1877" s="3" t="s">
-        <v>5864</v>
+        <v>5863</v>
       </c>
       <c r="C1877" s="3" t="s">
         <v>3</v>
@@ -50283,7 +50283,7 @@
         <v>947155</v>
       </c>
       <c r="B1883" s="3" t="s">
-        <v>5562</v>
+        <v>5561</v>
       </c>
       <c r="C1883" s="3" t="s">
         <v>3</v>
@@ -50521,7 +50521,7 @@
         <v>956445</v>
       </c>
       <c r="B1897" s="3" t="s">
-        <v>5865</v>
+        <v>5864</v>
       </c>
       <c r="C1897" s="3" t="s">
         <v>3</v>
@@ -50623,7 +50623,7 @@
         <v>960578</v>
       </c>
       <c r="B1903" s="3" t="s">
-        <v>5866</v>
+        <v>5865</v>
       </c>
       <c r="C1903" s="3" t="s">
         <v>3</v>
@@ -50674,7 +50674,7 @@
         <v>962282</v>
       </c>
       <c r="B1906" s="3" t="s">
-        <v>5867</v>
+        <v>5866</v>
       </c>
       <c r="C1906" s="3" t="s">
         <v>3</v>
@@ -50742,7 +50742,7 @@
         <v>963991</v>
       </c>
       <c r="B1910" s="3" t="s">
-        <v>5868</v>
+        <v>5867</v>
       </c>
       <c r="C1910" s="3" t="s">
         <v>3</v>
@@ -50861,7 +50861,7 @@
         <v>976272</v>
       </c>
       <c r="B1917" s="3" t="s">
-        <v>5563</v>
+        <v>5562</v>
       </c>
       <c r="C1917" s="3" t="s">
         <v>3</v>
@@ -50878,7 +50878,7 @@
         <v>976274</v>
       </c>
       <c r="B1918" s="3" t="s">
-        <v>5869</v>
+        <v>5868</v>
       </c>
       <c r="C1918" s="3" t="s">
         <v>3</v>
@@ -51014,7 +51014,7 @@
         <v>980825</v>
       </c>
       <c r="B1926" s="3" t="s">
-        <v>5495</v>
+        <v>5494</v>
       </c>
       <c r="C1926" s="3" t="s">
         <v>3</v>
@@ -51082,7 +51082,7 @@
         <v>985161</v>
       </c>
       <c r="B1930" s="3" t="s">
-        <v>5564</v>
+        <v>5563</v>
       </c>
       <c r="C1930" s="3" t="s">
         <v>3</v>
@@ -51116,7 +51116,7 @@
         <v>986735</v>
       </c>
       <c r="B1932" s="3" t="s">
-        <v>5870</v>
+        <v>5869</v>
       </c>
       <c r="C1932" s="3" t="s">
         <v>3</v>
@@ -51133,7 +51133,7 @@
         <v>987620</v>
       </c>
       <c r="B1933" s="3" t="s">
-        <v>5565</v>
+        <v>5564</v>
       </c>
       <c r="C1933" s="3" t="s">
         <v>3</v>
@@ -51303,7 +51303,7 @@
         <v>994764</v>
       </c>
       <c r="B1943" s="3" t="s">
-        <v>5566</v>
+        <v>5565</v>
       </c>
       <c r="C1943" s="3" t="s">
         <v>3</v>
@@ -51320,7 +51320,7 @@
         <v>994840</v>
       </c>
       <c r="B1944" s="3" t="s">
-        <v>5567</v>
+        <v>5566</v>
       </c>
       <c r="C1944" s="3" t="s">
         <v>3</v>
@@ -51337,7 +51337,7 @@
         <v>994932</v>
       </c>
       <c r="B1945" s="3" t="s">
-        <v>5871</v>
+        <v>5870</v>
       </c>
       <c r="C1945" s="3" t="s">
         <v>3</v>
@@ -51609,7 +51609,7 @@
         <v>1009758</v>
       </c>
       <c r="B1961" s="3" t="s">
-        <v>5568</v>
+        <v>5567</v>
       </c>
       <c r="C1961" s="3" t="s">
         <v>3</v>
@@ -51711,7 +51711,7 @@
         <v>1011533</v>
       </c>
       <c r="B1967" s="3" t="s">
-        <v>5872</v>
+        <v>5871</v>
       </c>
       <c r="C1967" s="3" t="s">
         <v>3</v>
@@ -51779,7 +51779,7 @@
         <v>1012491</v>
       </c>
       <c r="B1971" s="3" t="s">
-        <v>5873</v>
+        <v>5872</v>
       </c>
       <c r="C1971" s="3" t="s">
         <v>3</v>
@@ -51813,7 +51813,7 @@
         <v>1013869</v>
       </c>
       <c r="B1973" s="3" t="s">
-        <v>5874</v>
+        <v>5873</v>
       </c>
       <c r="C1973" s="3" t="s">
         <v>3</v>
@@ -51864,7 +51864,7 @@
         <v>1016541</v>
       </c>
       <c r="B1976" s="3" t="s">
-        <v>5875</v>
+        <v>5874</v>
       </c>
       <c r="C1976" s="3" t="s">
         <v>3</v>
@@ -51881,7 +51881,7 @@
         <v>1018117</v>
       </c>
       <c r="B1977" s="3" t="s">
-        <v>5876</v>
+        <v>5875</v>
       </c>
       <c r="C1977" s="3" t="s">
         <v>3</v>
@@ -51898,7 +51898,7 @@
         <v>1018638</v>
       </c>
       <c r="B1978" s="3" t="s">
-        <v>5877</v>
+        <v>5876</v>
       </c>
       <c r="C1978" s="3" t="s">
         <v>3</v>
@@ -51966,7 +51966,7 @@
         <v>1021214</v>
       </c>
       <c r="B1982" s="3" t="s">
-        <v>5878</v>
+        <v>5877</v>
       </c>
       <c r="C1982" s="3" t="s">
         <v>3</v>
@@ -52000,7 +52000,7 @@
         <v>1024377</v>
       </c>
       <c r="B1984" s="3" t="s">
-        <v>5879</v>
+        <v>5878</v>
       </c>
       <c r="C1984" s="3" t="s">
         <v>3</v>
@@ -52034,7 +52034,7 @@
         <v>1026143</v>
       </c>
       <c r="B1986" s="3" t="s">
-        <v>5569</v>
+        <v>5568</v>
       </c>
       <c r="C1986" s="3" t="s">
         <v>3</v>
@@ -52102,7 +52102,7 @@
         <v>1028997</v>
       </c>
       <c r="B1990" s="3" t="s">
-        <v>5570</v>
+        <v>5569</v>
       </c>
       <c r="C1990" s="3" t="s">
         <v>3</v>
@@ -52136,7 +52136,7 @@
         <v>1031747</v>
       </c>
       <c r="B1992" s="3" t="s">
-        <v>5880</v>
+        <v>5879</v>
       </c>
       <c r="C1992" s="3" t="s">
         <v>3</v>
@@ -52221,7 +52221,7 @@
         <v>1037645</v>
       </c>
       <c r="B1997" s="3" t="s">
-        <v>5571</v>
+        <v>5570</v>
       </c>
       <c r="C1997" s="3" t="s">
         <v>3</v>
@@ -52255,7 +52255,7 @@
         <v>1039852</v>
       </c>
       <c r="B1999" s="3" t="s">
-        <v>5572</v>
+        <v>5571</v>
       </c>
       <c r="C1999" s="3" t="s">
         <v>3</v>
@@ -52340,7 +52340,7 @@
         <v>1046931</v>
       </c>
       <c r="B2004" s="3" t="s">
-        <v>5573</v>
+        <v>5572</v>
       </c>
       <c r="C2004" s="3" t="s">
         <v>3</v>
@@ -52374,7 +52374,7 @@
         <v>1048745</v>
       </c>
       <c r="B2006" s="3" t="s">
-        <v>5881</v>
+        <v>5880</v>
       </c>
       <c r="C2006" s="3" t="s">
         <v>3</v>
@@ -52476,7 +52476,7 @@
         <v>1050566</v>
       </c>
       <c r="B2012" s="3" t="s">
-        <v>5574</v>
+        <v>5573</v>
       </c>
       <c r="C2012" s="3" t="s">
         <v>3</v>
@@ -52561,7 +52561,7 @@
         <v>1052686</v>
       </c>
       <c r="B2017" s="3" t="s">
-        <v>5575</v>
+        <v>5574</v>
       </c>
       <c r="C2017" s="3" t="s">
         <v>3</v>
@@ -52629,7 +52629,7 @@
         <v>1056353</v>
       </c>
       <c r="B2021" s="3" t="s">
-        <v>5882</v>
+        <v>5881</v>
       </c>
       <c r="C2021" s="3" t="s">
         <v>3</v>
@@ -52680,7 +52680,7 @@
         <v>1059131</v>
       </c>
       <c r="B2024" s="3" t="s">
-        <v>5576</v>
+        <v>5575</v>
       </c>
       <c r="C2024" s="3" t="s">
         <v>3</v>
@@ -52697,7 +52697,7 @@
         <v>1060800</v>
       </c>
       <c r="B2025" s="3" t="s">
-        <v>5577</v>
+        <v>5576</v>
       </c>
       <c r="C2025" s="3" t="s">
         <v>3</v>
@@ -52799,7 +52799,7 @@
         <v>1068978</v>
       </c>
       <c r="B2031" s="3" t="s">
-        <v>5883</v>
+        <v>5882</v>
       </c>
       <c r="C2031" s="3" t="s">
         <v>3</v>
@@ -52833,7 +52833,7 @@
         <v>1071021</v>
       </c>
       <c r="B2033" s="3" t="s">
-        <v>5578</v>
+        <v>5577</v>
       </c>
       <c r="C2033" s="3" t="s">
         <v>3</v>
@@ -52901,7 +52901,7 @@
         <v>1073213</v>
       </c>
       <c r="B2037" s="3" t="s">
-        <v>5884</v>
+        <v>5883</v>
       </c>
       <c r="C2037" s="3" t="s">
         <v>3</v>
@@ -52918,7 +52918,7 @@
         <v>1073948</v>
       </c>
       <c r="B2038" s="3" t="s">
-        <v>5579</v>
+        <v>5578</v>
       </c>
       <c r="C2038" s="3" t="s">
         <v>3</v>
@@ -52952,7 +52952,7 @@
         <v>1074228</v>
       </c>
       <c r="B2040" s="3" t="s">
-        <v>5885</v>
+        <v>5884</v>
       </c>
       <c r="C2040" s="3" t="s">
         <v>3</v>
@@ -53054,7 +53054,7 @@
         <v>1078485</v>
       </c>
       <c r="B2046" s="3" t="s">
-        <v>5886</v>
+        <v>5885</v>
       </c>
       <c r="C2046" s="3" t="s">
         <v>3</v>
@@ -53190,7 +53190,7 @@
         <v>1084345</v>
       </c>
       <c r="B2054" s="3" t="s">
-        <v>5887</v>
+        <v>5886</v>
       </c>
       <c r="C2054" s="3" t="s">
         <v>3</v>
@@ -53343,7 +53343,7 @@
         <v>1091726</v>
       </c>
       <c r="B2063" s="3" t="s">
-        <v>5580</v>
+        <v>5579</v>
       </c>
       <c r="C2063" s="3" t="s">
         <v>3</v>
@@ -53479,7 +53479,7 @@
         <v>1099041</v>
       </c>
       <c r="B2071" s="3" t="s">
-        <v>5581</v>
+        <v>5580</v>
       </c>
       <c r="C2071" s="3" t="s">
         <v>3</v>
@@ -53530,7 +53530,7 @@
         <v>1101870</v>
       </c>
       <c r="B2074" s="3" t="s">
-        <v>5888</v>
+        <v>5887</v>
       </c>
       <c r="C2074" s="3" t="s">
         <v>3</v>
@@ -53547,7 +53547,7 @@
         <v>1102128</v>
       </c>
       <c r="B2075" s="3" t="s">
-        <v>5582</v>
+        <v>5581</v>
       </c>
       <c r="C2075" s="3" t="s">
         <v>3</v>
@@ -53802,7 +53802,7 @@
         <v>1112419</v>
       </c>
       <c r="B2090" s="3" t="s">
-        <v>5889</v>
+        <v>5888</v>
       </c>
       <c r="C2090" s="3" t="s">
         <v>3</v>
@@ -53921,7 +53921,7 @@
         <v>1123804</v>
       </c>
       <c r="B2097" s="3" t="s">
-        <v>5583</v>
+        <v>5582</v>
       </c>
       <c r="C2097" s="3" t="s">
         <v>3</v>
@@ -54040,7 +54040,7 @@
         <v>1128085</v>
       </c>
       <c r="B2104" s="3" t="s">
-        <v>5584</v>
+        <v>5583</v>
       </c>
       <c r="C2104" s="3" t="s">
         <v>3</v>
@@ -54057,7 +54057,7 @@
         <v>1128680</v>
       </c>
       <c r="B2105" s="3" t="s">
-        <v>5890</v>
+        <v>5889</v>
       </c>
       <c r="C2105" s="3" t="s">
         <v>3</v>
@@ -54142,7 +54142,7 @@
         <v>1131013</v>
       </c>
       <c r="B2110" s="3" t="s">
-        <v>5891</v>
+        <v>5890</v>
       </c>
       <c r="C2110" s="3" t="s">
         <v>3</v>
@@ -54176,7 +54176,7 @@
         <v>1133475</v>
       </c>
       <c r="B2112" s="3" t="s">
-        <v>5585</v>
+        <v>5584</v>
       </c>
       <c r="C2112" s="3" t="s">
         <v>3</v>
@@ -54312,7 +54312,7 @@
         <v>1140377</v>
       </c>
       <c r="B2120" s="3" t="s">
-        <v>5586</v>
+        <v>5585</v>
       </c>
       <c r="C2120" s="3" t="s">
         <v>3</v>
@@ -54397,7 +54397,7 @@
         <v>1143864</v>
       </c>
       <c r="B2125" s="3" t="s">
-        <v>5892</v>
+        <v>5891</v>
       </c>
       <c r="C2125" s="3" t="s">
         <v>3</v>
@@ -54550,7 +54550,7 @@
         <v>1151083</v>
       </c>
       <c r="B2134" s="3" t="s">
-        <v>5587</v>
+        <v>5586</v>
       </c>
       <c r="C2134" s="3" t="s">
         <v>3</v>
@@ -54992,7 +54992,7 @@
         <v>1197166</v>
       </c>
       <c r="B2160" s="3" t="s">
-        <v>5588</v>
+        <v>5587</v>
       </c>
       <c r="C2160" s="3" t="s">
         <v>3</v>
@@ -55026,7 +55026,7 @@
         <v>1199451</v>
       </c>
       <c r="B2162" s="3" t="s">
-        <v>5893</v>
+        <v>5892</v>
       </c>
       <c r="C2162" s="3" t="s">
         <v>3</v>
@@ -55213,7 +55213,7 @@
         <v>1204446</v>
       </c>
       <c r="B2173" s="3" t="s">
-        <v>5589</v>
+        <v>5588</v>
       </c>
       <c r="C2173" s="3" t="s">
         <v>3</v>
@@ -55298,7 +55298,7 @@
         <v>1208680</v>
       </c>
       <c r="B2178" s="3" t="s">
-        <v>5590</v>
+        <v>5589</v>
       </c>
       <c r="C2178" s="3" t="s">
         <v>3</v>
@@ -55434,7 +55434,7 @@
         <v>1217078</v>
       </c>
       <c r="B2186" s="3" t="s">
-        <v>5894</v>
+        <v>5893</v>
       </c>
       <c r="C2186" s="3" t="s">
         <v>3</v>
@@ -55451,7 +55451,7 @@
         <v>1218167</v>
       </c>
       <c r="B2187" s="3" t="s">
-        <v>5591</v>
+        <v>5590</v>
       </c>
       <c r="C2187" s="3" t="s">
         <v>3</v>
@@ -55468,7 +55468,7 @@
         <v>1218658</v>
       </c>
       <c r="B2188" s="3" t="s">
-        <v>5592</v>
+        <v>5591</v>
       </c>
       <c r="C2188" s="3" t="s">
         <v>3</v>
@@ -55502,7 +55502,7 @@
         <v>1219803</v>
       </c>
       <c r="B2190" s="3" t="s">
-        <v>5895</v>
+        <v>5894</v>
       </c>
       <c r="C2190" s="3" t="s">
         <v>3</v>
@@ -55570,7 +55570,7 @@
         <v>1225266</v>
       </c>
       <c r="B2194" s="3" t="s">
-        <v>5896</v>
+        <v>5895</v>
       </c>
       <c r="C2194" s="3" t="s">
         <v>3</v>
@@ -55706,7 +55706,7 @@
         <v>1236427</v>
       </c>
       <c r="B2202" s="3" t="s">
-        <v>5897</v>
+        <v>5896</v>
       </c>
       <c r="C2202" s="3" t="s">
         <v>3</v>
@@ -55740,7 +55740,7 @@
         <v>1239005</v>
       </c>
       <c r="B2204" s="3" t="s">
-        <v>5898</v>
+        <v>5897</v>
       </c>
       <c r="C2204" s="3" t="s">
         <v>3</v>
@@ -55893,7 +55893,7 @@
         <v>1245373</v>
       </c>
       <c r="B2213" s="3" t="s">
-        <v>5899</v>
+        <v>5898</v>
       </c>
       <c r="C2213" s="3" t="s">
         <v>3</v>
@@ -55910,7 +55910,7 @@
         <v>1246547</v>
       </c>
       <c r="B2214" s="3" t="s">
-        <v>5900</v>
+        <v>5899</v>
       </c>
       <c r="C2214" s="3" t="s">
         <v>3</v>
@@ -55995,7 +55995,7 @@
         <v>1253912</v>
       </c>
       <c r="B2219" s="3" t="s">
-        <v>5593</v>
+        <v>5592</v>
       </c>
       <c r="C2219" s="3" t="s">
         <v>3</v>
@@ -56097,7 +56097,7 @@
         <v>1257253</v>
       </c>
       <c r="B2225" s="3" t="s">
-        <v>5901</v>
+        <v>5900</v>
       </c>
       <c r="C2225" s="3" t="s">
         <v>3</v>
@@ -56165,7 +56165,7 @@
         <v>1260769</v>
       </c>
       <c r="B2229" s="3" t="s">
-        <v>5902</v>
+        <v>5901</v>
       </c>
       <c r="C2229" s="3" t="s">
         <v>3</v>
@@ -56199,7 +56199,7 @@
         <v>1261859</v>
       </c>
       <c r="B2231" s="3" t="s">
-        <v>5594</v>
+        <v>5593</v>
       </c>
       <c r="C2231" s="3" t="s">
         <v>3</v>
@@ -56318,7 +56318,7 @@
         <v>1274405</v>
       </c>
       <c r="B2238" s="3" t="s">
-        <v>5903</v>
+        <v>5902</v>
       </c>
       <c r="C2238" s="3" t="s">
         <v>3</v>
@@ -56454,7 +56454,7 @@
         <v>1285695</v>
       </c>
       <c r="B2246" s="3" t="s">
-        <v>5595</v>
+        <v>5594</v>
       </c>
       <c r="C2246" s="3" t="s">
         <v>3</v>
@@ -56675,7 +56675,7 @@
         <v>1304324</v>
       </c>
       <c r="B2259" s="3" t="s">
-        <v>5596</v>
+        <v>5595</v>
       </c>
       <c r="C2259" s="3" t="s">
         <v>3</v>
@@ -56828,7 +56828,7 @@
         <v>1312513</v>
       </c>
       <c r="B2268" s="3" t="s">
-        <v>5904</v>
+        <v>5903</v>
       </c>
       <c r="C2268" s="3" t="s">
         <v>3</v>
@@ -56845,7 +56845,7 @@
         <v>1312635</v>
       </c>
       <c r="B2269" s="3" t="s">
-        <v>5597</v>
+        <v>5596</v>
       </c>
       <c r="C2269" s="3" t="s">
         <v>3</v>
@@ -56896,7 +56896,7 @@
         <v>1317946</v>
       </c>
       <c r="B2272" s="3" t="s">
-        <v>5598</v>
+        <v>5597</v>
       </c>
       <c r="C2272" s="3" t="s">
         <v>3</v>
@@ -57100,7 +57100,7 @@
         <v>1335418</v>
       </c>
       <c r="B2284" s="3" t="s">
-        <v>5599</v>
+        <v>5598</v>
       </c>
       <c r="C2284" s="3" t="s">
         <v>3</v>
@@ -57134,7 +57134,7 @@
         <v>1336417</v>
       </c>
       <c r="B2286" s="3" t="s">
-        <v>5905</v>
+        <v>5904</v>
       </c>
       <c r="C2286" s="3" t="s">
         <v>3</v>
@@ -57372,7 +57372,7 @@
         <v>1350483</v>
       </c>
       <c r="B2300" s="3" t="s">
-        <v>5600</v>
+        <v>5599</v>
       </c>
       <c r="C2300" s="3" t="s">
         <v>3</v>
@@ -57406,7 +57406,7 @@
         <v>1351666</v>
       </c>
       <c r="B2302" s="3" t="s">
-        <v>5601</v>
+        <v>5600</v>
       </c>
       <c r="C2302" s="3" t="s">
         <v>3</v>
@@ -57763,7 +57763,7 @@
         <v>1385822</v>
       </c>
       <c r="B2323" s="3" t="s">
-        <v>5906</v>
+        <v>5905</v>
       </c>
       <c r="C2323" s="3" t="s">
         <v>3</v>
@@ -57848,7 +57848,7 @@
         <v>1390207</v>
       </c>
       <c r="B2328" s="3" t="s">
-        <v>5602</v>
+        <v>5601</v>
       </c>
       <c r="C2328" s="3" t="s">
         <v>3</v>
@@ -57967,7 +57967,7 @@
         <v>1397375</v>
       </c>
       <c r="B2335" s="3" t="s">
-        <v>5907</v>
+        <v>5906</v>
       </c>
       <c r="C2335" s="3" t="s">
         <v>3</v>
@@ -58086,7 +58086,7 @@
         <v>1409685</v>
       </c>
       <c r="B2342" s="3" t="s">
-        <v>5603</v>
+        <v>5602</v>
       </c>
       <c r="C2342" s="3" t="s">
         <v>3</v>
@@ -58239,7 +58239,7 @@
         <v>1419661</v>
       </c>
       <c r="B2351" s="3" t="s">
-        <v>5604</v>
+        <v>5603</v>
       </c>
       <c r="C2351" s="3" t="s">
         <v>3</v>
@@ -58324,7 +58324,7 @@
         <v>1422247</v>
       </c>
       <c r="B2356" s="3" t="s">
-        <v>5605</v>
+        <v>5604</v>
       </c>
       <c r="C2356" s="3" t="s">
         <v>3</v>
@@ -58375,7 +58375,7 @@
         <v>1422846</v>
       </c>
       <c r="B2359" s="3" t="s">
-        <v>5908</v>
+        <v>5907</v>
       </c>
       <c r="C2359" s="3" t="s">
         <v>3</v>
@@ -58409,7 +58409,7 @@
         <v>1423880</v>
       </c>
       <c r="B2361" s="3" t="s">
-        <v>5606</v>
+        <v>5605</v>
       </c>
       <c r="C2361" s="3" t="s">
         <v>3</v>
@@ -58562,7 +58562,7 @@
         <v>1429968</v>
       </c>
       <c r="B2370" s="3" t="s">
-        <v>5607</v>
+        <v>5606</v>
       </c>
       <c r="C2370" s="3" t="s">
         <v>3</v>
@@ -58715,7 +58715,7 @@
         <v>1442654</v>
       </c>
       <c r="B2379" s="3" t="s">
-        <v>5909</v>
+        <v>5908</v>
       </c>
       <c r="C2379" s="3" t="s">
         <v>3</v>
@@ -58766,7 +58766,7 @@
         <v>1447752</v>
       </c>
       <c r="B2382" s="3" t="s">
-        <v>5910</v>
+        <v>5909</v>
       </c>
       <c r="C2382" s="3" t="s">
         <v>3</v>
@@ -58868,7 +58868,7 @@
         <v>1452913</v>
       </c>
       <c r="B2388" s="3" t="s">
-        <v>5608</v>
+        <v>5607</v>
       </c>
       <c r="C2388" s="3" t="s">
         <v>3</v>
@@ -59038,7 +59038,7 @@
         <v>1465959</v>
       </c>
       <c r="B2398" s="3" t="s">
-        <v>5609</v>
+        <v>5608</v>
       </c>
       <c r="C2398" s="3" t="s">
         <v>3</v>
@@ -59157,7 +59157,7 @@
         <v>1474089</v>
       </c>
       <c r="B2405" s="3" t="s">
-        <v>5610</v>
+        <v>5609</v>
       </c>
       <c r="C2405" s="3" t="s">
         <v>3</v>
@@ -59344,7 +59344,7 @@
         <v>1481741</v>
       </c>
       <c r="B2416" s="3" t="s">
-        <v>5911</v>
+        <v>5910</v>
       </c>
       <c r="C2416" s="3" t="s">
         <v>3</v>
@@ -59378,7 +59378,7 @@
         <v>1482046</v>
       </c>
       <c r="B2418" s="3" t="s">
-        <v>5611</v>
+        <v>5610</v>
       </c>
       <c r="C2418" s="3" t="s">
         <v>3</v>
@@ -59667,7 +59667,7 @@
         <v>1516688</v>
       </c>
       <c r="B2435" s="3" t="s">
-        <v>5612</v>
+        <v>5611</v>
       </c>
       <c r="C2435" s="3" t="s">
         <v>3</v>
@@ -59701,7 +59701,7 @@
         <v>1516796</v>
       </c>
       <c r="B2437" s="3" t="s">
-        <v>5613</v>
+        <v>5612</v>
       </c>
       <c r="C2437" s="3" t="s">
         <v>3</v>
@@ -59718,7 +59718,7 @@
         <v>1517415</v>
       </c>
       <c r="B2438" s="3" t="s">
-        <v>5614</v>
+        <v>5613</v>
       </c>
       <c r="C2438" s="3" t="s">
         <v>3</v>
@@ -59769,7 +59769,7 @@
         <v>1522681</v>
       </c>
       <c r="B2441" s="3" t="s">
-        <v>5615</v>
+        <v>5614</v>
       </c>
       <c r="C2441" s="3" t="s">
         <v>3</v>
@@ -59939,7 +59939,7 @@
         <v>1530118</v>
       </c>
       <c r="B2451" s="3" t="s">
-        <v>5912</v>
+        <v>5911</v>
       </c>
       <c r="C2451" s="3" t="s">
         <v>3</v>
@@ -60296,7 +60296,7 @@
         <v>1563243</v>
       </c>
       <c r="B2472" s="3" t="s">
-        <v>5913</v>
+        <v>5912</v>
       </c>
       <c r="C2472" s="3" t="s">
         <v>3</v>
@@ -60517,7 +60517,7 @@
         <v>1578153</v>
       </c>
       <c r="B2485" s="3" t="s">
-        <v>5914</v>
+        <v>5913</v>
       </c>
       <c r="C2485" s="3" t="s">
         <v>3</v>
@@ -60534,7 +60534,7 @@
         <v>1578200</v>
       </c>
       <c r="B2486" s="3" t="s">
-        <v>5616</v>
+        <v>5615</v>
       </c>
       <c r="C2486" s="3" t="s">
         <v>3</v>
@@ -60568,7 +60568,7 @@
         <v>1583807</v>
       </c>
       <c r="B2488" s="3" t="s">
-        <v>5617</v>
+        <v>5616</v>
       </c>
       <c r="C2488" s="3" t="s">
         <v>3</v>
@@ -60738,7 +60738,7 @@
         <v>1593477</v>
       </c>
       <c r="B2498" s="3" t="s">
-        <v>5915</v>
+        <v>5914</v>
       </c>
       <c r="C2498" s="3" t="s">
         <v>3</v>
@@ -60925,7 +60925,7 @@
         <v>1603362</v>
       </c>
       <c r="B2509" s="3" t="s">
-        <v>5916</v>
+        <v>5915</v>
       </c>
       <c r="C2509" s="3" t="s">
         <v>3</v>
@@ -60959,7 +60959,7 @@
         <v>1605525</v>
       </c>
       <c r="B2511" s="3" t="s">
-        <v>5917</v>
+        <v>5916</v>
       </c>
       <c r="C2511" s="3" t="s">
         <v>3</v>
@@ -61027,7 +61027,7 @@
         <v>1606578</v>
       </c>
       <c r="B2515" s="3" t="s">
-        <v>5918</v>
+        <v>5917</v>
       </c>
       <c r="C2515" s="3" t="s">
         <v>3</v>
@@ -61112,7 +61112,7 @@
         <v>1608791</v>
       </c>
       <c r="B2520" s="3" t="s">
-        <v>5618</v>
+        <v>5617</v>
       </c>
       <c r="C2520" s="3" t="s">
         <v>3</v>
@@ -61129,7 +61129,7 @@
         <v>1611527</v>
       </c>
       <c r="B2521" s="3" t="s">
-        <v>5619</v>
+        <v>5618</v>
       </c>
       <c r="C2521" s="3" t="s">
         <v>3</v>
@@ -61401,7 +61401,7 @@
         <v>1625129</v>
       </c>
       <c r="B2537" s="3" t="s">
-        <v>5620</v>
+        <v>5619</v>
       </c>
       <c r="C2537" s="3" t="s">
         <v>3</v>
@@ -61996,7 +61996,7 @@
         <v>1657935</v>
       </c>
       <c r="B2572" s="3" t="s">
-        <v>5621</v>
+        <v>5620</v>
       </c>
       <c r="C2572" s="3" t="s">
         <v>3</v>
@@ -62132,7 +62132,7 @@
         <v>1665231</v>
       </c>
       <c r="B2580" s="3" t="s">
-        <v>5622</v>
+        <v>5621</v>
       </c>
       <c r="C2580" s="3" t="s">
         <v>3</v>
@@ -62234,7 +62234,7 @@
         <v>1671262</v>
       </c>
       <c r="B2586" s="3" t="s">
-        <v>5919</v>
+        <v>5918</v>
       </c>
       <c r="C2586" s="3" t="s">
         <v>3</v>
@@ -62659,7 +62659,7 @@
         <v>1699443</v>
       </c>
       <c r="B2611" s="3" t="s">
-        <v>5920</v>
+        <v>5919</v>
       </c>
       <c r="C2611" s="3" t="s">
         <v>3</v>
@@ -62727,7 +62727,7 @@
         <v>1701693</v>
       </c>
       <c r="B2615" s="3" t="s">
-        <v>5623</v>
+        <v>5622</v>
       </c>
       <c r="C2615" s="3" t="s">
         <v>3</v>
@@ -62778,7 +62778,7 @@
         <v>1707533</v>
       </c>
       <c r="B2618" s="3" t="s">
-        <v>5921</v>
+        <v>5920</v>
       </c>
       <c r="C2618" s="3" t="s">
         <v>3</v>
@@ -62795,7 +62795,7 @@
         <v>1709011</v>
       </c>
       <c r="B2619" s="3" t="s">
-        <v>5922</v>
+        <v>5921</v>
       </c>
       <c r="C2619" s="3" t="s">
         <v>3</v>
@@ -62812,7 +62812,7 @@
         <v>1709744</v>
       </c>
       <c r="B2620" s="3" t="s">
-        <v>5624</v>
+        <v>5623</v>
       </c>
       <c r="C2620" s="3" t="s">
         <v>3</v>
@@ -62880,7 +62880,7 @@
         <v>1713978</v>
       </c>
       <c r="B2624" s="3" t="s">
-        <v>5625</v>
+        <v>5624</v>
       </c>
       <c r="C2624" s="3" t="s">
         <v>3</v>
@@ -62999,7 +62999,7 @@
         <v>1716746</v>
       </c>
       <c r="B2631" s="3" t="s">
-        <v>5923</v>
+        <v>5922</v>
       </c>
       <c r="C2631" s="3" t="s">
         <v>3</v>
@@ -63254,7 +63254,7 @@
         <v>1730428</v>
       </c>
       <c r="B2646" s="3" t="s">
-        <v>5626</v>
+        <v>5625</v>
       </c>
       <c r="C2646" s="3" t="s">
         <v>3</v>
@@ -63526,7 +63526,7 @@
         <v>1741495</v>
       </c>
       <c r="B2662" s="3" t="s">
-        <v>5627</v>
+        <v>5626</v>
       </c>
       <c r="C2662" s="3" t="s">
         <v>3</v>
@@ -63713,7 +63713,7 @@
         <v>1760183</v>
       </c>
       <c r="B2673" s="3" t="s">
-        <v>5628</v>
+        <v>5627</v>
       </c>
       <c r="C2673" s="3" t="s">
         <v>3</v>
@@ -63832,7 +63832,7 @@
         <v>1774566</v>
       </c>
       <c r="B2680" s="3" t="s">
-        <v>5924</v>
+        <v>5923</v>
       </c>
       <c r="C2680" s="3" t="s">
         <v>3</v>
@@ -63951,7 +63951,7 @@
         <v>1784838</v>
       </c>
       <c r="B2687" s="3" t="s">
-        <v>5629</v>
+        <v>5628</v>
       </c>
       <c r="C2687" s="3" t="s">
         <v>3</v>
@@ -63968,7 +63968,7 @@
         <v>1785221</v>
       </c>
       <c r="B2688" s="3" t="s">
-        <v>5630</v>
+        <v>5629</v>
       </c>
       <c r="C2688" s="3" t="s">
         <v>3</v>
@@ -64002,7 +64002,7 @@
         <v>1788095</v>
       </c>
       <c r="B2690" s="3" t="s">
-        <v>5925</v>
+        <v>5924</v>
       </c>
       <c r="C2690" s="3" t="s">
         <v>3</v>
@@ -64019,7 +64019,7 @@
         <v>1788387</v>
       </c>
       <c r="B2691" s="3" t="s">
-        <v>5631</v>
+        <v>5630</v>
       </c>
       <c r="C2691" s="3" t="s">
         <v>3</v>
@@ -64274,7 +64274,7 @@
         <v>1799298</v>
       </c>
       <c r="B2706" s="3" t="s">
-        <v>5926</v>
+        <v>5925</v>
       </c>
       <c r="C2706" s="3" t="s">
         <v>3</v>
@@ -64461,7 +64461,7 @@
         <v>1817438</v>
       </c>
       <c r="B2717" s="3" t="s">
-        <v>5632</v>
+        <v>5631</v>
       </c>
       <c r="C2717" s="3" t="s">
         <v>3</v>
@@ -64495,7 +64495,7 @@
         <v>1824240</v>
       </c>
       <c r="B2719" s="3" t="s">
-        <v>5927</v>
+        <v>5926</v>
       </c>
       <c r="C2719" s="3" t="s">
         <v>3</v>
@@ -64512,7 +64512,7 @@
         <v>1828587</v>
       </c>
       <c r="B2720" s="3" t="s">
-        <v>5928</v>
+        <v>5927</v>
       </c>
       <c r="C2720" s="3" t="s">
         <v>3</v>
@@ -64580,7 +64580,7 @@
         <v>1836903</v>
       </c>
       <c r="B2724" s="3" t="s">
-        <v>5929</v>
+        <v>5928</v>
       </c>
       <c r="C2724" s="3" t="s">
         <v>3</v>
@@ -64954,7 +64954,7 @@
         <v>1853556</v>
       </c>
       <c r="B2746" s="3" t="s">
-        <v>5633</v>
+        <v>5632</v>
       </c>
       <c r="C2746" s="3" t="s">
         <v>3</v>
@@ -65107,7 +65107,7 @@
         <v>1864820</v>
       </c>
       <c r="B2755" s="3" t="s">
-        <v>5634</v>
+        <v>5633</v>
       </c>
       <c r="C2755" s="3" t="s">
         <v>3</v>
@@ -65141,7 +65141,7 @@
         <v>1871096</v>
       </c>
       <c r="B2757" s="3" t="s">
-        <v>5635</v>
+        <v>5634</v>
       </c>
       <c r="C2757" s="3" t="s">
         <v>3</v>
@@ -65192,7 +65192,7 @@
         <v>1876106</v>
       </c>
       <c r="B2760" s="3" t="s">
-        <v>5636</v>
+        <v>5635</v>
       </c>
       <c r="C2760" s="3" t="s">
         <v>3</v>
@@ -65226,7 +65226,7 @@
         <v>1877654</v>
       </c>
       <c r="B2762" s="3" t="s">
-        <v>5637</v>
+        <v>5636</v>
       </c>
       <c r="C2762" s="3" t="s">
         <v>3</v>
@@ -65277,7 +65277,7 @@
         <v>1885837</v>
       </c>
       <c r="B2765" s="3" t="s">
-        <v>5638</v>
+        <v>5637</v>
       </c>
       <c r="C2765" s="3" t="s">
         <v>3</v>
@@ -65413,7 +65413,7 @@
         <v>1894218</v>
       </c>
       <c r="B2773" s="3" t="s">
-        <v>5639</v>
+        <v>5638</v>
       </c>
       <c r="C2773" s="3" t="s">
         <v>3</v>
@@ -65464,7 +65464,7 @@
         <v>1897397</v>
       </c>
       <c r="B2776" s="3" t="s">
-        <v>5640</v>
+        <v>5639</v>
       </c>
       <c r="C2776" s="3" t="s">
         <v>3</v>
@@ -65532,7 +65532,7 @@
         <v>1902089</v>
       </c>
       <c r="B2780" s="3" t="s">
-        <v>5641</v>
+        <v>5640</v>
       </c>
       <c r="C2780" s="3" t="s">
         <v>3</v>
@@ -65617,7 +65617,7 @@
         <v>1912440</v>
       </c>
       <c r="B2785" s="3" t="s">
-        <v>5642</v>
+        <v>5641</v>
       </c>
       <c r="C2785" s="3" t="s">
         <v>3</v>
@@ -65719,7 +65719,7 @@
         <v>1922769</v>
       </c>
       <c r="B2791" s="3" t="s">
-        <v>5930</v>
+        <v>5929</v>
       </c>
       <c r="C2791" s="3" t="s">
         <v>3</v>
@@ -65753,7 +65753,7 @@
         <v>1924572</v>
       </c>
       <c r="B2793" s="3" t="s">
-        <v>5643</v>
+        <v>5642</v>
       </c>
       <c r="C2793" s="3" t="s">
         <v>3</v>
@@ -65770,7 +65770,7 @@
         <v>1925698</v>
       </c>
       <c r="B2794" s="3" t="s">
-        <v>5931</v>
+        <v>5930</v>
       </c>
       <c r="C2794" s="3" t="s">
         <v>3</v>
@@ -65991,7 +65991,7 @@
         <v>1936005</v>
       </c>
       <c r="B2807" s="3" t="s">
-        <v>5932</v>
+        <v>5931</v>
       </c>
       <c r="C2807" s="3" t="s">
         <v>3</v>
@@ -66008,7 +66008,7 @@
         <v>1936921</v>
       </c>
       <c r="B2808" s="3" t="s">
-        <v>5644</v>
+        <v>5643</v>
       </c>
       <c r="C2808" s="3" t="s">
         <v>3</v>
@@ -66144,7 +66144,7 @@
         <v>1945526</v>
       </c>
       <c r="B2816" s="3" t="s">
-        <v>5645</v>
+        <v>5644</v>
       </c>
       <c r="C2816" s="3" t="s">
         <v>3</v>
@@ -66161,7 +66161,7 @@
         <v>1945782</v>
       </c>
       <c r="B2817" s="3" t="s">
-        <v>5646</v>
+        <v>5645</v>
       </c>
       <c r="C2817" s="3" t="s">
         <v>3</v>
@@ -66212,7 +66212,7 @@
         <v>1947939</v>
       </c>
       <c r="B2820" s="3" t="s">
-        <v>5933</v>
+        <v>5932</v>
       </c>
       <c r="C2820" s="3" t="s">
         <v>3</v>
@@ -66229,7 +66229,7 @@
         <v>1948863</v>
       </c>
       <c r="B2821" s="3" t="s">
-        <v>5934</v>
+        <v>5933</v>
       </c>
       <c r="C2821" s="3" t="s">
         <v>3</v>
@@ -66246,7 +66246,7 @@
         <v>1949059</v>
       </c>
       <c r="B2822" s="3" t="s">
-        <v>5647</v>
+        <v>5646</v>
       </c>
       <c r="C2822" s="3" t="s">
         <v>3</v>
@@ -66569,7 +66569,7 @@
         <v>1968563</v>
       </c>
       <c r="B2841" s="3" t="s">
-        <v>5648</v>
+        <v>5647</v>
       </c>
       <c r="C2841" s="3" t="s">
         <v>3</v>
@@ -66603,7 +66603,7 @@
         <v>1970348</v>
       </c>
       <c r="B2843" s="3" t="s">
-        <v>5649</v>
+        <v>5648</v>
       </c>
       <c r="C2843" s="3" t="s">
         <v>3</v>
@@ -66637,7 +66637,7 @@
         <v>1977273</v>
       </c>
       <c r="B2845" s="3" t="s">
-        <v>5935</v>
+        <v>5934</v>
       </c>
       <c r="C2845" s="3" t="s">
         <v>3</v>
@@ -66654,7 +66654,7 @@
         <v>1981639</v>
       </c>
       <c r="B2846" s="3" t="s">
-        <v>5936</v>
+        <v>5935</v>
       </c>
       <c r="C2846" s="3" t="s">
         <v>3</v>
@@ -66841,7 +66841,7 @@
         <v>2004435</v>
       </c>
       <c r="B2857" s="3" t="s">
-        <v>5650</v>
+        <v>5649</v>
       </c>
       <c r="C2857" s="3" t="s">
         <v>3</v>
@@ -66858,7 +66858,7 @@
         <v>2005460</v>
       </c>
       <c r="B2858" s="3" t="s">
-        <v>5651</v>
+        <v>5650</v>
       </c>
       <c r="C2858" s="3" t="s">
         <v>3</v>
@@ -66892,7 +66892,7 @@
         <v>2006759</v>
       </c>
       <c r="B2860" s="3" t="s">
-        <v>5937</v>
+        <v>5936</v>
       </c>
       <c r="C2860" s="3" t="s">
         <v>3</v>
@@ -66926,7 +66926,7 @@
         <v>2007122</v>
       </c>
       <c r="B2862" s="3" t="s">
-        <v>5652</v>
+        <v>5651</v>
       </c>
       <c r="C2862" s="3" t="s">
         <v>3</v>
@@ -67045,7 +67045,7 @@
         <v>2015755</v>
       </c>
       <c r="B2869" s="3" t="s">
-        <v>5653</v>
+        <v>5652</v>
       </c>
       <c r="C2869" s="3" t="s">
         <v>3</v>
@@ -67232,7 +67232,7 @@
         <v>2031153</v>
       </c>
       <c r="B2880" s="3" t="s">
-        <v>5938</v>
+        <v>5937</v>
       </c>
       <c r="C2880" s="3" t="s">
         <v>3</v>
@@ -67317,7 +67317,7 @@
         <v>2035055</v>
       </c>
       <c r="B2885" s="3" t="s">
-        <v>5654</v>
+        <v>5653</v>
       </c>
       <c r="C2885" s="3" t="s">
         <v>3</v>
@@ -67368,7 +67368,7 @@
         <v>2039927</v>
       </c>
       <c r="B2888" s="3" t="s">
-        <v>5655</v>
+        <v>5654</v>
       </c>
       <c r="C2888" s="3" t="s">
         <v>3</v>
@@ -67844,7 +67844,7 @@
         <v>2067751</v>
       </c>
       <c r="B2916" s="3" t="s">
-        <v>5656</v>
+        <v>5655</v>
       </c>
       <c r="C2916" s="3" t="s">
         <v>3</v>
@@ -67912,7 +67912,7 @@
         <v>2071331</v>
       </c>
       <c r="B2920" s="3" t="s">
-        <v>5657</v>
+        <v>5656</v>
       </c>
       <c r="C2920" s="3" t="s">
         <v>3</v>
@@ -67946,7 +67946,7 @@
         <v>2072627</v>
       </c>
       <c r="B2922" s="3" t="s">
-        <v>5939</v>
+        <v>5938</v>
       </c>
       <c r="C2922" s="3" t="s">
         <v>3</v>
@@ -67980,7 +67980,7 @@
         <v>2078387</v>
       </c>
       <c r="B2924" s="3" t="s">
-        <v>5658</v>
+        <v>5657</v>
       </c>
       <c r="C2924" s="3" t="s">
         <v>3</v>
@@ -67997,7 +67997,7 @@
         <v>2079588</v>
       </c>
       <c r="B2925" s="3" t="s">
-        <v>5940</v>
+        <v>5939</v>
       </c>
       <c r="C2925" s="3" t="s">
         <v>3</v>
@@ -68031,7 +68031,7 @@
         <v>2082859</v>
       </c>
       <c r="B2927" s="3" t="s">
-        <v>5941</v>
+        <v>5940</v>
       </c>
       <c r="C2927" s="3" t="s">
         <v>3</v>
@@ -68269,7 +68269,7 @@
         <v>2093311</v>
       </c>
       <c r="B2941" s="3" t="s">
-        <v>5659</v>
+        <v>5658</v>
       </c>
       <c r="C2941" s="3" t="s">
         <v>3</v>
@@ -68473,7 +68473,7 @@
         <v>2102652</v>
       </c>
       <c r="B2953" s="3" t="s">
-        <v>5660</v>
+        <v>5659</v>
       </c>
       <c r="C2953" s="3" t="s">
         <v>3</v>
@@ -68507,7 +68507,7 @@
         <v>2102961</v>
       </c>
       <c r="B2955" s="3" t="s">
-        <v>5661</v>
+        <v>5660</v>
       </c>
       <c r="C2955" s="3" t="s">
         <v>3</v>
@@ -68541,7 +68541,7 @@
         <v>2107643</v>
       </c>
       <c r="B2957" s="3" t="s">
-        <v>5942</v>
+        <v>5941</v>
       </c>
       <c r="C2957" s="3" t="s">
         <v>3</v>
@@ -68711,7 +68711,7 @@
         <v>2118160</v>
       </c>
       <c r="B2967" s="3" t="s">
-        <v>5662</v>
+        <v>5661</v>
       </c>
       <c r="C2967" s="3" t="s">
         <v>3</v>
@@ -68728,7 +68728,7 @@
         <v>2120883</v>
       </c>
       <c r="B2968" s="3" t="s">
-        <v>5663</v>
+        <v>5662</v>
       </c>
       <c r="C2968" s="3" t="s">
         <v>3</v>
@@ -68830,7 +68830,7 @@
         <v>2124341</v>
       </c>
       <c r="B2974" s="3" t="s">
-        <v>5664</v>
+        <v>5663</v>
       </c>
       <c r="C2974" s="3" t="s">
         <v>3</v>

</xml_diff>

<commit_message>
--CAMBIOS EN LOS EXPORTADORES DE EXCEL PARA QUE SE ADECUEN A LA IMPLEMENTACION DEL CONVERSOR DE TIPOS DE EXCEL
</commit_message>
<xml_diff>
--- a/Control de Facturas/Assets/Plantillas/BENEFICIARIOS AGUA, GAS Y LUZ.xlsx
+++ b/Control de Facturas/Assets/Plantillas/BENEFICIARIOS AGUA, GAS Y LUZ.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Programa Servicios Basicos\Control de Facturas\Assets\Plantillas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0EABAC1B-E0EE-475C-A16F-ACEF90B62114}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D01BC49-F234-4406-9097-3601DBFC5031}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{82731452-31CB-4A50-BC16-E3FD7323D481}"/>
   </bookViews>
@@ -17281,9 +17281,6 @@
     <t>COOP.DEPROVISION,OBRASYSERVICIOSPUBLICOSLAGUNAPAIVA</t>
   </si>
   <si>
-    <t>COOPICOOPERATIVAINTEGRALREGIONALDEPROVISIONDESERVICIOSSOCIALESYPUBLICOS,OBRAS,PRODUCCION</t>
-  </si>
-  <si>
     <t>ENTEMUNICIPALAGUASDETRASLASIERRA</t>
   </si>
   <si>
@@ -17879,6 +17876,9 @@
   </si>
   <si>
     <t>EPE</t>
+  </si>
+  <si>
+    <t>LA COOPI</t>
   </si>
 </sst>
 </file>
@@ -18479,7 +18479,7 @@
         <v>1357</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>5942</v>
+        <v>5941</v>
       </c>
       <c r="C12" s="3" t="s">
         <v>3</v>
@@ -18496,7 +18496,7 @@
         <v>1361</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>5949</v>
+        <v>5948</v>
       </c>
       <c r="C13" s="3" t="s">
         <v>3</v>
@@ -21454,7 +21454,7 @@
         <v>14626</v>
       </c>
       <c r="B187" s="5" t="s">
-        <v>5946</v>
+        <v>5945</v>
       </c>
       <c r="C187" s="3" t="s">
         <v>3</v>
@@ -23545,7 +23545,7 @@
         <v>67354</v>
       </c>
       <c r="B310" s="5" t="s">
-        <v>5948</v>
+        <v>5947</v>
       </c>
       <c r="C310" s="3" t="s">
         <v>3</v>
@@ -23562,7 +23562,7 @@
         <v>67776</v>
       </c>
       <c r="B311" s="5" t="s">
-        <v>5944</v>
+        <v>5943</v>
       </c>
       <c r="C311" s="3" t="s">
         <v>3</v>
@@ -25874,7 +25874,7 @@
         <v>127673</v>
       </c>
       <c r="B447" s="5" t="s">
-        <v>5943</v>
+        <v>5942</v>
       </c>
       <c r="C447" s="3" t="s">
         <v>3</v>
@@ -30072,8 +30072,8 @@
       <c r="A694" s="2">
         <v>260696</v>
       </c>
-      <c r="B694" s="3" t="s">
-        <v>5750</v>
+      <c r="B694" s="5" t="s">
+        <v>5949</v>
       </c>
       <c r="C694" s="3" t="s">
         <v>3</v>
@@ -30158,7 +30158,7 @@
         <v>262595</v>
       </c>
       <c r="B699" s="3" t="s">
-        <v>5751</v>
+        <v>5750</v>
       </c>
       <c r="C699" s="3" t="s">
         <v>3</v>
@@ -30209,7 +30209,7 @@
         <v>262648</v>
       </c>
       <c r="B702" s="3" t="s">
-        <v>5752</v>
+        <v>5751</v>
       </c>
       <c r="C702" s="3" t="s">
         <v>3</v>
@@ -30328,7 +30328,7 @@
         <v>269554</v>
       </c>
       <c r="B709" s="3" t="s">
-        <v>5753</v>
+        <v>5752</v>
       </c>
       <c r="C709" s="3" t="s">
         <v>3</v>
@@ -30515,7 +30515,7 @@
         <v>276933</v>
       </c>
       <c r="B720" s="3" t="s">
-        <v>5754</v>
+        <v>5753</v>
       </c>
       <c r="C720" s="3" t="s">
         <v>3</v>
@@ -30583,7 +30583,7 @@
         <v>278058</v>
       </c>
       <c r="B724" s="3" t="s">
-        <v>5755</v>
+        <v>5754</v>
       </c>
       <c r="C724" s="3" t="s">
         <v>3</v>
@@ -30651,7 +30651,7 @@
         <v>281556</v>
       </c>
       <c r="B728" s="3" t="s">
-        <v>5756</v>
+        <v>5755</v>
       </c>
       <c r="C728" s="3" t="s">
         <v>3</v>
@@ -30736,7 +30736,7 @@
         <v>285507</v>
       </c>
       <c r="B733" s="3" t="s">
-        <v>5757</v>
+        <v>5756</v>
       </c>
       <c r="C733" s="3" t="s">
         <v>3</v>
@@ -30821,7 +30821,7 @@
         <v>287851</v>
       </c>
       <c r="B738" s="3" t="s">
-        <v>5758</v>
+        <v>5757</v>
       </c>
       <c r="C738" s="3" t="s">
         <v>3</v>
@@ -30957,7 +30957,7 @@
         <v>291978</v>
       </c>
       <c r="B746" s="3" t="s">
-        <v>5759</v>
+        <v>5758</v>
       </c>
       <c r="C746" s="3" t="s">
         <v>3</v>
@@ -30991,7 +30991,7 @@
         <v>295086</v>
       </c>
       <c r="B748" s="3" t="s">
-        <v>5760</v>
+        <v>5759</v>
       </c>
       <c r="C748" s="3" t="s">
         <v>3</v>
@@ -31008,7 +31008,7 @@
         <v>297792</v>
       </c>
       <c r="B749" s="3" t="s">
-        <v>5761</v>
+        <v>5760</v>
       </c>
       <c r="C749" s="3" t="s">
         <v>3</v>
@@ -31025,7 +31025,7 @@
         <v>298556</v>
       </c>
       <c r="B750" s="3" t="s">
-        <v>5762</v>
+        <v>5761</v>
       </c>
       <c r="C750" s="3" t="s">
         <v>3</v>
@@ -31093,7 +31093,7 @@
         <v>300800</v>
       </c>
       <c r="B754" s="3" t="s">
-        <v>5763</v>
+        <v>5762</v>
       </c>
       <c r="C754" s="3" t="s">
         <v>3</v>
@@ -31110,7 +31110,7 @@
         <v>301705</v>
       </c>
       <c r="B755" s="3" t="s">
-        <v>5764</v>
+        <v>5763</v>
       </c>
       <c r="C755" s="3" t="s">
         <v>3</v>
@@ -31144,7 +31144,7 @@
         <v>307867</v>
       </c>
       <c r="B757" s="3" t="s">
-        <v>5765</v>
+        <v>5764</v>
       </c>
       <c r="C757" s="3" t="s">
         <v>3</v>
@@ -31229,7 +31229,7 @@
         <v>316725</v>
       </c>
       <c r="B762" s="5" t="s">
-        <v>5947</v>
+        <v>5946</v>
       </c>
       <c r="C762" s="3" t="s">
         <v>3</v>
@@ -31399,7 +31399,7 @@
         <v>324503</v>
       </c>
       <c r="B772" s="3" t="s">
-        <v>5766</v>
+        <v>5765</v>
       </c>
       <c r="C772" s="3" t="s">
         <v>3</v>
@@ -31416,7 +31416,7 @@
         <v>324977</v>
       </c>
       <c r="B773" s="3" t="s">
-        <v>5767</v>
+        <v>5766</v>
       </c>
       <c r="C773" s="3" t="s">
         <v>3</v>
@@ -31501,7 +31501,7 @@
         <v>327658</v>
       </c>
       <c r="B778" s="3" t="s">
-        <v>5768</v>
+        <v>5767</v>
       </c>
       <c r="C778" s="3" t="s">
         <v>3</v>
@@ -31518,7 +31518,7 @@
         <v>328124</v>
       </c>
       <c r="B779" s="3" t="s">
-        <v>5769</v>
+        <v>5768</v>
       </c>
       <c r="C779" s="3" t="s">
         <v>3</v>
@@ -31858,7 +31858,7 @@
         <v>343290</v>
       </c>
       <c r="B799" s="3" t="s">
-        <v>5770</v>
+        <v>5769</v>
       </c>
       <c r="C799" s="3" t="s">
         <v>3</v>
@@ -31943,7 +31943,7 @@
         <v>345453</v>
       </c>
       <c r="B804" s="3" t="s">
-        <v>5771</v>
+        <v>5770</v>
       </c>
       <c r="C804" s="3" t="s">
         <v>3</v>
@@ -32028,7 +32028,7 @@
         <v>347739</v>
       </c>
       <c r="B809" s="3" t="s">
-        <v>5772</v>
+        <v>5771</v>
       </c>
       <c r="C809" s="3" t="s">
         <v>3</v>
@@ -32096,7 +32096,7 @@
         <v>350234</v>
       </c>
       <c r="B813" s="3" t="s">
-        <v>5773</v>
+        <v>5772</v>
       </c>
       <c r="C813" s="3" t="s">
         <v>3</v>
@@ -32470,7 +32470,7 @@
         <v>365501</v>
       </c>
       <c r="B835" s="3" t="s">
-        <v>5774</v>
+        <v>5773</v>
       </c>
       <c r="C835" s="3" t="s">
         <v>3</v>
@@ -32742,7 +32742,7 @@
         <v>372272</v>
       </c>
       <c r="B851" s="3" t="s">
-        <v>5775</v>
+        <v>5774</v>
       </c>
       <c r="C851" s="3" t="s">
         <v>3</v>
@@ -32759,7 +32759,7 @@
         <v>372443</v>
       </c>
       <c r="B852" s="3" t="s">
-        <v>5776</v>
+        <v>5775</v>
       </c>
       <c r="C852" s="3" t="s">
         <v>3</v>
@@ -32861,7 +32861,7 @@
         <v>373863</v>
       </c>
       <c r="B858" s="3" t="s">
-        <v>5777</v>
+        <v>5776</v>
       </c>
       <c r="C858" s="3" t="s">
         <v>3</v>
@@ -33116,7 +33116,7 @@
         <v>384192</v>
       </c>
       <c r="B873" s="3" t="s">
-        <v>5778</v>
+        <v>5777</v>
       </c>
       <c r="C873" s="3" t="s">
         <v>3</v>
@@ -33354,7 +33354,7 @@
         <v>389701</v>
       </c>
       <c r="B887" s="3" t="s">
-        <v>5779</v>
+        <v>5778</v>
       </c>
       <c r="C887" s="3" t="s">
         <v>3</v>
@@ -33388,7 +33388,7 @@
         <v>392098</v>
       </c>
       <c r="B889" s="3" t="s">
-        <v>5780</v>
+        <v>5779</v>
       </c>
       <c r="C889" s="3" t="s">
         <v>3</v>
@@ -33473,7 +33473,7 @@
         <v>394655</v>
       </c>
       <c r="B894" s="3" t="s">
-        <v>5781</v>
+        <v>5780</v>
       </c>
       <c r="C894" s="3" t="s">
         <v>3</v>
@@ -33490,7 +33490,7 @@
         <v>394709</v>
       </c>
       <c r="B895" s="3" t="s">
-        <v>5782</v>
+        <v>5781</v>
       </c>
       <c r="C895" s="3" t="s">
         <v>3</v>
@@ -33507,7 +33507,7 @@
         <v>394861</v>
       </c>
       <c r="B896" s="3" t="s">
-        <v>5783</v>
+        <v>5782</v>
       </c>
       <c r="C896" s="3" t="s">
         <v>3</v>
@@ -33541,7 +33541,7 @@
         <v>395525</v>
       </c>
       <c r="B898" s="3" t="s">
-        <v>5784</v>
+        <v>5783</v>
       </c>
       <c r="C898" s="3" t="s">
         <v>3</v>
@@ -33609,7 +33609,7 @@
         <v>397509</v>
       </c>
       <c r="B902" s="3" t="s">
-        <v>5785</v>
+        <v>5784</v>
       </c>
       <c r="C902" s="3" t="s">
         <v>3</v>
@@ -33915,7 +33915,7 @@
         <v>409909</v>
       </c>
       <c r="B920" s="3" t="s">
-        <v>5786</v>
+        <v>5785</v>
       </c>
       <c r="C920" s="3" t="s">
         <v>3</v>
@@ -34153,7 +34153,7 @@
         <v>413789</v>
       </c>
       <c r="B934" s="3" t="s">
-        <v>5787</v>
+        <v>5786</v>
       </c>
       <c r="C934" s="3" t="s">
         <v>3</v>
@@ -34187,7 +34187,7 @@
         <v>415197</v>
       </c>
       <c r="B936" s="3" t="s">
-        <v>5788</v>
+        <v>5787</v>
       </c>
       <c r="C936" s="3" t="s">
         <v>3</v>
@@ -34629,7 +34629,7 @@
         <v>429725</v>
       </c>
       <c r="B962" s="3" t="s">
-        <v>5789</v>
+        <v>5788</v>
       </c>
       <c r="C962" s="3" t="s">
         <v>3</v>
@@ -34714,7 +34714,7 @@
         <v>431885</v>
       </c>
       <c r="B967" s="3" t="s">
-        <v>5790</v>
+        <v>5789</v>
       </c>
       <c r="C967" s="3" t="s">
         <v>3</v>
@@ -34748,7 +34748,7 @@
         <v>432712</v>
       </c>
       <c r="B969" s="3" t="s">
-        <v>5791</v>
+        <v>5790</v>
       </c>
       <c r="C969" s="3" t="s">
         <v>3</v>
@@ -34867,7 +34867,7 @@
         <v>436912</v>
       </c>
       <c r="B976" s="3" t="s">
-        <v>5792</v>
+        <v>5791</v>
       </c>
       <c r="C976" s="3" t="s">
         <v>3</v>
@@ -35037,7 +35037,7 @@
         <v>441593</v>
       </c>
       <c r="B986" s="3" t="s">
-        <v>5793</v>
+        <v>5792</v>
       </c>
       <c r="C986" s="3" t="s">
         <v>3</v>
@@ -35054,7 +35054,7 @@
         <v>441873</v>
       </c>
       <c r="B987" s="3" t="s">
-        <v>5794</v>
+        <v>5793</v>
       </c>
       <c r="C987" s="3" t="s">
         <v>3</v>
@@ -35207,7 +35207,7 @@
         <v>445141</v>
       </c>
       <c r="B996" s="3" t="s">
-        <v>5795</v>
+        <v>5794</v>
       </c>
       <c r="C996" s="3" t="s">
         <v>3</v>
@@ -35224,7 +35224,7 @@
         <v>448194</v>
       </c>
       <c r="B997" s="3" t="s">
-        <v>5796</v>
+        <v>5795</v>
       </c>
       <c r="C997" s="3" t="s">
         <v>3</v>
@@ -35241,7 +35241,7 @@
         <v>448240</v>
       </c>
       <c r="B998" s="3" t="s">
-        <v>5797</v>
+        <v>5796</v>
       </c>
       <c r="C998" s="3" t="s">
         <v>3</v>
@@ -35360,7 +35360,7 @@
         <v>452102</v>
       </c>
       <c r="B1005" s="3" t="s">
-        <v>5798</v>
+        <v>5797</v>
       </c>
       <c r="C1005" s="3" t="s">
         <v>3</v>
@@ -35411,7 +35411,7 @@
         <v>454896</v>
       </c>
       <c r="B1008" s="3" t="s">
-        <v>5799</v>
+        <v>5798</v>
       </c>
       <c r="C1008" s="3" t="s">
         <v>3</v>
@@ -35632,7 +35632,7 @@
         <v>462720</v>
       </c>
       <c r="B1021" s="3" t="s">
-        <v>5800</v>
+        <v>5799</v>
       </c>
       <c r="C1021" s="3" t="s">
         <v>3</v>
@@ -35870,7 +35870,7 @@
         <v>467162</v>
       </c>
       <c r="B1035" s="3" t="s">
-        <v>5801</v>
+        <v>5800</v>
       </c>
       <c r="C1035" s="3" t="s">
         <v>3</v>
@@ -35938,7 +35938,7 @@
         <v>468937</v>
       </c>
       <c r="B1039" s="3" t="s">
-        <v>5802</v>
+        <v>5801</v>
       </c>
       <c r="C1039" s="3" t="s">
         <v>3</v>
@@ -35989,7 +35989,7 @@
         <v>470779</v>
       </c>
       <c r="B1042" s="3" t="s">
-        <v>5803</v>
+        <v>5802</v>
       </c>
       <c r="C1042" s="3" t="s">
         <v>3</v>
@@ -36125,7 +36125,7 @@
         <v>474589</v>
       </c>
       <c r="B1050" s="3" t="s">
-        <v>5804</v>
+        <v>5803</v>
       </c>
       <c r="C1050" s="3" t="s">
         <v>3</v>
@@ -36142,7 +36142,7 @@
         <v>475153</v>
       </c>
       <c r="B1051" s="3" t="s">
-        <v>5805</v>
+        <v>5804</v>
       </c>
       <c r="C1051" s="3" t="s">
         <v>3</v>
@@ -36159,7 +36159,7 @@
         <v>475328</v>
       </c>
       <c r="B1052" s="3" t="s">
-        <v>5806</v>
+        <v>5805</v>
       </c>
       <c r="C1052" s="3" t="s">
         <v>3</v>
@@ -36210,7 +36210,7 @@
         <v>476653</v>
       </c>
       <c r="B1055" s="3" t="s">
-        <v>5807</v>
+        <v>5806</v>
       </c>
       <c r="C1055" s="3" t="s">
         <v>3</v>
@@ -36465,7 +36465,7 @@
         <v>482080</v>
       </c>
       <c r="B1070" s="3" t="s">
-        <v>5808</v>
+        <v>5807</v>
       </c>
       <c r="C1070" s="3" t="s">
         <v>3</v>
@@ -36635,7 +36635,7 @@
         <v>485612</v>
       </c>
       <c r="B1080" s="5" t="s">
-        <v>5945</v>
+        <v>5944</v>
       </c>
       <c r="C1080" s="3" t="s">
         <v>3</v>
@@ -36703,7 +36703,7 @@
         <v>487468</v>
       </c>
       <c r="B1084" s="3" t="s">
-        <v>5809</v>
+        <v>5808</v>
       </c>
       <c r="C1084" s="3" t="s">
         <v>3</v>
@@ -37230,7 +37230,7 @@
         <v>504519</v>
       </c>
       <c r="B1115" s="3" t="s">
-        <v>5810</v>
+        <v>5809</v>
       </c>
       <c r="C1115" s="3" t="s">
         <v>3</v>
@@ -38131,7 +38131,7 @@
         <v>523966</v>
       </c>
       <c r="B1168" s="3" t="s">
-        <v>5811</v>
+        <v>5810</v>
       </c>
       <c r="C1168" s="3" t="s">
         <v>3</v>
@@ -38216,7 +38216,7 @@
         <v>527287</v>
       </c>
       <c r="B1173" s="3" t="s">
-        <v>5812</v>
+        <v>5811</v>
       </c>
       <c r="C1173" s="3" t="s">
         <v>3</v>
@@ -38335,7 +38335,7 @@
         <v>529899</v>
       </c>
       <c r="B1180" s="3" t="s">
-        <v>5813</v>
+        <v>5812</v>
       </c>
       <c r="C1180" s="3" t="s">
         <v>3</v>
@@ -38420,7 +38420,7 @@
         <v>530968</v>
       </c>
       <c r="B1185" s="3" t="s">
-        <v>5814</v>
+        <v>5813</v>
       </c>
       <c r="C1185" s="3" t="s">
         <v>3</v>
@@ -38658,7 +38658,7 @@
         <v>537706</v>
       </c>
       <c r="B1199" s="3" t="s">
-        <v>5815</v>
+        <v>5814</v>
       </c>
       <c r="C1199" s="3" t="s">
         <v>3</v>
@@ -38794,7 +38794,7 @@
         <v>539572</v>
       </c>
       <c r="B1207" s="3" t="s">
-        <v>5816</v>
+        <v>5815</v>
       </c>
       <c r="C1207" s="3" t="s">
         <v>3</v>
@@ -38896,7 +38896,7 @@
         <v>541312</v>
       </c>
       <c r="B1213" s="3" t="s">
-        <v>5817</v>
+        <v>5816</v>
       </c>
       <c r="C1213" s="3" t="s">
         <v>3</v>
@@ -39457,7 +39457,7 @@
         <v>552534</v>
       </c>
       <c r="B1246" s="3" t="s">
-        <v>5818</v>
+        <v>5817</v>
       </c>
       <c r="C1246" s="3" t="s">
         <v>3</v>
@@ -39525,7 +39525,7 @@
         <v>554185</v>
       </c>
       <c r="B1250" s="3" t="s">
-        <v>5819</v>
+        <v>5818</v>
       </c>
       <c r="C1250" s="3" t="s">
         <v>3</v>
@@ -39576,7 +39576,7 @@
         <v>554929</v>
       </c>
       <c r="B1253" s="3" t="s">
-        <v>5820</v>
+        <v>5819</v>
       </c>
       <c r="C1253" s="3" t="s">
         <v>3</v>
@@ -39644,7 +39644,7 @@
         <v>555954</v>
       </c>
       <c r="B1257" s="3" t="s">
-        <v>5821</v>
+        <v>5820</v>
       </c>
       <c r="C1257" s="3" t="s">
         <v>3</v>
@@ -39661,7 +39661,7 @@
         <v>555959</v>
       </c>
       <c r="B1258" s="3" t="s">
-        <v>5822</v>
+        <v>5821</v>
       </c>
       <c r="C1258" s="3" t="s">
         <v>3</v>
@@ -39763,7 +39763,7 @@
         <v>559580</v>
       </c>
       <c r="B1264" s="3" t="s">
-        <v>5823</v>
+        <v>5822</v>
       </c>
       <c r="C1264" s="3" t="s">
         <v>3</v>
@@ -39797,7 +39797,7 @@
         <v>559956</v>
       </c>
       <c r="B1266" s="3" t="s">
-        <v>5824</v>
+        <v>5823</v>
       </c>
       <c r="C1266" s="3" t="s">
         <v>3</v>
@@ -40222,7 +40222,7 @@
         <v>567118</v>
       </c>
       <c r="B1291" s="3" t="s">
-        <v>5825</v>
+        <v>5824</v>
       </c>
       <c r="C1291" s="3" t="s">
         <v>3</v>
@@ -40239,7 +40239,7 @@
         <v>567465</v>
       </c>
       <c r="B1292" s="3" t="s">
-        <v>5826</v>
+        <v>5825</v>
       </c>
       <c r="C1292" s="3" t="s">
         <v>3</v>
@@ -40273,7 +40273,7 @@
         <v>567772</v>
       </c>
       <c r="B1294" s="3" t="s">
-        <v>5827</v>
+        <v>5826</v>
       </c>
       <c r="C1294" s="3" t="s">
         <v>3</v>
@@ -40392,7 +40392,7 @@
         <v>570624</v>
       </c>
       <c r="B1301" s="3" t="s">
-        <v>5828</v>
+        <v>5827</v>
       </c>
       <c r="C1301" s="3" t="s">
         <v>3</v>
@@ -40698,7 +40698,7 @@
         <v>581820</v>
       </c>
       <c r="B1319" s="3" t="s">
-        <v>5829</v>
+        <v>5828</v>
       </c>
       <c r="C1319" s="3" t="s">
         <v>3</v>
@@ -40919,7 +40919,7 @@
         <v>585234</v>
       </c>
       <c r="B1332" s="3" t="s">
-        <v>5830</v>
+        <v>5829</v>
       </c>
       <c r="C1332" s="3" t="s">
         <v>3</v>
@@ -41344,7 +41344,7 @@
         <v>594675</v>
       </c>
       <c r="B1357" s="3" t="s">
-        <v>5831</v>
+        <v>5830</v>
       </c>
       <c r="C1357" s="3" t="s">
         <v>3</v>
@@ -41667,7 +41667,7 @@
         <v>601844</v>
       </c>
       <c r="B1376" s="3" t="s">
-        <v>5832</v>
+        <v>5831</v>
       </c>
       <c r="C1376" s="3" t="s">
         <v>3</v>
@@ -41888,7 +41888,7 @@
         <v>606982</v>
       </c>
       <c r="B1389" s="3" t="s">
-        <v>5833</v>
+        <v>5832</v>
       </c>
       <c r="C1389" s="3" t="s">
         <v>3</v>
@@ -42330,7 +42330,7 @@
         <v>613079</v>
       </c>
       <c r="B1415" s="3" t="s">
-        <v>5834</v>
+        <v>5833</v>
       </c>
       <c r="C1415" s="3" t="s">
         <v>3</v>
@@ -42364,7 +42364,7 @@
         <v>614449</v>
       </c>
       <c r="B1417" s="3" t="s">
-        <v>5835</v>
+        <v>5834</v>
       </c>
       <c r="C1417" s="3" t="s">
         <v>3</v>
@@ -43792,7 +43792,7 @@
         <v>644774</v>
       </c>
       <c r="B1501" s="3" t="s">
-        <v>5836</v>
+        <v>5835</v>
       </c>
       <c r="C1501" s="3" t="s">
         <v>3</v>
@@ -43809,7 +43809,7 @@
         <v>645456</v>
       </c>
       <c r="B1502" s="3" t="s">
-        <v>5837</v>
+        <v>5836</v>
       </c>
       <c r="C1502" s="3" t="s">
         <v>3</v>
@@ -43826,7 +43826,7 @@
         <v>646120</v>
       </c>
       <c r="B1503" s="3" t="s">
-        <v>5838</v>
+        <v>5837</v>
       </c>
       <c r="C1503" s="3" t="s">
         <v>3</v>
@@ -43928,7 +43928,7 @@
         <v>646636</v>
       </c>
       <c r="B1509" s="3" t="s">
-        <v>5839</v>
+        <v>5838</v>
       </c>
       <c r="C1509" s="3" t="s">
         <v>3</v>
@@ -43945,7 +43945,7 @@
         <v>646742</v>
       </c>
       <c r="B1510" s="3" t="s">
-        <v>5840</v>
+        <v>5839</v>
       </c>
       <c r="C1510" s="3" t="s">
         <v>3</v>
@@ -43979,7 +43979,7 @@
         <v>647191</v>
       </c>
       <c r="B1512" s="3" t="s">
-        <v>5841</v>
+        <v>5840</v>
       </c>
       <c r="C1512" s="3" t="s">
         <v>3</v>
@@ -44115,7 +44115,7 @@
         <v>650292</v>
       </c>
       <c r="B1520" s="3" t="s">
-        <v>5842</v>
+        <v>5841</v>
       </c>
       <c r="C1520" s="3" t="s">
         <v>3</v>
@@ -44166,7 +44166,7 @@
         <v>651066</v>
       </c>
       <c r="B1523" s="3" t="s">
-        <v>5843</v>
+        <v>5842</v>
       </c>
       <c r="C1523" s="3" t="s">
         <v>3</v>
@@ -44353,7 +44353,7 @@
         <v>655324</v>
       </c>
       <c r="B1534" s="3" t="s">
-        <v>5844</v>
+        <v>5843</v>
       </c>
       <c r="C1534" s="3" t="s">
         <v>3</v>
@@ -44370,7 +44370,7 @@
         <v>655654</v>
       </c>
       <c r="B1535" s="3" t="s">
-        <v>5845</v>
+        <v>5844</v>
       </c>
       <c r="C1535" s="3" t="s">
         <v>3</v>
@@ -44778,7 +44778,7 @@
         <v>662129</v>
       </c>
       <c r="B1559" s="3" t="s">
-        <v>5846</v>
+        <v>5845</v>
       </c>
       <c r="C1559" s="3" t="s">
         <v>3</v>
@@ -45322,7 +45322,7 @@
         <v>673034</v>
       </c>
       <c r="B1591" s="3" t="s">
-        <v>5847</v>
+        <v>5846</v>
       </c>
       <c r="C1591" s="3" t="s">
         <v>3</v>
@@ -46121,7 +46121,7 @@
         <v>684053</v>
       </c>
       <c r="B1638" s="3" t="s">
-        <v>5848</v>
+        <v>5847</v>
       </c>
       <c r="C1638" s="3" t="s">
         <v>3</v>
@@ -46223,7 +46223,7 @@
         <v>684967</v>
       </c>
       <c r="B1644" s="3" t="s">
-        <v>5849</v>
+        <v>5848</v>
       </c>
       <c r="C1644" s="3" t="s">
         <v>3</v>
@@ -46274,7 +46274,7 @@
         <v>685601</v>
       </c>
       <c r="B1647" s="3" t="s">
-        <v>5850</v>
+        <v>5849</v>
       </c>
       <c r="C1647" s="3" t="s">
         <v>3</v>
@@ -46835,7 +46835,7 @@
         <v>689981</v>
       </c>
       <c r="B1680" s="3" t="s">
-        <v>5851</v>
+        <v>5850</v>
       </c>
       <c r="C1680" s="3" t="s">
         <v>3</v>
@@ -47124,7 +47124,7 @@
         <v>695239</v>
       </c>
       <c r="B1697" s="3" t="s">
-        <v>5852</v>
+        <v>5851</v>
       </c>
       <c r="C1697" s="3" t="s">
         <v>3</v>
@@ -47362,7 +47362,7 @@
         <v>700761</v>
       </c>
       <c r="B1711" s="3" t="s">
-        <v>5853</v>
+        <v>5852</v>
       </c>
       <c r="C1711" s="3" t="s">
         <v>3</v>
@@ -47889,7 +47889,7 @@
         <v>826937</v>
       </c>
       <c r="B1742" s="3" t="s">
-        <v>5854</v>
+        <v>5853</v>
       </c>
       <c r="C1742" s="3" t="s">
         <v>3</v>
@@ -48263,7 +48263,7 @@
         <v>838965</v>
       </c>
       <c r="B1764" s="3" t="s">
-        <v>5855</v>
+        <v>5854</v>
       </c>
       <c r="C1764" s="3" t="s">
         <v>3</v>
@@ -48297,7 +48297,7 @@
         <v>841373</v>
       </c>
       <c r="B1766" s="3" t="s">
-        <v>5856</v>
+        <v>5855</v>
       </c>
       <c r="C1766" s="3" t="s">
         <v>3</v>
@@ -48365,7 +48365,7 @@
         <v>841528</v>
       </c>
       <c r="B1770" s="3" t="s">
-        <v>5857</v>
+        <v>5856</v>
       </c>
       <c r="C1770" s="3" t="s">
         <v>3</v>
@@ -48569,7 +48569,7 @@
         <v>845513</v>
       </c>
       <c r="B1782" s="3" t="s">
-        <v>5858</v>
+        <v>5857</v>
       </c>
       <c r="C1782" s="3" t="s">
         <v>3</v>
@@ -48739,7 +48739,7 @@
         <v>851990</v>
       </c>
       <c r="B1792" s="3" t="s">
-        <v>5859</v>
+        <v>5858</v>
       </c>
       <c r="C1792" s="3" t="s">
         <v>3</v>
@@ -48841,7 +48841,7 @@
         <v>857892</v>
       </c>
       <c r="B1798" s="3" t="s">
-        <v>5860</v>
+        <v>5859</v>
       </c>
       <c r="C1798" s="3" t="s">
         <v>3</v>
@@ -48909,7 +48909,7 @@
         <v>860533</v>
       </c>
       <c r="B1802" s="3" t="s">
-        <v>5861</v>
+        <v>5860</v>
       </c>
       <c r="C1802" s="3" t="s">
         <v>3</v>
@@ -49249,7 +49249,7 @@
         <v>878176</v>
       </c>
       <c r="B1822" s="3" t="s">
-        <v>5862</v>
+        <v>5861</v>
       </c>
       <c r="C1822" s="3" t="s">
         <v>3</v>
@@ -50201,7 +50201,7 @@
         <v>939901</v>
       </c>
       <c r="B1878" s="3" t="s">
-        <v>5863</v>
+        <v>5862</v>
       </c>
       <c r="C1878" s="3" t="s">
         <v>3</v>
@@ -50541,7 +50541,7 @@
         <v>956445</v>
       </c>
       <c r="B1898" s="3" t="s">
-        <v>5864</v>
+        <v>5863</v>
       </c>
       <c r="C1898" s="3" t="s">
         <v>3</v>
@@ -50643,7 +50643,7 @@
         <v>960578</v>
       </c>
       <c r="B1904" s="3" t="s">
-        <v>5865</v>
+        <v>5864</v>
       </c>
       <c r="C1904" s="3" t="s">
         <v>3</v>
@@ -50694,7 +50694,7 @@
         <v>962282</v>
       </c>
       <c r="B1907" s="3" t="s">
-        <v>5866</v>
+        <v>5865</v>
       </c>
       <c r="C1907" s="3" t="s">
         <v>3</v>
@@ -50762,7 +50762,7 @@
         <v>963991</v>
       </c>
       <c r="B1911" s="3" t="s">
-        <v>5867</v>
+        <v>5866</v>
       </c>
       <c r="C1911" s="3" t="s">
         <v>3</v>
@@ -50898,7 +50898,7 @@
         <v>976274</v>
       </c>
       <c r="B1919" s="3" t="s">
-        <v>5868</v>
+        <v>5867</v>
       </c>
       <c r="C1919" s="3" t="s">
         <v>3</v>
@@ -51136,7 +51136,7 @@
         <v>986735</v>
       </c>
       <c r="B1933" s="3" t="s">
-        <v>5869</v>
+        <v>5868</v>
       </c>
       <c r="C1933" s="3" t="s">
         <v>3</v>
@@ -51357,7 +51357,7 @@
         <v>994932</v>
       </c>
       <c r="B1946" s="3" t="s">
-        <v>5870</v>
+        <v>5869</v>
       </c>
       <c r="C1946" s="3" t="s">
         <v>3</v>
@@ -51731,7 +51731,7 @@
         <v>1011533</v>
       </c>
       <c r="B1968" s="3" t="s">
-        <v>5871</v>
+        <v>5870</v>
       </c>
       <c r="C1968" s="3" t="s">
         <v>3</v>
@@ -51799,7 +51799,7 @@
         <v>1012491</v>
       </c>
       <c r="B1972" s="3" t="s">
-        <v>5872</v>
+        <v>5871</v>
       </c>
       <c r="C1972" s="3" t="s">
         <v>3</v>
@@ -51833,7 +51833,7 @@
         <v>1013869</v>
       </c>
       <c r="B1974" s="3" t="s">
-        <v>5873</v>
+        <v>5872</v>
       </c>
       <c r="C1974" s="3" t="s">
         <v>3</v>
@@ -51884,7 +51884,7 @@
         <v>1016541</v>
       </c>
       <c r="B1977" s="3" t="s">
-        <v>5874</v>
+        <v>5873</v>
       </c>
       <c r="C1977" s="3" t="s">
         <v>3</v>
@@ -51901,7 +51901,7 @@
         <v>1018117</v>
       </c>
       <c r="B1978" s="3" t="s">
-        <v>5875</v>
+        <v>5874</v>
       </c>
       <c r="C1978" s="3" t="s">
         <v>3</v>
@@ -51918,7 +51918,7 @@
         <v>1018638</v>
       </c>
       <c r="B1979" s="3" t="s">
-        <v>5876</v>
+        <v>5875</v>
       </c>
       <c r="C1979" s="3" t="s">
         <v>3</v>
@@ -51986,7 +51986,7 @@
         <v>1021214</v>
       </c>
       <c r="B1983" s="3" t="s">
-        <v>5877</v>
+        <v>5876</v>
       </c>
       <c r="C1983" s="3" t="s">
         <v>3</v>
@@ -52020,7 +52020,7 @@
         <v>1024377</v>
       </c>
       <c r="B1985" s="3" t="s">
-        <v>5878</v>
+        <v>5877</v>
       </c>
       <c r="C1985" s="3" t="s">
         <v>3</v>
@@ -52156,7 +52156,7 @@
         <v>1031747</v>
       </c>
       <c r="B1993" s="3" t="s">
-        <v>5879</v>
+        <v>5878</v>
       </c>
       <c r="C1993" s="3" t="s">
         <v>3</v>
@@ -52394,7 +52394,7 @@
         <v>1048745</v>
       </c>
       <c r="B2007" s="3" t="s">
-        <v>5880</v>
+        <v>5879</v>
       </c>
       <c r="C2007" s="3" t="s">
         <v>3</v>
@@ -52649,7 +52649,7 @@
         <v>1056353</v>
       </c>
       <c r="B2022" s="3" t="s">
-        <v>5881</v>
+        <v>5880</v>
       </c>
       <c r="C2022" s="3" t="s">
         <v>3</v>
@@ -52819,7 +52819,7 @@
         <v>1068978</v>
       </c>
       <c r="B2032" s="3" t="s">
-        <v>5882</v>
+        <v>5881</v>
       </c>
       <c r="C2032" s="3" t="s">
         <v>3</v>
@@ -52921,7 +52921,7 @@
         <v>1073213</v>
       </c>
       <c r="B2038" s="3" t="s">
-        <v>5883</v>
+        <v>5882</v>
       </c>
       <c r="C2038" s="3" t="s">
         <v>3</v>
@@ -52972,7 +52972,7 @@
         <v>1074228</v>
       </c>
       <c r="B2041" s="3" t="s">
-        <v>5884</v>
+        <v>5883</v>
       </c>
       <c r="C2041" s="3" t="s">
         <v>3</v>
@@ -53074,7 +53074,7 @@
         <v>1078485</v>
       </c>
       <c r="B2047" s="3" t="s">
-        <v>5885</v>
+        <v>5884</v>
       </c>
       <c r="C2047" s="3" t="s">
         <v>3</v>
@@ -53210,7 +53210,7 @@
         <v>1084345</v>
       </c>
       <c r="B2055" s="3" t="s">
-        <v>5886</v>
+        <v>5885</v>
       </c>
       <c r="C2055" s="3" t="s">
         <v>3</v>
@@ -53550,7 +53550,7 @@
         <v>1101870</v>
       </c>
       <c r="B2075" s="3" t="s">
-        <v>5887</v>
+        <v>5886</v>
       </c>
       <c r="C2075" s="3" t="s">
         <v>3</v>
@@ -53822,7 +53822,7 @@
         <v>1112419</v>
       </c>
       <c r="B2091" s="3" t="s">
-        <v>5888</v>
+        <v>5887</v>
       </c>
       <c r="C2091" s="3" t="s">
         <v>3</v>
@@ -54077,7 +54077,7 @@
         <v>1128680</v>
       </c>
       <c r="B2106" s="3" t="s">
-        <v>5889</v>
+        <v>5888</v>
       </c>
       <c r="C2106" s="3" t="s">
         <v>3</v>
@@ -54162,7 +54162,7 @@
         <v>1131013</v>
       </c>
       <c r="B2111" s="3" t="s">
-        <v>5890</v>
+        <v>5889</v>
       </c>
       <c r="C2111" s="3" t="s">
         <v>3</v>
@@ -54417,7 +54417,7 @@
         <v>1143864</v>
       </c>
       <c r="B2126" s="3" t="s">
-        <v>5891</v>
+        <v>5890</v>
       </c>
       <c r="C2126" s="3" t="s">
         <v>3</v>
@@ -55046,7 +55046,7 @@
         <v>1199451</v>
       </c>
       <c r="B2163" s="3" t="s">
-        <v>5892</v>
+        <v>5891</v>
       </c>
       <c r="C2163" s="3" t="s">
         <v>3</v>
@@ -55454,7 +55454,7 @@
         <v>1217078</v>
       </c>
       <c r="B2187" s="3" t="s">
-        <v>5893</v>
+        <v>5892</v>
       </c>
       <c r="C2187" s="3" t="s">
         <v>3</v>
@@ -55522,7 +55522,7 @@
         <v>1219803</v>
       </c>
       <c r="B2191" s="3" t="s">
-        <v>5894</v>
+        <v>5893</v>
       </c>
       <c r="C2191" s="3" t="s">
         <v>3</v>
@@ -55590,7 +55590,7 @@
         <v>1225266</v>
       </c>
       <c r="B2195" s="3" t="s">
-        <v>5895</v>
+        <v>5894</v>
       </c>
       <c r="C2195" s="3" t="s">
         <v>3</v>
@@ -55726,7 +55726,7 @@
         <v>1236427</v>
       </c>
       <c r="B2203" s="3" t="s">
-        <v>5896</v>
+        <v>5895</v>
       </c>
       <c r="C2203" s="3" t="s">
         <v>3</v>
@@ -55760,7 +55760,7 @@
         <v>1239005</v>
       </c>
       <c r="B2205" s="3" t="s">
-        <v>5897</v>
+        <v>5896</v>
       </c>
       <c r="C2205" s="3" t="s">
         <v>3</v>
@@ -55913,7 +55913,7 @@
         <v>1245373</v>
       </c>
       <c r="B2214" s="3" t="s">
-        <v>5898</v>
+        <v>5897</v>
       </c>
       <c r="C2214" s="3" t="s">
         <v>3</v>
@@ -55930,7 +55930,7 @@
         <v>1246547</v>
       </c>
       <c r="B2215" s="3" t="s">
-        <v>5899</v>
+        <v>5898</v>
       </c>
       <c r="C2215" s="3" t="s">
         <v>3</v>
@@ -56117,7 +56117,7 @@
         <v>1257253</v>
       </c>
       <c r="B2226" s="3" t="s">
-        <v>5900</v>
+        <v>5899</v>
       </c>
       <c r="C2226" s="3" t="s">
         <v>3</v>
@@ -56185,7 +56185,7 @@
         <v>1260769</v>
       </c>
       <c r="B2230" s="3" t="s">
-        <v>5901</v>
+        <v>5900</v>
       </c>
       <c r="C2230" s="3" t="s">
         <v>3</v>
@@ -56338,7 +56338,7 @@
         <v>1274405</v>
       </c>
       <c r="B2239" s="3" t="s">
-        <v>5902</v>
+        <v>5901</v>
       </c>
       <c r="C2239" s="3" t="s">
         <v>3</v>
@@ -56848,7 +56848,7 @@
         <v>1312513</v>
       </c>
       <c r="B2269" s="3" t="s">
-        <v>5903</v>
+        <v>5902</v>
       </c>
       <c r="C2269" s="3" t="s">
         <v>3</v>
@@ -57154,7 +57154,7 @@
         <v>1336417</v>
       </c>
       <c r="B2287" s="3" t="s">
-        <v>5904</v>
+        <v>5903</v>
       </c>
       <c r="C2287" s="3" t="s">
         <v>3</v>
@@ -57783,7 +57783,7 @@
         <v>1385822</v>
       </c>
       <c r="B2324" s="3" t="s">
-        <v>5905</v>
+        <v>5904</v>
       </c>
       <c r="C2324" s="3" t="s">
         <v>3</v>
@@ -57987,7 +57987,7 @@
         <v>1397375</v>
       </c>
       <c r="B2336" s="3" t="s">
-        <v>5906</v>
+        <v>5905</v>
       </c>
       <c r="C2336" s="3" t="s">
         <v>3</v>
@@ -58395,7 +58395,7 @@
         <v>1422846</v>
       </c>
       <c r="B2360" s="3" t="s">
-        <v>5907</v>
+        <v>5906</v>
       </c>
       <c r="C2360" s="3" t="s">
         <v>3</v>
@@ -58735,7 +58735,7 @@
         <v>1442654</v>
       </c>
       <c r="B2380" s="3" t="s">
-        <v>5908</v>
+        <v>5907</v>
       </c>
       <c r="C2380" s="3" t="s">
         <v>3</v>
@@ -58786,7 +58786,7 @@
         <v>1447752</v>
       </c>
       <c r="B2383" s="3" t="s">
-        <v>5909</v>
+        <v>5908</v>
       </c>
       <c r="C2383" s="3" t="s">
         <v>3</v>
@@ -59364,7 +59364,7 @@
         <v>1481741</v>
       </c>
       <c r="B2417" s="3" t="s">
-        <v>5910</v>
+        <v>5909</v>
       </c>
       <c r="C2417" s="3" t="s">
         <v>3</v>
@@ -59959,7 +59959,7 @@
         <v>1530118</v>
       </c>
       <c r="B2452" s="3" t="s">
-        <v>5911</v>
+        <v>5910</v>
       </c>
       <c r="C2452" s="3" t="s">
         <v>3</v>
@@ -60316,7 +60316,7 @@
         <v>1563243</v>
       </c>
       <c r="B2473" s="3" t="s">
-        <v>5912</v>
+        <v>5911</v>
       </c>
       <c r="C2473" s="3" t="s">
         <v>3</v>
@@ -60537,7 +60537,7 @@
         <v>1578153</v>
       </c>
       <c r="B2486" s="3" t="s">
-        <v>5913</v>
+        <v>5912</v>
       </c>
       <c r="C2486" s="3" t="s">
         <v>3</v>
@@ -60758,7 +60758,7 @@
         <v>1593477</v>
       </c>
       <c r="B2499" s="3" t="s">
-        <v>5914</v>
+        <v>5913</v>
       </c>
       <c r="C2499" s="3" t="s">
         <v>3</v>
@@ -60945,7 +60945,7 @@
         <v>1603362</v>
       </c>
       <c r="B2510" s="3" t="s">
-        <v>5915</v>
+        <v>5914</v>
       </c>
       <c r="C2510" s="3" t="s">
         <v>3</v>
@@ -60979,7 +60979,7 @@
         <v>1605525</v>
       </c>
       <c r="B2512" s="3" t="s">
-        <v>5916</v>
+        <v>5915</v>
       </c>
       <c r="C2512" s="3" t="s">
         <v>3</v>
@@ -61047,7 +61047,7 @@
         <v>1606578</v>
       </c>
       <c r="B2516" s="3" t="s">
-        <v>5917</v>
+        <v>5916</v>
       </c>
       <c r="C2516" s="3" t="s">
         <v>3</v>
@@ -62254,7 +62254,7 @@
         <v>1671262</v>
       </c>
       <c r="B2587" s="3" t="s">
-        <v>5918</v>
+        <v>5917</v>
       </c>
       <c r="C2587" s="3" t="s">
         <v>3</v>
@@ -62679,7 +62679,7 @@
         <v>1699443</v>
       </c>
       <c r="B2612" s="3" t="s">
-        <v>5919</v>
+        <v>5918</v>
       </c>
       <c r="C2612" s="3" t="s">
         <v>3</v>
@@ -62798,7 +62798,7 @@
         <v>1707533</v>
       </c>
       <c r="B2619" s="3" t="s">
-        <v>5920</v>
+        <v>5919</v>
       </c>
       <c r="C2619" s="3" t="s">
         <v>3</v>
@@ -62815,7 +62815,7 @@
         <v>1709011</v>
       </c>
       <c r="B2620" s="3" t="s">
-        <v>5921</v>
+        <v>5920</v>
       </c>
       <c r="C2620" s="3" t="s">
         <v>3</v>
@@ -63019,7 +63019,7 @@
         <v>1716746</v>
       </c>
       <c r="B2632" s="3" t="s">
-        <v>5922</v>
+        <v>5921</v>
       </c>
       <c r="C2632" s="3" t="s">
         <v>3</v>
@@ -63852,7 +63852,7 @@
         <v>1774566</v>
       </c>
       <c r="B2681" s="3" t="s">
-        <v>5923</v>
+        <v>5922</v>
       </c>
       <c r="C2681" s="3" t="s">
         <v>3</v>
@@ -64022,7 +64022,7 @@
         <v>1788095</v>
       </c>
       <c r="B2691" s="3" t="s">
-        <v>5924</v>
+        <v>5923</v>
       </c>
       <c r="C2691" s="3" t="s">
         <v>3</v>
@@ -64294,7 +64294,7 @@
         <v>1799298</v>
       </c>
       <c r="B2707" s="3" t="s">
-        <v>5925</v>
+        <v>5924</v>
       </c>
       <c r="C2707" s="3" t="s">
         <v>3</v>
@@ -64515,7 +64515,7 @@
         <v>1824240</v>
       </c>
       <c r="B2720" s="3" t="s">
-        <v>5926</v>
+        <v>5925</v>
       </c>
       <c r="C2720" s="3" t="s">
         <v>3</v>
@@ -64532,7 +64532,7 @@
         <v>1828587</v>
       </c>
       <c r="B2721" s="3" t="s">
-        <v>5927</v>
+        <v>5926</v>
       </c>
       <c r="C2721" s="3" t="s">
         <v>3</v>
@@ -64600,7 +64600,7 @@
         <v>1836903</v>
       </c>
       <c r="B2725" s="3" t="s">
-        <v>5928</v>
+        <v>5927</v>
       </c>
       <c r="C2725" s="3" t="s">
         <v>3</v>
@@ -65739,7 +65739,7 @@
         <v>1922769</v>
       </c>
       <c r="B2792" s="3" t="s">
-        <v>5929</v>
+        <v>5928</v>
       </c>
       <c r="C2792" s="3" t="s">
         <v>3</v>
@@ -65790,7 +65790,7 @@
         <v>1925698</v>
       </c>
       <c r="B2795" s="3" t="s">
-        <v>5930</v>
+        <v>5929</v>
       </c>
       <c r="C2795" s="3" t="s">
         <v>3</v>
@@ -66011,7 +66011,7 @@
         <v>1936005</v>
       </c>
       <c r="B2808" s="3" t="s">
-        <v>5931</v>
+        <v>5930</v>
       </c>
       <c r="C2808" s="3" t="s">
         <v>3</v>
@@ -66232,7 +66232,7 @@
         <v>1947939</v>
       </c>
       <c r="B2821" s="3" t="s">
-        <v>5932</v>
+        <v>5931</v>
       </c>
       <c r="C2821" s="3" t="s">
         <v>3</v>
@@ -66249,7 +66249,7 @@
         <v>1948863</v>
       </c>
       <c r="B2822" s="3" t="s">
-        <v>5933</v>
+        <v>5932</v>
       </c>
       <c r="C2822" s="3" t="s">
         <v>3</v>
@@ -66657,7 +66657,7 @@
         <v>1977273</v>
       </c>
       <c r="B2846" s="3" t="s">
-        <v>5934</v>
+        <v>5933</v>
       </c>
       <c r="C2846" s="3" t="s">
         <v>3</v>
@@ -66674,7 +66674,7 @@
         <v>1981639</v>
       </c>
       <c r="B2847" s="3" t="s">
-        <v>5935</v>
+        <v>5934</v>
       </c>
       <c r="C2847" s="3" t="s">
         <v>3</v>
@@ -66912,7 +66912,7 @@
         <v>2006759</v>
       </c>
       <c r="B2861" s="3" t="s">
-        <v>5936</v>
+        <v>5935</v>
       </c>
       <c r="C2861" s="3" t="s">
         <v>3</v>
@@ -67252,7 +67252,7 @@
         <v>2031153</v>
       </c>
       <c r="B2881" s="3" t="s">
-        <v>5937</v>
+        <v>5936</v>
       </c>
       <c r="C2881" s="3" t="s">
         <v>3</v>
@@ -67966,7 +67966,7 @@
         <v>2072627</v>
       </c>
       <c r="B2923" s="3" t="s">
-        <v>5938</v>
+        <v>5937</v>
       </c>
       <c r="C2923" s="3" t="s">
         <v>3</v>
@@ -68017,7 +68017,7 @@
         <v>2079588</v>
       </c>
       <c r="B2926" s="3" t="s">
-        <v>5939</v>
+        <v>5938</v>
       </c>
       <c r="C2926" s="3" t="s">
         <v>3</v>
@@ -68051,7 +68051,7 @@
         <v>2082859</v>
       </c>
       <c r="B2928" s="3" t="s">
-        <v>5940</v>
+        <v>5939</v>
       </c>
       <c r="C2928" s="3" t="s">
         <v>3</v>
@@ -68561,7 +68561,7 @@
         <v>2107643</v>
       </c>
       <c r="B2958" s="3" t="s">
-        <v>5941</v>
+        <v>5940</v>
       </c>
       <c r="C2958" s="3" t="s">
         <v>3</v>

</xml_diff>